<commit_message>
Sync monthly workload dashboard (2026-08-10 09:30)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -2737,4 +2737,291 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B861B575-3856-4655-A267-3B6B8C7EFE1D}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97985DF4-7659-4ADE-94EE-B9D205FDCABE}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FCC94F8-29C9-47D2-8A67-886FF34C66CD}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-10 09:39)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Dashboard\.dashboard-repo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/.dashboard-repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8E16A501-FAEC-4B26-9B92-75F1AB5720BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BBCF357E-DEEB-4D80-807F-D51E5846AC23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8949F011-D5F1-45DB-B1BA-C006FB97D7E9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CF64029C-E273-4608-92F9-6DB45903B822}"/>
   </bookViews>
   <sheets>
     <sheet name="Financial Forecast" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>Financial Forecast</t>
   </si>
   <si>
-    <t>Construction_Portfolio_Template - Data base.xlsx  ·  สร้างเมื่อ 2026-08-10 09:28</t>
+    <t>Construction_Portfolio_Template - Data base.xlsx  ·  สร้างเมื่อ 2026-08-10 09:38</t>
   </si>
   <si>
     <t>สีหัวเดือน:</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46C9C9AA-5018-4C51-B075-9080AE23EEE0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADE3C5A0-6F5E-4ABA-B64A-7799043CC670}">
   <dimension ref="A1:AE50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -837,10 +837,10 @@
       <c r="L7" s="12"/>
       <c r="M7" s="12"/>
       <c r="N7" s="12"/>
-      <c r="O7" s="12"/>
-      <c r="P7" s="12">
+      <c r="O7" s="12">
         <v>130714.54399999999</v>
       </c>
+      <c r="P7" s="12"/>
       <c r="Q7" s="12"/>
       <c r="R7" s="12"/>
       <c r="S7" s="12"/>
@@ -926,9 +926,11 @@
       <c r="R9" s="12"/>
       <c r="S9" s="12"/>
       <c r="T9" s="12"/>
-      <c r="U9" s="12"/>
+      <c r="U9" s="12">
+        <v>163839.85600000003</v>
+      </c>
       <c r="V9" s="12">
-        <v>327679.71200000006</v>
+        <v>163839.85600000003</v>
       </c>
       <c r="W9" s="12"/>
       <c r="X9" s="12"/>
@@ -1001,9 +1003,11 @@
       <c r="L11" s="12"/>
       <c r="M11" s="12"/>
       <c r="N11" s="12"/>
-      <c r="O11" s="12"/>
+      <c r="O11" s="12">
+        <v>230527.16000000003</v>
+      </c>
       <c r="P11" s="12">
-        <v>461054.32000000007</v>
+        <v>230527.16000000003</v>
       </c>
       <c r="Q11" s="12"/>
       <c r="R11" s="12"/>
@@ -1085,9 +1089,11 @@
       <c r="O13" s="12"/>
       <c r="P13" s="12"/>
       <c r="Q13" s="12"/>
-      <c r="R13" s="12"/>
+      <c r="R13" s="12">
+        <v>129184.43200000002</v>
+      </c>
       <c r="S13" s="12">
-        <v>387553.29600000003</v>
+        <v>258368.86400000003</v>
       </c>
       <c r="T13" s="12"/>
       <c r="U13" s="12"/>
@@ -1169,10 +1175,10 @@
       <c r="V15" s="12"/>
       <c r="W15" s="12"/>
       <c r="X15" s="12"/>
-      <c r="Y15" s="12"/>
-      <c r="Z15" s="12">
+      <c r="Y15" s="12">
         <v>252247.67999999999</v>
       </c>
+      <c r="Z15" s="12"/>
       <c r="AA15" s="12"/>
       <c r="AB15" s="12"/>
       <c r="AC15" s="12"/>
@@ -1316,10 +1322,10 @@
       <c r="O19" s="12"/>
       <c r="P19" s="12"/>
       <c r="Q19" s="12"/>
-      <c r="R19" s="12"/>
-      <c r="S19" s="12">
+      <c r="R19" s="12">
         <v>462444.47200000001</v>
       </c>
+      <c r="S19" s="12"/>
       <c r="T19" s="12">
         <v>346833.35399999999</v>
       </c>
@@ -1480,11 +1486,13 @@
       <c r="O23" s="12"/>
       <c r="P23" s="12"/>
       <c r="Q23" s="12"/>
-      <c r="R23" s="12"/>
+      <c r="R23" s="12">
+        <v>130841.12</v>
+      </c>
       <c r="S23" s="12"/>
       <c r="T23" s="12"/>
       <c r="U23" s="12">
-        <v>261682.24</v>
+        <v>130841.12</v>
       </c>
       <c r="V23" s="12"/>
       <c r="W23" s="12"/>
@@ -1642,9 +1650,11 @@
       <c r="O27" s="12"/>
       <c r="P27" s="12"/>
       <c r="Q27" s="12"/>
-      <c r="R27" s="12"/>
+      <c r="R27" s="12">
+        <v>32000</v>
+      </c>
       <c r="S27" s="12">
-        <v>112000</v>
+        <v>80000</v>
       </c>
       <c r="T27" s="12"/>
       <c r="U27" s="12"/>
@@ -1720,10 +1730,10 @@
       <c r="R29" s="12"/>
       <c r="S29" s="12"/>
       <c r="T29" s="12"/>
-      <c r="U29" s="12"/>
-      <c r="V29" s="12">
+      <c r="U29" s="12">
         <v>479984.00800000003</v>
       </c>
+      <c r="V29" s="12"/>
       <c r="W29" s="12">
         <v>479984.00800000003</v>
       </c>
@@ -1797,10 +1807,10 @@
       <c r="L31" s="12"/>
       <c r="M31" s="12"/>
       <c r="N31" s="12"/>
-      <c r="O31" s="12"/>
-      <c r="P31" s="12">
+      <c r="O31" s="12">
         <v>240000</v>
       </c>
+      <c r="P31" s="12"/>
       <c r="Q31" s="12">
         <v>180000</v>
       </c>
@@ -1878,9 +1888,11 @@
       <c r="L33" s="12"/>
       <c r="M33" s="12"/>
       <c r="N33" s="12"/>
-      <c r="O33" s="12"/>
+      <c r="O33" s="12">
+        <v>127059.20000000001</v>
+      </c>
       <c r="P33" s="12">
-        <v>254118.40000000002</v>
+        <v>127059.20000000001</v>
       </c>
       <c r="Q33" s="12"/>
       <c r="R33" s="12">
@@ -1962,9 +1974,11 @@
       <c r="Q35" s="12"/>
       <c r="R35" s="12"/>
       <c r="S35" s="12"/>
-      <c r="T35" s="12"/>
+      <c r="T35" s="12">
+        <v>333125.2</v>
+      </c>
       <c r="U35" s="12">
-        <v>666250.4</v>
+        <v>333125.2</v>
       </c>
       <c r="V35" s="12"/>
       <c r="W35" s="12"/>
@@ -2026,9 +2040,11 @@
       <c r="B37" t="s">
         <v>38</v>
       </c>
-      <c r="C37" s="12"/>
+      <c r="C37" s="12">
+        <v>136494.53600000002</v>
+      </c>
       <c r="D37" s="12">
-        <v>272989.07200000004</v>
+        <v>136494.53600000002</v>
       </c>
       <c r="E37" s="12"/>
       <c r="F37" s="12"/>
@@ -2107,9 +2123,11 @@
       <c r="B39" t="s">
         <v>38</v>
       </c>
-      <c r="C39" s="12"/>
+      <c r="C39" s="12">
+        <v>266680</v>
+      </c>
       <c r="D39" s="12">
-        <v>533360</v>
+        <v>266680</v>
       </c>
       <c r="E39" s="12"/>
       <c r="F39" s="12"/>
@@ -2206,10 +2224,10 @@
       <c r="R41" s="12"/>
       <c r="S41" s="12"/>
       <c r="T41" s="12"/>
-      <c r="U41" s="12"/>
-      <c r="V41" s="12">
+      <c r="U41" s="12">
         <v>184000</v>
       </c>
+      <c r="V41" s="12"/>
       <c r="W41" s="12">
         <v>184000</v>
       </c>
@@ -2288,11 +2306,9 @@
       <c r="Q43" s="12"/>
       <c r="R43" s="12"/>
       <c r="S43" s="12"/>
-      <c r="T43" s="12">
-        <v>82752</v>
-      </c>
+      <c r="T43" s="12"/>
       <c r="U43" s="12">
-        <v>124128</v>
+        <v>206880</v>
       </c>
       <c r="V43" s="12"/>
       <c r="W43" s="12"/>
@@ -2461,10 +2477,10 @@
         <v>59</v>
       </c>
       <c r="C48" s="15">
-        <v>0</v>
+        <v>403174.53600000002</v>
       </c>
       <c r="D48" s="15">
-        <v>806349.07200000004</v>
+        <v>403174.53600000002</v>
       </c>
       <c r="E48" s="15">
         <v>0</v>
@@ -2497,28 +2513,28 @@
         <v>0</v>
       </c>
       <c r="O48" s="15">
-        <v>0</v>
+        <v>728300.9040000001</v>
       </c>
       <c r="P48" s="15">
-        <v>1085887.264</v>
+        <v>357586.36000000004</v>
       </c>
       <c r="Q48" s="15">
         <v>180000</v>
       </c>
       <c r="R48" s="15">
-        <v>378909.68000000005</v>
+        <v>1133379.7040000001</v>
       </c>
       <c r="S48" s="15">
-        <v>1780213.4480000001</v>
+        <v>1156584.5440000002</v>
       </c>
       <c r="T48" s="15">
-        <v>1387044.338</v>
+        <v>1637417.5379999999</v>
       </c>
       <c r="U48" s="15">
-        <v>1527082.98</v>
+        <v>1973692.524</v>
       </c>
       <c r="V48" s="15">
-        <v>1311613.7200000002</v>
+        <v>483789.85600000003</v>
       </c>
       <c r="W48" s="15">
         <v>1464107.362</v>
@@ -2527,10 +2543,10 @@
         <v>0</v>
       </c>
       <c r="Y48" s="15">
-        <v>486128.12800000003</v>
+        <v>738375.80799999996</v>
       </c>
       <c r="Z48" s="15">
-        <v>828016.12400000007</v>
+        <v>575768.44400000002</v>
       </c>
       <c r="AA48" s="15">
         <v>118822.8</v>
@@ -2647,7 +2663,7 @@
         <v>61</v>
       </c>
       <c r="C50" s="13">
-        <v>-139012.5</v>
+        <v>264162.03600000002</v>
       </c>
       <c r="D50" s="13">
         <v>435649.07200000004</v>
@@ -2683,345 +2699,58 @@
         <v>435649.07200000004</v>
       </c>
       <c r="O50" s="13">
-        <v>206196.77200000006</v>
+        <v>934497.67600000021</v>
       </c>
       <c r="P50" s="13">
-        <v>1068098.0360000001</v>
+        <v>1068098.0360000003</v>
       </c>
       <c r="Q50" s="13">
-        <v>1018695.3360000001</v>
+        <v>1018695.3360000004</v>
       </c>
       <c r="R50" s="13">
-        <v>1125005.0160000003</v>
+        <v>1879475.0400000005</v>
       </c>
       <c r="S50" s="13">
-        <v>2580814.7550000004</v>
+        <v>2711655.8750000009</v>
       </c>
       <c r="T50" s="13">
-        <v>3228183.7720000003</v>
+        <v>3609398.0920000011</v>
       </c>
       <c r="U50" s="13">
-        <v>4203932.9520000005</v>
+        <v>5031756.8160000015</v>
       </c>
       <c r="V50" s="13">
-        <v>5250705.8720000004</v>
+        <v>5250705.8720000014</v>
       </c>
       <c r="W50" s="13">
-        <v>6081686.034</v>
+        <v>6081686.0340000018</v>
       </c>
       <c r="X50" s="13">
-        <v>6057686.034</v>
+        <v>6057686.0340000018</v>
       </c>
       <c r="Y50" s="13">
-        <v>6387839.7920000004</v>
+        <v>6640087.4720000019</v>
       </c>
       <c r="Z50" s="13">
-        <v>7052582.3859999999</v>
+        <v>7052582.3860000018</v>
       </c>
       <c r="AA50" s="13">
-        <v>7103109.9859999996</v>
+        <v>7103109.9860000014</v>
       </c>
       <c r="AB50" s="13">
-        <v>7263084.9859999996</v>
+        <v>7263084.9860000014</v>
       </c>
       <c r="AC50" s="13">
-        <v>7263084.9859999996</v>
+        <v>7263084.9860000014</v>
       </c>
       <c r="AD50" s="13">
-        <v>7220084.9859999996</v>
+        <v>7220084.9860000014</v>
       </c>
       <c r="AE50" s="13">
-        <v>7312084.9859999996</v>
+        <v>7312084.9860000014</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B861B575-3856-4655-A267-3B6B8C7EFE1D}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97985DF4-7659-4ADE-94EE-B9D205FDCABE}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FCC94F8-29C9-47D2-8A67-886FF34C66CD}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-10 09:40)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/.dashboard-repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BBCF357E-DEEB-4D80-807F-D51E5846AC23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C47D6DDF-6AE0-4DAE-A889-EB6906611ED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CF64029C-E273-4608-92F9-6DB45903B822}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9BB38DA6-1B19-45E3-8F2C-5B54890A2C36}"/>
   </bookViews>
   <sheets>
     <sheet name="Financial Forecast" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>Financial Forecast</t>
   </si>
   <si>
-    <t>Construction_Portfolio_Template - Data base.xlsx  ·  สร้างเมื่อ 2026-08-10 09:38</t>
+    <t>Construction_Portfolio_Template - Data base.xlsx  ·  สร้างเมื่อ 2026-08-10 09:40</t>
   </si>
   <si>
     <t>สีหัวเดือน:</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADE3C5A0-6F5E-4ABA-B64A-7799043CC670}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3EAE26F-C8B8-4ED0-B560-7D6BFE5D7219}">
   <dimension ref="A1:AE50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-10 14:30)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/.dashboard-repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{963017B4-53D9-4AF3-B6F6-E851B4583C8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD835354-46E8-4980-9269-B273579FD1A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{545DDBC0-AF08-4386-9A2A-33B930F4978B}"/>
+    <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="8880" xr2:uid="{5FC50B19-4B18-49BF-9065-33B7F999D487}"/>
   </bookViews>
   <sheets>
     <sheet name="2025" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
     <t>Financial Forecast 2025  (พ.ศ. 2568)</t>
   </si>
   <si>
-    <t>Construction_Portfolio_Template - Data base.xlsx  ·  สร้างเมื่อ 2026-08-10 09:46</t>
+    <t>Construction_Portfolio_Template - Data base.xlsx  ·  สร้างเมื่อ 2026-08-10 14:29</t>
   </si>
   <si>
     <t>สีหัวเดือน:</t>
@@ -648,7 +648,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB35C85C-013D-4A82-B8F7-D2C8697FDB0B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16CA0734-6B9F-46A8-B141-B5152868967D}">
   <dimension ref="A1:N14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -961,7 +961,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{950030FA-545F-4228-93F7-542F02D578EB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1723BFDA-46A6-4356-965C-8E521BAC1F96}">
   <dimension ref="A1:N50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2092,7 +2092,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E27F3F0-E98A-4458-BCFB-BC621CDAC032}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D999DE1B-F8D4-4FC2-A0CC-80824CB8D893}">
   <dimension ref="A1:N20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-10 14:46)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -2515,4 +2515,291 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02877852-E817-449C-8523-361B0A0350DD}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B2E1A52-4259-4B4C-BF30-AA35502792D9}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7BB0381-FCD2-405D-BA9B-8E3B5AA17D87}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-10 14:52)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Dashboard\.dashboard-repo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/.dashboard-repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F31682B-68EB-4F35-8C74-3D9CA505BD4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8D79197E-E372-4D57-9C5F-A06345C51491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="8880" xr2:uid="{ED8BB402-B8CB-41FD-A13B-A4A73B677B1C}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{02D4ED39-8C7B-42B8-BF59-76F77D0E6138}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="57">
   <si>
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (20 โครงการ PO)</t>
   </si>
@@ -54,6 +54,90 @@
   </si>
   <si>
     <t>Total (฿)</t>
+  </si>
+  <si>
+    <t>Mar-25</t>
+  </si>
+  <si>
+    <t>Apr-25</t>
+  </si>
+  <si>
+    <t>May-25</t>
+  </si>
+  <si>
+    <t>Jun-25</t>
+  </si>
+  <si>
+    <t>Jul-25</t>
+  </si>
+  <si>
+    <t>Aug-25</t>
+  </si>
+  <si>
+    <t>Sep-25</t>
+  </si>
+  <si>
+    <t>Oct-25</t>
+  </si>
+  <si>
+    <t>Nov-25</t>
+  </si>
+  <si>
+    <t>Dec-25</t>
+  </si>
+  <si>
+    <t>Jan-26</t>
+  </si>
+  <si>
+    <t>Feb-26</t>
+  </si>
+  <si>
+    <t>Mar-26</t>
+  </si>
+  <si>
+    <t>Apr-26</t>
+  </si>
+  <si>
+    <t>May-26</t>
+  </si>
+  <si>
+    <t>Jun-26</t>
+  </si>
+  <si>
+    <t>Jul-26</t>
+  </si>
+  <si>
+    <t>Aug-26</t>
+  </si>
+  <si>
+    <t>Sep-26</t>
+  </si>
+  <si>
+    <t>Oct-26</t>
+  </si>
+  <si>
+    <t>Nov-26</t>
+  </si>
+  <si>
+    <t>Dec-26</t>
+  </si>
+  <si>
+    <t>Jan-27</t>
+  </si>
+  <si>
+    <t>Feb-27</t>
+  </si>
+  <si>
+    <t>Mar-27</t>
+  </si>
+  <si>
+    <t>Apr-27</t>
+  </si>
+  <si>
+    <t>May-27</t>
+  </si>
+  <si>
+    <t>Jun-27</t>
   </si>
   <si>
     <t>รวม (฿)</t>
@@ -191,7 +275,7 @@
     </font>
     <font>
       <b/>
-      <sz val="9"/>
+      <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -256,7 +340,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="16" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -607,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F366D27-C29F-4F82-9D12-4C4E0A57E221}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82B05CFD-A9B7-4A0F-BA78-8B2DE727E57C}">
   <dimension ref="A1:AE52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -730,97 +814,97 @@
       <c r="B5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="7">
-        <v>46106</v>
-      </c>
-      <c r="D5" s="7">
-        <v>46137</v>
-      </c>
-      <c r="E5" s="7">
-        <v>46167</v>
-      </c>
-      <c r="F5" s="7">
-        <v>46198</v>
-      </c>
-      <c r="G5" s="7">
-        <v>46228</v>
-      </c>
-      <c r="H5" s="7">
-        <v>46259</v>
-      </c>
-      <c r="I5" s="7">
-        <v>46290</v>
-      </c>
-      <c r="J5" s="7">
-        <v>46320</v>
-      </c>
-      <c r="K5" s="7">
-        <v>46351</v>
-      </c>
-      <c r="L5" s="7">
-        <v>46381</v>
-      </c>
-      <c r="M5" s="7">
-        <v>46048</v>
-      </c>
-      <c r="N5" s="7">
-        <v>46079</v>
-      </c>
-      <c r="O5" s="7">
-        <v>46107</v>
-      </c>
-      <c r="P5" s="7">
-        <v>46138</v>
-      </c>
-      <c r="Q5" s="7">
-        <v>46168</v>
-      </c>
-      <c r="R5" s="7">
-        <v>46199</v>
-      </c>
-      <c r="S5" s="7">
-        <v>46229</v>
-      </c>
-      <c r="T5" s="7">
-        <v>46260</v>
-      </c>
-      <c r="U5" s="7">
-        <v>46291</v>
-      </c>
-      <c r="V5" s="7">
-        <v>46321</v>
-      </c>
-      <c r="W5" s="7">
-        <v>46352</v>
-      </c>
-      <c r="X5" s="7">
-        <v>46382</v>
-      </c>
-      <c r="Y5" s="7">
-        <v>46049</v>
-      </c>
-      <c r="Z5" s="7">
-        <v>46080</v>
-      </c>
-      <c r="AA5" s="7">
-        <v>46108</v>
-      </c>
-      <c r="AB5" s="7">
-        <v>46139</v>
-      </c>
-      <c r="AC5" s="7">
-        <v>46169</v>
-      </c>
-      <c r="AD5" s="7">
-        <v>46200</v>
+      <c r="C5" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q5" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="R5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="S5" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="T5" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="U5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="V5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="W5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="X5" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB5" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="AC5" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD5" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="AE5" s="6" t="s">
-        <v>5</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="B6" s="10">
         <v>204329</v>
@@ -865,7 +949,7 @@
     </row>
     <row r="7" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B7" s="10">
         <v>247811</v>
@@ -908,7 +992,7 @@
     </row>
     <row r="8" spans="1:31" ht="80.400000000000006" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="B8" s="10">
         <v>381094</v>
@@ -951,7 +1035,7 @@
     </row>
     <row r="9" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="B9" s="10">
         <v>171649.53</v>
@@ -994,7 +1078,7 @@
     </row>
     <row r="10" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="B10" s="10">
         <v>419106.8</v>
@@ -1037,7 +1121,7 @@
     </row>
     <row r="11" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="B11" s="10">
         <v>215894</v>
@@ -1080,7 +1164,7 @@
     </row>
     <row r="12" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="B12" s="10">
         <v>578949</v>
@@ -1123,7 +1207,7 @@
     </row>
     <row r="13" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="B13" s="10">
         <v>347023</v>
@@ -1166,7 +1250,7 @@
     </row>
     <row r="14" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="B14" s="10">
         <v>204228</v>
@@ -1209,7 +1293,7 @@
     </row>
     <row r="15" spans="1:31" ht="69" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="B15" s="10">
         <v>990489.03</v>
@@ -1254,7 +1338,7 @@
     </row>
     <row r="16" spans="1:31" ht="69" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="B16" s="10">
         <v>80000</v>
@@ -1295,7 +1379,7 @@
     </row>
     <row r="17" spans="1:31" ht="69" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="B17" s="10">
         <v>685243</v>
@@ -1338,7 +1422,7 @@
     </row>
     <row r="18" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="B18" s="10">
         <v>407876</v>
@@ -1381,7 +1465,7 @@
     </row>
     <row r="19" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="B19" s="10">
         <v>172970</v>
@@ -1424,7 +1508,7 @@
     </row>
     <row r="20" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="B20" s="10">
         <v>521250.5</v>
@@ -1467,7 +1551,7 @@
     </row>
     <row r="21" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="B21" s="10">
         <v>239148</v>
@@ -1510,7 +1594,7 @@
     </row>
     <row r="22" spans="1:31" ht="69" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="B22" s="10">
         <v>394488</v>
@@ -1553,7 +1637,7 @@
     </row>
     <row r="23" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="B23" s="10">
         <v>283387</v>
@@ -1596,7 +1680,7 @@
     </row>
     <row r="24" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="B24" s="10">
         <v>58000</v>
@@ -1639,7 +1723,7 @@
     </row>
     <row r="25" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="B25" s="10">
         <v>490896</v>
@@ -1684,7 +1768,7 @@
     </row>
     <row r="26" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="B26" s="12">
         <v>7093831.8600000003</v>
@@ -1779,7 +1863,7 @@
     </row>
     <row r="28" spans="1:31" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -1819,97 +1903,97 @@
       <c r="B29" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C29" s="7">
-        <v>46106</v>
-      </c>
-      <c r="D29" s="7">
-        <v>46137</v>
-      </c>
-      <c r="E29" s="7">
-        <v>46167</v>
-      </c>
-      <c r="F29" s="7">
-        <v>46198</v>
-      </c>
-      <c r="G29" s="7">
-        <v>46228</v>
-      </c>
-      <c r="H29" s="7">
-        <v>46259</v>
-      </c>
-      <c r="I29" s="7">
-        <v>46290</v>
-      </c>
-      <c r="J29" s="7">
-        <v>46320</v>
-      </c>
-      <c r="K29" s="7">
-        <v>46351</v>
-      </c>
-      <c r="L29" s="7">
-        <v>46381</v>
-      </c>
-      <c r="M29" s="7">
-        <v>46048</v>
-      </c>
-      <c r="N29" s="7">
-        <v>46079</v>
-      </c>
-      <c r="O29" s="7">
-        <v>46107</v>
-      </c>
-      <c r="P29" s="7">
-        <v>46138</v>
-      </c>
-      <c r="Q29" s="7">
-        <v>46168</v>
-      </c>
-      <c r="R29" s="7">
-        <v>46199</v>
-      </c>
-      <c r="S29" s="7">
-        <v>46229</v>
-      </c>
-      <c r="T29" s="7">
-        <v>46260</v>
-      </c>
-      <c r="U29" s="7">
-        <v>46291</v>
-      </c>
-      <c r="V29" s="7">
-        <v>46321</v>
-      </c>
-      <c r="W29" s="7">
-        <v>46352</v>
-      </c>
-      <c r="X29" s="7">
-        <v>46382</v>
-      </c>
-      <c r="Y29" s="7">
-        <v>46049</v>
-      </c>
-      <c r="Z29" s="7">
-        <v>46080</v>
-      </c>
-      <c r="AA29" s="7">
-        <v>46108</v>
-      </c>
-      <c r="AB29" s="7">
-        <v>46139</v>
-      </c>
-      <c r="AC29" s="7">
-        <v>46169</v>
-      </c>
-      <c r="AD29" s="7">
-        <v>46200</v>
+      <c r="C29" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J29" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="K29" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="L29" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="M29" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="N29" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="O29" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P29" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q29" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="R29" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="S29" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="T29" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="U29" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="V29" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="W29" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="X29" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y29" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z29" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA29" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB29" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="AC29" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD29" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="AE29" s="6" t="s">
-        <v>5</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="B30" s="10">
         <v>326786.36</v>
@@ -1954,7 +2038,7 @@
     </row>
     <row r="31" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B31" s="10">
         <v>409599.64</v>
@@ -1997,7 +2081,7 @@
     </row>
     <row r="32" spans="1:31" ht="80.400000000000006" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="B32" s="10">
         <v>576317.9</v>
@@ -2040,7 +2124,7 @@
     </row>
     <row r="33" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="B33" s="10">
         <v>322961.08</v>
@@ -2083,7 +2167,7 @@
     </row>
     <row r="34" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="B34" s="10">
         <v>630619.19999999995</v>
@@ -2126,7 +2210,7 @@
     </row>
     <row r="35" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="B35" s="10">
         <v>338450.2</v>
@@ -2169,7 +2253,7 @@
     </row>
     <row r="36" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="B36" s="10">
         <v>1156111.18</v>
@@ -2212,7 +2296,7 @@
     </row>
     <row r="37" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="B37" s="10">
         <v>594114</v>
@@ -2255,7 +2339,7 @@
     </row>
     <row r="38" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="B38" s="10">
         <v>327102.8</v>
@@ -2298,7 +2382,7 @@
     </row>
     <row r="39" spans="1:31" ht="69" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="B39" s="10">
         <v>1707089</v>
@@ -2343,7 +2427,7 @@
     </row>
     <row r="40" spans="1:31" ht="69" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="B40" s="10">
         <v>80000</v>
@@ -2384,7 +2468,7 @@
     </row>
     <row r="41" spans="1:31" ht="69" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="B41" s="10">
         <v>1199960.02</v>
@@ -2427,7 +2511,7 @@
     </row>
     <row r="42" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="B42" s="10">
         <v>600000</v>
@@ -2470,7 +2554,7 @@
     </row>
     <row r="43" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A43" s="9" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="B43" s="10">
         <v>317648</v>
@@ -2513,7 +2597,7 @@
     </row>
     <row r="44" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="B44" s="10">
         <v>832813</v>
@@ -2556,7 +2640,7 @@
     </row>
     <row r="45" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="B45" s="10">
         <v>341236.34</v>
@@ -2599,7 +2683,7 @@
     </row>
     <row r="46" spans="1:31" ht="69" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="B46" s="10">
         <v>666700</v>
@@ -2642,7 +2726,7 @@
     </row>
     <row r="47" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="B47" s="10">
         <v>460000</v>
@@ -2685,7 +2769,7 @@
     </row>
     <row r="48" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="B48" s="10">
         <v>206880</v>
@@ -2728,7 +2812,7 @@
     </row>
     <row r="49" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="B49" s="10">
         <v>799875</v>
@@ -2773,7 +2857,7 @@
     </row>
     <row r="50" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="B50" s="12">
         <v>11894263.719999999</v>
@@ -2868,7 +2952,7 @@
     </row>
     <row r="52" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>

</xml_diff>

<commit_message>
Rebuild Excel export in the IAQ Construction form
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -2995,4 +2995,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7BD3B104-9ADA-4665-A2A5-7653CB6F4F54}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98452712-719C-4C9F-829B-6D7F4742FDF2}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F270FCD-7F77-41D6-9446-9B8558CEA253}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-10 15:33)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/.dashboard-repo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Dashboard\.dashboard-repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8D79197E-E372-4D57-9C5F-A06345C51491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{63E5A9AB-A611-4CCA-B02E-2FB82A0F6521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{02D4ED39-8C7B-42B8-BF59-76F77D0E6138}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{3A182371-689F-4AB0-9027-60B39D162AFC}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="58">
   <si>
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (20 โครงการ PO)</t>
   </si>
@@ -47,7 +47,7 @@
     <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-10</t>
   </si>
   <si>
-    <t>① Cost รายเดือน (฿)</t>
+    <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
   </si>
   <si>
     <t>โครงการ (Project)</t>
@@ -56,6 +56,9 @@
     <t>Total (฿)</t>
   </si>
   <si>
+    <t>Feb-25</t>
+  </si>
+  <si>
     <t>Mar-25</t>
   </si>
   <si>
@@ -206,10 +209,10 @@
     <t>รวมทั้งหมด (Total)</t>
   </si>
   <si>
-    <t>② Forecast Revenue รายเดือน (฿)  —  งวด 40/40/20 (Cons.Start / FF / SF)</t>
-  </si>
-  <si>
-    <t>หมายเหตุ: งวดตามวัน Start Date / End Date (First Fix) / Delivery Date จาก Master Schedule · Cost = Budget Actual, Forecast = Sale Price จาก Summary Report</t>
+    <t>② Forecast Revenue รายเดือน (฿)  —  รับงวด 1-3 ตามวันที่จริง</t>
+  </si>
+  <si>
+    <t>หมายเหตุ: ตัวเลขชุดเดียวกับกราฟ Financial Forecast บน Dashboard · Cost = เงินจ่ายผู้รับเหมา คอลัมน์ K/N/P ลงตามวันที่ L/O/Q · Forecast = รับงวด 1 (Sale Price x 40% ลงวันที่ L) + งวด 2 (คอลัมน์ S วันที่ T) + งวด 3 (คอลัมน์ U วันที่ V) · นับเฉพาะรายการที่มีวันที่ในชีต</t>
   </si>
 </sst>
 </file>
@@ -691,18 +694,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82B05CFD-A9B7-4A0F-BA78-8B2DE727E57C}">
-  <dimension ref="A1:AE52"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C3620D9-DE81-4A50-ACC9-47BD8B542B35}">
+  <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
     <col min="2" max="2" width="15" style="1" customWidth="1"/>
-    <col min="3" max="30" width="11" style="1" customWidth="1"/>
-    <col min="31" max="31" width="15" style="1" customWidth="1"/>
-    <col min="32" max="16384" width="8.88671875" style="1"/>
+    <col min="3" max="31" width="11" style="1" customWidth="1"/>
+    <col min="32" max="32" width="15" style="1" customWidth="1"/>
+    <col min="33" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:32" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -736,8 +739,9 @@
       <c r="AC1" s="2"/>
       <c r="AD1" s="2"/>
       <c r="AE1" s="2"/>
-    </row>
-    <row r="2" spans="1:31" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AF1" s="2"/>
+    </row>
+    <row r="2" spans="1:32" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -771,8 +775,9 @@
       <c r="AC2" s="3"/>
       <c r="AD2" s="3"/>
       <c r="AE2" s="3"/>
-    </row>
-    <row r="4" spans="1:31" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF2" s="3"/>
+    </row>
+    <row r="4" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -806,8 +811,9 @@
       <c r="AC4" s="5"/>
       <c r="AD4" s="5"/>
       <c r="AE4" s="5"/>
-    </row>
-    <row r="5" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF4" s="5"/>
+    </row>
+    <row r="5" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
@@ -898,16 +904,19 @@
       <c r="AD5" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="AE5" s="6" t="s">
+      <c r="AE5" s="7" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="6" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="AF5" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6" s="10">
-        <v>204329</v>
+        <v>117000</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
@@ -922,17 +931,17 @@
       <c r="M6" s="8"/>
       <c r="N6" s="8"/>
       <c r="O6" s="8">
-        <v>81731.600000000006</v>
-      </c>
-      <c r="P6" s="8">
-        <v>81731.600000000006</v>
-      </c>
-      <c r="Q6" s="8"/>
+        <v>39000</v>
+      </c>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8">
+        <v>65000</v>
+      </c>
       <c r="R6" s="8"/>
-      <c r="S6" s="8"/>
-      <c r="T6" s="8">
-        <v>40865.800000000003</v>
-      </c>
+      <c r="S6" s="8">
+        <v>13000</v>
+      </c>
+      <c r="T6" s="8"/>
       <c r="U6" s="8"/>
       <c r="V6" s="8"/>
       <c r="W6" s="8"/>
@@ -943,16 +952,17 @@
       <c r="AB6" s="8"/>
       <c r="AC6" s="8"/>
       <c r="AD6" s="8"/>
-      <c r="AE6" s="10">
-        <v>204329</v>
-      </c>
-    </row>
-    <row r="7" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="AE6" s="8"/>
+      <c r="AF6" s="10">
+        <v>117000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="10">
-        <v>247811</v>
+        <v>139446</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
@@ -973,29 +983,32 @@
       <c r="S7" s="8"/>
       <c r="T7" s="8"/>
       <c r="U7" s="8">
-        <v>198248.80000000002</v>
-      </c>
-      <c r="V7" s="8"/>
-      <c r="W7" s="8"/>
-      <c r="X7" s="8">
-        <v>49562.200000000004</v>
-      </c>
+        <v>41833.799999999996</v>
+      </c>
+      <c r="V7" s="8">
+        <v>69723</v>
+      </c>
+      <c r="W7" s="8">
+        <v>27889.200000000001</v>
+      </c>
+      <c r="X7" s="8"/>
       <c r="Y7" s="8"/>
       <c r="Z7" s="8"/>
       <c r="AA7" s="8"/>
       <c r="AB7" s="8"/>
       <c r="AC7" s="8"/>
       <c r="AD7" s="8"/>
-      <c r="AE7" s="10">
-        <v>247811</v>
-      </c>
-    </row>
-    <row r="8" spans="1:31" ht="80.400000000000006" x14ac:dyDescent="0.25">
+      <c r="AE7" s="8"/>
+      <c r="AF7" s="10">
+        <v>139446</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B8" s="10">
-        <v>381094</v>
+        <v>280000</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
@@ -1010,15 +1023,17 @@
       <c r="M8" s="8"/>
       <c r="N8" s="8"/>
       <c r="O8" s="8">
-        <v>304875.2</v>
-      </c>
-      <c r="P8" s="8"/>
+        <v>84000</v>
+      </c>
+      <c r="P8" s="8">
+        <v>140000</v>
+      </c>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="8">
-        <v>76218.8</v>
-      </c>
-      <c r="T8" s="8"/>
+      <c r="S8" s="8"/>
+      <c r="T8" s="8">
+        <v>56000</v>
+      </c>
       <c r="U8" s="8"/>
       <c r="V8" s="8"/>
       <c r="W8" s="8"/>
@@ -1029,16 +1044,17 @@
       <c r="AB8" s="8"/>
       <c r="AC8" s="8"/>
       <c r="AD8" s="8"/>
-      <c r="AE8" s="10">
-        <v>381094</v>
-      </c>
-    </row>
-    <row r="9" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="AE8" s="8"/>
+      <c r="AF8" s="10">
+        <v>280000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9" s="10">
-        <v>171649.53</v>
+        <v>89000</v>
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
@@ -1054,13 +1070,13 @@
       <c r="N9" s="8"/>
       <c r="O9" s="8"/>
       <c r="P9" s="8"/>
-      <c r="Q9" s="8">
-        <v>34329.906000000003</v>
-      </c>
+      <c r="Q9" s="8"/>
       <c r="R9" s="8">
-        <v>137319.62400000001</v>
-      </c>
-      <c r="S9" s="8"/>
+        <v>71200</v>
+      </c>
+      <c r="S9" s="8">
+        <v>17800</v>
+      </c>
       <c r="T9" s="8"/>
       <c r="U9" s="8"/>
       <c r="V9" s="8"/>
@@ -1072,16 +1088,17 @@
       <c r="AB9" s="8"/>
       <c r="AC9" s="8"/>
       <c r="AD9" s="8"/>
-      <c r="AE9" s="10">
-        <v>171649.53</v>
-      </c>
-    </row>
-    <row r="10" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="AE9" s="8"/>
+      <c r="AF9" s="10">
+        <v>89000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B10" s="10">
-        <v>419106.8</v>
+        <v>0</v>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
@@ -1105,26 +1122,23 @@
       <c r="V10" s="8"/>
       <c r="W10" s="8"/>
       <c r="X10" s="8"/>
-      <c r="Y10" s="8">
-        <v>335285.44</v>
-      </c>
-      <c r="Z10" s="8">
-        <v>83821.36</v>
-      </c>
+      <c r="Y10" s="8"/>
+      <c r="Z10" s="8"/>
       <c r="AA10" s="8"/>
       <c r="AB10" s="8"/>
       <c r="AC10" s="8"/>
       <c r="AD10" s="8"/>
-      <c r="AE10" s="10">
-        <v>419106.8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="AE10" s="8"/>
+      <c r="AF10" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B11" s="10">
-        <v>215894</v>
+        <v>138000</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
@@ -1140,13 +1154,13 @@
       <c r="N11" s="8"/>
       <c r="O11" s="8"/>
       <c r="P11" s="8"/>
-      <c r="Q11" s="8">
-        <v>86357.6</v>
-      </c>
+      <c r="Q11" s="8"/>
       <c r="R11" s="8">
-        <v>129536.40000000001</v>
-      </c>
-      <c r="S11" s="8"/>
+        <v>41400</v>
+      </c>
+      <c r="S11" s="8">
+        <v>96600</v>
+      </c>
       <c r="T11" s="8"/>
       <c r="U11" s="8"/>
       <c r="V11" s="8"/>
@@ -1158,16 +1172,17 @@
       <c r="AB11" s="8"/>
       <c r="AC11" s="8"/>
       <c r="AD11" s="8"/>
-      <c r="AE11" s="10">
-        <v>215894</v>
-      </c>
-    </row>
-    <row r="12" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="AE11" s="8"/>
+      <c r="AF11" s="10">
+        <v>138000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B12" s="10">
-        <v>578949</v>
+        <v>280000</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
@@ -1185,15 +1200,17 @@
       <c r="P12" s="8"/>
       <c r="Q12" s="8"/>
       <c r="R12" s="8">
-        <v>463159.2</v>
+        <v>84000</v>
       </c>
       <c r="S12" s="8"/>
-      <c r="T12" s="8"/>
+      <c r="T12" s="8">
+        <v>140000</v>
+      </c>
       <c r="U12" s="8"/>
-      <c r="V12" s="8">
-        <v>115789.8</v>
-      </c>
-      <c r="W12" s="8"/>
+      <c r="V12" s="8"/>
+      <c r="W12" s="8">
+        <v>56000</v>
+      </c>
       <c r="X12" s="8"/>
       <c r="Y12" s="8"/>
       <c r="Z12" s="8"/>
@@ -1201,16 +1218,17 @@
       <c r="AB12" s="8"/>
       <c r="AC12" s="8"/>
       <c r="AD12" s="8"/>
-      <c r="AE12" s="10">
-        <v>578949</v>
-      </c>
-    </row>
-    <row r="13" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="AE12" s="8"/>
+      <c r="AF12" s="10">
+        <v>280000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B13" s="10">
-        <v>347023</v>
+        <v>233247.9</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
@@ -1233,27 +1251,28 @@
       <c r="U13" s="8"/>
       <c r="V13" s="8"/>
       <c r="W13" s="8"/>
-      <c r="X13" s="8">
-        <v>277618.40000000002</v>
-      </c>
-      <c r="Y13" s="8"/>
+      <c r="X13" s="8"/>
+      <c r="Y13" s="8">
+        <v>69974.37</v>
+      </c>
       <c r="Z13" s="8">
-        <v>69404.600000000006</v>
+        <v>163273.53</v>
       </c>
       <c r="AA13" s="8"/>
       <c r="AB13" s="8"/>
       <c r="AC13" s="8"/>
       <c r="AD13" s="8"/>
-      <c r="AE13" s="10">
-        <v>347023</v>
-      </c>
-    </row>
-    <row r="14" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="AE13" s="8"/>
+      <c r="AF13" s="10">
+        <v>233247.9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B14" s="10">
-        <v>204228</v>
+        <v>120000</v>
       </c>
       <c r="C14" s="8"/>
       <c r="D14" s="8"/>
@@ -1270,33 +1289,36 @@
       <c r="O14" s="8"/>
       <c r="P14" s="8"/>
       <c r="Q14" s="8"/>
-      <c r="R14" s="8"/>
+      <c r="R14" s="8">
+        <v>36000</v>
+      </c>
       <c r="S14" s="8"/>
-      <c r="T14" s="8">
-        <v>163382.40000000002</v>
-      </c>
-      <c r="U14" s="8"/>
+      <c r="T14" s="8"/>
+      <c r="U14" s="8">
+        <v>60000</v>
+      </c>
       <c r="V14" s="8"/>
       <c r="W14" s="8"/>
-      <c r="X14" s="8"/>
-      <c r="Y14" s="8">
-        <v>40845.600000000006</v>
-      </c>
+      <c r="X14" s="8">
+        <v>24000</v>
+      </c>
+      <c r="Y14" s="8"/>
       <c r="Z14" s="8"/>
       <c r="AA14" s="8"/>
       <c r="AB14" s="8"/>
       <c r="AC14" s="8"/>
       <c r="AD14" s="8"/>
-      <c r="AE14" s="10">
-        <v>204228</v>
-      </c>
-    </row>
-    <row r="15" spans="1:31" ht="69" x14ac:dyDescent="0.25">
+      <c r="AE14" s="8"/>
+      <c r="AF14" s="10">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B15" s="10">
-        <v>990489.03</v>
+        <v>656679.03</v>
       </c>
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
@@ -1313,14 +1335,12 @@
       <c r="O15" s="8"/>
       <c r="P15" s="8"/>
       <c r="Q15" s="8"/>
-      <c r="R15" s="8">
-        <v>396195.61200000002</v>
-      </c>
+      <c r="R15" s="8"/>
       <c r="S15" s="8">
-        <v>396195.61200000002</v>
+        <v>197003.709</v>
       </c>
       <c r="T15" s="8">
-        <v>198097.80600000001</v>
+        <v>459675.321</v>
       </c>
       <c r="U15" s="8"/>
       <c r="V15" s="8"/>
@@ -1332,16 +1352,17 @@
       <c r="AB15" s="8"/>
       <c r="AC15" s="8"/>
       <c r="AD15" s="8"/>
-      <c r="AE15" s="10">
-        <v>990489.03</v>
-      </c>
-    </row>
-    <row r="16" spans="1:31" ht="69" x14ac:dyDescent="0.25">
+      <c r="AE15" s="8"/>
+      <c r="AF15" s="10">
+        <v>656679.03</v>
+      </c>
+    </row>
+    <row r="16" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B16" s="10">
-        <v>80000</v>
+        <v>40000</v>
       </c>
       <c r="C16" s="8"/>
       <c r="D16" s="8"/>
@@ -1359,7 +1380,7 @@
       <c r="P16" s="8"/>
       <c r="Q16" s="8"/>
       <c r="R16" s="8">
-        <v>80000</v>
+        <v>40000</v>
       </c>
       <c r="S16" s="8"/>
       <c r="T16" s="8"/>
@@ -1373,16 +1394,17 @@
       <c r="AB16" s="8"/>
       <c r="AC16" s="8"/>
       <c r="AD16" s="8"/>
-      <c r="AE16" s="10">
-        <v>80000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:31" ht="69" x14ac:dyDescent="0.25">
+      <c r="AE16" s="8"/>
+      <c r="AF16" s="10">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17" s="10">
-        <v>685243</v>
+        <v>430000</v>
       </c>
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
@@ -1403,29 +1425,32 @@
       <c r="S17" s="8"/>
       <c r="T17" s="8"/>
       <c r="U17" s="8">
-        <v>548194.4</v>
+        <v>129000</v>
       </c>
       <c r="V17" s="8"/>
-      <c r="W17" s="8"/>
-      <c r="X17" s="8">
-        <v>137048.6</v>
-      </c>
-      <c r="Y17" s="8"/>
+      <c r="W17" s="8">
+        <v>215000</v>
+      </c>
+      <c r="X17" s="8"/>
+      <c r="Y17" s="8">
+        <v>86000</v>
+      </c>
       <c r="Z17" s="8"/>
       <c r="AA17" s="8"/>
       <c r="AB17" s="8"/>
       <c r="AC17" s="8"/>
       <c r="AD17" s="8"/>
-      <c r="AE17" s="10">
-        <v>685243</v>
-      </c>
-    </row>
-    <row r="18" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="AE17" s="8"/>
+      <c r="AF17" s="10">
+        <v>430000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B18" s="10">
-        <v>407876</v>
+        <v>234861</v>
       </c>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -1440,12 +1465,12 @@
       <c r="M18" s="8"/>
       <c r="N18" s="8"/>
       <c r="O18" s="8">
-        <v>326300.80000000005</v>
-      </c>
-      <c r="P18" s="8">
-        <v>81575.200000000012</v>
-      </c>
-      <c r="Q18" s="8"/>
+        <v>70458.3</v>
+      </c>
+      <c r="P18" s="8"/>
+      <c r="Q18" s="8">
+        <v>164402.70000000001</v>
+      </c>
       <c r="R18" s="8"/>
       <c r="S18" s="8"/>
       <c r="T18" s="8"/>
@@ -1459,16 +1484,17 @@
       <c r="AB18" s="8"/>
       <c r="AC18" s="8"/>
       <c r="AD18" s="8"/>
-      <c r="AE18" s="10">
-        <v>407876</v>
-      </c>
-    </row>
-    <row r="19" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="AE18" s="8"/>
+      <c r="AF18" s="10">
+        <v>234861</v>
+      </c>
+    </row>
+    <row r="19" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B19" s="10">
-        <v>172970</v>
+        <v>119980</v>
       </c>
       <c r="C19" s="8"/>
       <c r="D19" s="8"/>
@@ -1483,10 +1509,10 @@
       <c r="M19" s="8"/>
       <c r="N19" s="8"/>
       <c r="O19" s="8">
-        <v>138376</v>
+        <v>35994</v>
       </c>
       <c r="P19" s="8">
-        <v>34594</v>
+        <v>83986</v>
       </c>
       <c r="Q19" s="8"/>
       <c r="R19" s="8"/>
@@ -1502,16 +1528,17 @@
       <c r="AB19" s="8"/>
       <c r="AC19" s="8"/>
       <c r="AD19" s="8"/>
-      <c r="AE19" s="10">
-        <v>172970</v>
-      </c>
-    </row>
-    <row r="20" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="AE19" s="8"/>
+      <c r="AF19" s="10">
+        <v>119980</v>
+      </c>
+    </row>
+    <row r="20" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B20" s="10">
-        <v>521250.5</v>
+        <v>280000</v>
       </c>
       <c r="C20" s="8"/>
       <c r="D20" s="8"/>
@@ -1531,12 +1558,14 @@
       <c r="R20" s="8"/>
       <c r="S20" s="8"/>
       <c r="T20" s="8">
-        <v>417000.4</v>
-      </c>
-      <c r="U20" s="8"/>
+        <v>84000</v>
+      </c>
+      <c r="U20" s="8">
+        <v>140000</v>
+      </c>
       <c r="V20" s="8"/>
       <c r="W20" s="8">
-        <v>104250.1</v>
+        <v>56000</v>
       </c>
       <c r="X20" s="8"/>
       <c r="Y20" s="8"/>
@@ -1545,21 +1574,24 @@
       <c r="AB20" s="8"/>
       <c r="AC20" s="8"/>
       <c r="AD20" s="8"/>
-      <c r="AE20" s="10">
-        <v>521250.5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="AE20" s="8"/>
+      <c r="AF20" s="10">
+        <v>280000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B21" s="10">
         <v>239148</v>
       </c>
       <c r="C21" s="8">
-        <v>191318.40000000002</v>
-      </c>
-      <c r="D21" s="8"/>
+        <v>71744.399999999994</v>
+      </c>
+      <c r="D21" s="8">
+        <v>119574</v>
+      </c>
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
       <c r="G21" s="8"/>
@@ -1575,11 +1607,11 @@
       <c r="Q21" s="8"/>
       <c r="R21" s="8"/>
       <c r="S21" s="8"/>
-      <c r="T21" s="8">
+      <c r="T21" s="8"/>
+      <c r="U21" s="8"/>
+      <c r="V21" s="8">
         <v>47829.600000000006</v>
       </c>
-      <c r="U21" s="8"/>
-      <c r="V21" s="8"/>
       <c r="W21" s="8"/>
       <c r="X21" s="8"/>
       <c r="Y21" s="8"/>
@@ -1588,21 +1620,24 @@
       <c r="AB21" s="8"/>
       <c r="AC21" s="8"/>
       <c r="AD21" s="8"/>
-      <c r="AE21" s="10">
+      <c r="AE21" s="8"/>
+      <c r="AF21" s="10">
         <v>239148</v>
       </c>
     </row>
-    <row r="22" spans="1:31" ht="69" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B22" s="10">
-        <v>394488</v>
+        <v>224226.99999999997</v>
       </c>
       <c r="C22" s="8">
-        <v>315590.40000000002</v>
-      </c>
-      <c r="D22" s="8"/>
+        <v>67268.099999999991</v>
+      </c>
+      <c r="D22" s="8">
+        <v>112113.5</v>
+      </c>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
@@ -1619,10 +1654,10 @@
       <c r="R22" s="8"/>
       <c r="S22" s="8"/>
       <c r="T22" s="8"/>
-      <c r="U22" s="8">
-        <v>78897.600000000006</v>
-      </c>
-      <c r="V22" s="8"/>
+      <c r="U22" s="8"/>
+      <c r="V22" s="8">
+        <v>44845.4</v>
+      </c>
       <c r="W22" s="8"/>
       <c r="X22" s="8"/>
       <c r="Y22" s="8"/>
@@ -1631,16 +1666,17 @@
       <c r="AB22" s="8"/>
       <c r="AC22" s="8"/>
       <c r="AD22" s="8"/>
-      <c r="AE22" s="10">
-        <v>394488</v>
-      </c>
-    </row>
-    <row r="23" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="AE22" s="8"/>
+      <c r="AF22" s="10">
+        <v>224226.99999999997</v>
+      </c>
+    </row>
+    <row r="23" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B23" s="10">
-        <v>283387</v>
+        <v>215000</v>
       </c>
       <c r="C23" s="8"/>
       <c r="D23" s="8"/>
@@ -1661,10 +1697,12 @@
       <c r="S23" s="8"/>
       <c r="T23" s="8"/>
       <c r="U23" s="8">
-        <v>226709.6</v>
+        <v>64500</v>
       </c>
       <c r="V23" s="8"/>
-      <c r="W23" s="8"/>
+      <c r="W23" s="8">
+        <v>107500</v>
+      </c>
       <c r="X23" s="8"/>
       <c r="Y23" s="8"/>
       <c r="Z23" s="8"/>
@@ -1672,18 +1710,19 @@
       <c r="AB23" s="8"/>
       <c r="AC23" s="8"/>
       <c r="AD23" s="8">
-        <v>56677.4</v>
-      </c>
-      <c r="AE23" s="10">
-        <v>283387</v>
-      </c>
-    </row>
-    <row r="24" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
+        <v>43000</v>
+      </c>
+      <c r="AE23" s="8"/>
+      <c r="AF23" s="10">
+        <v>215000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B24" s="10">
-        <v>58000</v>
+        <v>116000</v>
       </c>
       <c r="C24" s="8"/>
       <c r="D24" s="8"/>
@@ -1701,13 +1740,11 @@
       <c r="P24" s="8"/>
       <c r="Q24" s="8"/>
       <c r="R24" s="8"/>
-      <c r="S24" s="8">
-        <v>23200</v>
-      </c>
-      <c r="T24" s="8">
-        <v>34800</v>
-      </c>
-      <c r="U24" s="8"/>
+      <c r="S24" s="8"/>
+      <c r="T24" s="8"/>
+      <c r="U24" s="8">
+        <v>116000</v>
+      </c>
       <c r="V24" s="8"/>
       <c r="W24" s="8"/>
       <c r="X24" s="8"/>
@@ -1717,16 +1754,17 @@
       <c r="AB24" s="8"/>
       <c r="AC24" s="8"/>
       <c r="AD24" s="8"/>
-      <c r="AE24" s="10">
-        <v>58000</v>
-      </c>
-    </row>
-    <row r="25" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="AE24" s="8"/>
+      <c r="AF24" s="10">
+        <v>116000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B25" s="10">
-        <v>490896</v>
+        <v>341476</v>
       </c>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
@@ -1746,38 +1784,39 @@
       <c r="R25" s="8"/>
       <c r="S25" s="8"/>
       <c r="T25" s="8"/>
-      <c r="U25" s="8">
-        <v>196358.40000000002</v>
-      </c>
+      <c r="U25" s="8"/>
       <c r="V25" s="8">
-        <v>196358.40000000002</v>
-      </c>
-      <c r="W25" s="8"/>
+        <v>102442.8</v>
+      </c>
+      <c r="W25" s="8">
+        <v>170738</v>
+      </c>
       <c r="X25" s="8"/>
       <c r="Y25" s="8"/>
       <c r="Z25" s="8"/>
       <c r="AA25" s="8">
-        <v>98179.200000000012</v>
+        <v>68295.199999999997</v>
       </c>
       <c r="AB25" s="8"/>
       <c r="AC25" s="8"/>
       <c r="AD25" s="8"/>
-      <c r="AE25" s="10">
-        <v>490896</v>
-      </c>
-    </row>
-    <row r="26" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AE25" s="8"/>
+      <c r="AF25" s="10">
+        <v>341476</v>
+      </c>
+    </row>
+    <row r="26" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B26" s="12">
-        <v>7093831.8600000003</v>
+        <v>4294064.93</v>
       </c>
       <c r="C26" s="12">
-        <v>506908.80000000005</v>
+        <v>139012.5</v>
       </c>
       <c r="D26" s="12">
-        <v>0</v>
+        <v>231687.5</v>
       </c>
       <c r="E26" s="12">
         <v>0</v>
@@ -1810,43 +1849,43 @@
         <v>0</v>
       </c>
       <c r="O26" s="12">
-        <v>851283.60000000009</v>
+        <v>229452.3</v>
       </c>
       <c r="P26" s="12">
-        <v>197900.80000000002</v>
+        <v>223986</v>
       </c>
       <c r="Q26" s="12">
-        <v>120687.50600000001</v>
+        <v>229402.7</v>
       </c>
       <c r="R26" s="12">
-        <v>1206210.8360000001</v>
+        <v>272600</v>
       </c>
       <c r="S26" s="12">
-        <v>495614.41200000001</v>
+        <v>324403.70900000003</v>
       </c>
       <c r="T26" s="12">
-        <v>901976.00600000005</v>
+        <v>739675.321</v>
       </c>
       <c r="U26" s="12">
-        <v>1248408.8000000003</v>
+        <v>551333.80000000005</v>
       </c>
       <c r="V26" s="12">
-        <v>312148.2</v>
+        <v>264840.8</v>
       </c>
       <c r="W26" s="12">
-        <v>104250.1</v>
+        <v>633127.19999999995</v>
       </c>
       <c r="X26" s="12">
-        <v>464229.20000000007</v>
+        <v>24000</v>
       </c>
       <c r="Y26" s="12">
-        <v>376131.04000000004</v>
+        <v>155974.37</v>
       </c>
       <c r="Z26" s="12">
-        <v>153225.96000000002</v>
+        <v>163273.53</v>
       </c>
       <c r="AA26" s="12">
-        <v>98179.200000000012</v>
+        <v>68295.199999999997</v>
       </c>
       <c r="AB26" s="12">
         <v>0</v>
@@ -1855,15 +1894,18 @@
         <v>0</v>
       </c>
       <c r="AD26" s="12">
-        <v>56677.4</v>
+        <v>43000</v>
       </c>
       <c r="AE26" s="12">
-        <v>7093831.8600000003</v>
-      </c>
-    </row>
-    <row r="28" spans="1:31" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="AF26" s="12">
+        <v>4294064.93</v>
+      </c>
+    </row>
+    <row r="28" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -1895,8 +1937,9 @@
       <c r="AC28" s="5"/>
       <c r="AD28" s="5"/>
       <c r="AE28" s="5"/>
-    </row>
-    <row r="29" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF28" s="5"/>
+    </row>
+    <row r="29" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>3</v>
       </c>
@@ -1987,13 +2030,16 @@
       <c r="AD29" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="AE29" s="6" t="s">
+      <c r="AE29" s="7" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="30" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="AF29" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B30" s="10">
         <v>326786.36</v>
@@ -2013,16 +2059,16 @@
       <c r="O30" s="8">
         <v>130714.54399999999</v>
       </c>
-      <c r="P30" s="8">
-        <v>130714.54399999999</v>
-      </c>
+      <c r="P30" s="8"/>
       <c r="Q30" s="8"/>
       <c r="R30" s="8"/>
       <c r="S30" s="8"/>
       <c r="T30" s="8">
+        <v>130714.54399999999</v>
+      </c>
+      <c r="U30" s="8">
         <v>65357.271999999997</v>
       </c>
-      <c r="U30" s="8"/>
       <c r="V30" s="8"/>
       <c r="W30" s="8"/>
       <c r="X30" s="8"/>
@@ -2032,16 +2078,17 @@
       <c r="AB30" s="8"/>
       <c r="AC30" s="8"/>
       <c r="AD30" s="8"/>
-      <c r="AE30" s="10">
+      <c r="AE30" s="8"/>
+      <c r="AF30" s="10">
         <v>326786.36</v>
       </c>
     </row>
-    <row r="31" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B31" s="10">
-        <v>409599.64</v>
+        <v>409599.64000000007</v>
       </c>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
@@ -2062,29 +2109,32 @@
       <c r="S31" s="8"/>
       <c r="T31" s="8"/>
       <c r="U31" s="8">
-        <v>327679.71200000006</v>
-      </c>
-      <c r="V31" s="8"/>
+        <v>163839.85600000003</v>
+      </c>
+      <c r="V31" s="8">
+        <v>163839.85600000003</v>
+      </c>
       <c r="W31" s="8"/>
-      <c r="X31" s="8">
+      <c r="X31" s="8"/>
+      <c r="Y31" s="8">
         <v>81919.928000000014</v>
       </c>
-      <c r="Y31" s="8"/>
       <c r="Z31" s="8"/>
       <c r="AA31" s="8"/>
       <c r="AB31" s="8"/>
       <c r="AC31" s="8"/>
       <c r="AD31" s="8"/>
-      <c r="AE31" s="10">
-        <v>409599.64</v>
-      </c>
-    </row>
-    <row r="32" spans="1:31" ht="80.400000000000006" x14ac:dyDescent="0.25">
+      <c r="AE31" s="8"/>
+      <c r="AF31" s="10">
+        <v>409599.64000000007</v>
+      </c>
+    </row>
+    <row r="32" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B32" s="10">
-        <v>576317.9</v>
+        <v>537273.12000000011</v>
       </c>
       <c r="C32" s="8"/>
       <c r="D32" s="8"/>
@@ -2099,15 +2149,17 @@
       <c r="M32" s="8"/>
       <c r="N32" s="8"/>
       <c r="O32" s="8">
-        <v>461054.32000000007</v>
-      </c>
-      <c r="P32" s="8"/>
+        <v>230527.16000000003</v>
+      </c>
+      <c r="P32" s="8">
+        <v>230527.16000000003</v>
+      </c>
       <c r="Q32" s="8"/>
       <c r="R32" s="8"/>
-      <c r="S32" s="8">
-        <v>115263.58000000002</v>
-      </c>
-      <c r="T32" s="8"/>
+      <c r="S32" s="8"/>
+      <c r="T32" s="8">
+        <v>76218.8</v>
+      </c>
       <c r="U32" s="8"/>
       <c r="V32" s="8"/>
       <c r="W32" s="8"/>
@@ -2118,16 +2170,17 @@
       <c r="AB32" s="8"/>
       <c r="AC32" s="8"/>
       <c r="AD32" s="8"/>
-      <c r="AE32" s="10">
-        <v>576317.9</v>
-      </c>
-    </row>
-    <row r="33" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="AE32" s="8"/>
+      <c r="AF32" s="10">
+        <v>537273.12000000011</v>
+      </c>
+    </row>
+    <row r="33" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B33" s="10">
-        <v>322961.08</v>
+        <v>387553.29600000003</v>
       </c>
       <c r="C33" s="8"/>
       <c r="D33" s="8"/>
@@ -2143,13 +2196,13 @@
       <c r="N33" s="8"/>
       <c r="O33" s="8"/>
       <c r="P33" s="8"/>
-      <c r="Q33" s="8">
-        <v>64592.216000000008</v>
-      </c>
+      <c r="Q33" s="8"/>
       <c r="R33" s="8">
+        <v>129184.43200000002</v>
+      </c>
+      <c r="S33" s="8">
         <v>258368.86400000003</v>
       </c>
-      <c r="S33" s="8"/>
       <c r="T33" s="8"/>
       <c r="U33" s="8"/>
       <c r="V33" s="8"/>
@@ -2161,16 +2214,17 @@
       <c r="AB33" s="8"/>
       <c r="AC33" s="8"/>
       <c r="AD33" s="8"/>
-      <c r="AE33" s="10">
-        <v>322961.08</v>
-      </c>
-    </row>
-    <row r="34" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="AE33" s="8"/>
+      <c r="AF33" s="10">
+        <v>387553.29600000003</v>
+      </c>
+    </row>
+    <row r="34" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B34" s="10">
-        <v>630619.19999999995</v>
+        <v>252247.67999999999</v>
       </c>
       <c r="C34" s="8"/>
       <c r="D34" s="8"/>
@@ -2195,25 +2249,24 @@
       <c r="W34" s="8"/>
       <c r="X34" s="8"/>
       <c r="Y34" s="8">
-        <v>504495.35999999999</v>
-      </c>
-      <c r="Z34" s="8">
-        <v>126123.84</v>
-      </c>
+        <v>252247.67999999999</v>
+      </c>
+      <c r="Z34" s="8"/>
       <c r="AA34" s="8"/>
       <c r="AB34" s="8"/>
       <c r="AC34" s="8"/>
       <c r="AD34" s="8"/>
-      <c r="AE34" s="10">
-        <v>630619.19999999995</v>
-      </c>
-    </row>
-    <row r="35" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="AE34" s="8"/>
+      <c r="AF34" s="10">
+        <v>252247.67999999999</v>
+      </c>
+    </row>
+    <row r="35" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B35" s="10">
-        <v>338450.2</v>
+        <v>338450.20000000007</v>
       </c>
       <c r="C35" s="8"/>
       <c r="D35" s="8"/>
@@ -2229,14 +2282,16 @@
       <c r="N35" s="8"/>
       <c r="O35" s="8"/>
       <c r="P35" s="8"/>
-      <c r="Q35" s="8">
+      <c r="Q35" s="8"/>
+      <c r="R35" s="8">
         <v>135380.08000000002</v>
       </c>
-      <c r="R35" s="8">
-        <v>203070.12000000002</v>
-      </c>
-      <c r="S35" s="8"/>
-      <c r="T35" s="8"/>
+      <c r="S35" s="8">
+        <v>135380.08000000002</v>
+      </c>
+      <c r="T35" s="8">
+        <v>67690.040000000008</v>
+      </c>
       <c r="U35" s="8"/>
       <c r="V35" s="8"/>
       <c r="W35" s="8"/>
@@ -2247,13 +2302,14 @@
       <c r="AB35" s="8"/>
       <c r="AC35" s="8"/>
       <c r="AD35" s="8"/>
-      <c r="AE35" s="10">
-        <v>338450.2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="AE35" s="8"/>
+      <c r="AF35" s="10">
+        <v>338450.20000000007</v>
+      </c>
+    </row>
+    <row r="36" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B36" s="10">
         <v>1156111.18</v>
@@ -2274,15 +2330,17 @@
       <c r="P36" s="8"/>
       <c r="Q36" s="8"/>
       <c r="R36" s="8">
-        <v>924888.94400000002</v>
+        <v>462444.47200000001</v>
       </c>
       <c r="S36" s="8"/>
-      <c r="T36" s="8"/>
+      <c r="T36" s="8">
+        <v>346833.35399999999</v>
+      </c>
       <c r="U36" s="8"/>
-      <c r="V36" s="8">
-        <v>231222.236</v>
-      </c>
-      <c r="W36" s="8"/>
+      <c r="V36" s="8"/>
+      <c r="W36" s="8">
+        <v>346833.35399999999</v>
+      </c>
       <c r="X36" s="8"/>
       <c r="Y36" s="8"/>
       <c r="Z36" s="8"/>
@@ -2290,13 +2348,14 @@
       <c r="AB36" s="8"/>
       <c r="AC36" s="8"/>
       <c r="AD36" s="8"/>
-      <c r="AE36" s="10">
+      <c r="AE36" s="8"/>
+      <c r="AF36" s="10">
         <v>1156111.18</v>
       </c>
     </row>
-    <row r="37" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B37" s="10">
         <v>594114</v>
@@ -2322,27 +2381,30 @@
       <c r="U37" s="8"/>
       <c r="V37" s="8"/>
       <c r="W37" s="8"/>
-      <c r="X37" s="8">
-        <v>475291.2</v>
-      </c>
-      <c r="Y37" s="8"/>
+      <c r="X37" s="8"/>
+      <c r="Y37" s="8">
+        <v>237645.6</v>
+      </c>
       <c r="Z37" s="8">
+        <v>237645.6</v>
+      </c>
+      <c r="AA37" s="8">
         <v>118822.8</v>
       </c>
-      <c r="AA37" s="8"/>
       <c r="AB37" s="8"/>
       <c r="AC37" s="8"/>
       <c r="AD37" s="8"/>
-      <c r="AE37" s="10">
+      <c r="AE37" s="8"/>
+      <c r="AF37" s="10">
         <v>594114</v>
       </c>
     </row>
-    <row r="38" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B38" s="10">
-        <v>327102.8</v>
+        <v>359813.07999999996</v>
       </c>
       <c r="C38" s="8"/>
       <c r="D38" s="8"/>
@@ -2359,33 +2421,36 @@
       <c r="O38" s="8"/>
       <c r="P38" s="8"/>
       <c r="Q38" s="8"/>
-      <c r="R38" s="8"/>
+      <c r="R38" s="8">
+        <v>130841.12</v>
+      </c>
       <c r="S38" s="8"/>
-      <c r="T38" s="8">
-        <v>261682.24</v>
-      </c>
-      <c r="U38" s="8"/>
+      <c r="T38" s="8"/>
+      <c r="U38" s="8">
+        <v>130841.12</v>
+      </c>
       <c r="V38" s="8"/>
       <c r="W38" s="8"/>
       <c r="X38" s="8"/>
-      <c r="Y38" s="8">
-        <v>65420.56</v>
-      </c>
-      <c r="Z38" s="8"/>
+      <c r="Y38" s="8"/>
+      <c r="Z38" s="8">
+        <v>98130.84</v>
+      </c>
       <c r="AA38" s="8"/>
       <c r="AB38" s="8"/>
       <c r="AC38" s="8"/>
       <c r="AD38" s="8"/>
-      <c r="AE38" s="10">
-        <v>327102.8</v>
-      </c>
-    </row>
-    <row r="39" spans="1:31" ht="69" x14ac:dyDescent="0.25">
+      <c r="AE38" s="8"/>
+      <c r="AF38" s="10">
+        <v>359813.07999999996</v>
+      </c>
+    </row>
+    <row r="39" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B39" s="10">
-        <v>1707089</v>
+        <v>1707089.0000000002</v>
       </c>
       <c r="C39" s="8"/>
       <c r="D39" s="8"/>
@@ -2402,16 +2467,16 @@
       <c r="O39" s="8"/>
       <c r="P39" s="8"/>
       <c r="Q39" s="8"/>
-      <c r="R39" s="8">
-        <v>682835.60000000009</v>
-      </c>
+      <c r="R39" s="8"/>
       <c r="S39" s="8">
         <v>682835.60000000009</v>
       </c>
       <c r="T39" s="8">
+        <v>682835.60000000009</v>
+      </c>
+      <c r="U39" s="8">
         <v>341417.80000000005</v>
       </c>
-      <c r="U39" s="8"/>
       <c r="V39" s="8"/>
       <c r="W39" s="8"/>
       <c r="X39" s="8"/>
@@ -2421,16 +2486,17 @@
       <c r="AB39" s="8"/>
       <c r="AC39" s="8"/>
       <c r="AD39" s="8"/>
-      <c r="AE39" s="10">
-        <v>1707089</v>
-      </c>
-    </row>
-    <row r="40" spans="1:31" ht="69" x14ac:dyDescent="0.25">
+      <c r="AE39" s="8"/>
+      <c r="AF39" s="10">
+        <v>1707089.0000000002</v>
+      </c>
+    </row>
+    <row r="40" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B40" s="10">
-        <v>80000</v>
+        <v>112000</v>
       </c>
       <c r="C40" s="8"/>
       <c r="D40" s="8"/>
@@ -2448,9 +2514,11 @@
       <c r="P40" s="8"/>
       <c r="Q40" s="8"/>
       <c r="R40" s="8">
+        <v>32000</v>
+      </c>
+      <c r="S40" s="8">
         <v>80000</v>
       </c>
-      <c r="S40" s="8"/>
       <c r="T40" s="8"/>
       <c r="U40" s="8"/>
       <c r="V40" s="8"/>
@@ -2462,13 +2530,14 @@
       <c r="AB40" s="8"/>
       <c r="AC40" s="8"/>
       <c r="AD40" s="8"/>
-      <c r="AE40" s="10">
-        <v>80000</v>
-      </c>
-    </row>
-    <row r="41" spans="1:31" ht="69" x14ac:dyDescent="0.25">
+      <c r="AE40" s="8"/>
+      <c r="AF40" s="10">
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B41" s="10">
         <v>1199960.02</v>
@@ -2492,26 +2561,29 @@
       <c r="S41" s="8"/>
       <c r="T41" s="8"/>
       <c r="U41" s="8">
-        <v>959968.01600000006</v>
+        <v>479984.00800000003</v>
       </c>
       <c r="V41" s="8"/>
-      <c r="W41" s="8"/>
-      <c r="X41" s="8">
+      <c r="W41" s="8">
+        <v>479984.00800000003</v>
+      </c>
+      <c r="X41" s="8"/>
+      <c r="Y41" s="8"/>
+      <c r="Z41" s="8">
         <v>239992.00400000002</v>
       </c>
-      <c r="Y41" s="8"/>
-      <c r="Z41" s="8"/>
       <c r="AA41" s="8"/>
       <c r="AB41" s="8"/>
       <c r="AC41" s="8"/>
       <c r="AD41" s="8"/>
-      <c r="AE41" s="10">
+      <c r="AE41" s="8"/>
+      <c r="AF41" s="10">
         <v>1199960.02</v>
       </c>
     </row>
-    <row r="42" spans="1:31" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B42" s="10">
         <v>600000</v>
@@ -2529,13 +2601,15 @@
       <c r="M42" s="8"/>
       <c r="N42" s="8"/>
       <c r="O42" s="8">
-        <v>480000</v>
-      </c>
-      <c r="P42" s="8">
-        <v>120000</v>
-      </c>
-      <c r="Q42" s="8"/>
-      <c r="R42" s="8"/>
+        <v>240000</v>
+      </c>
+      <c r="P42" s="8"/>
+      <c r="Q42" s="8">
+        <v>180000</v>
+      </c>
+      <c r="R42" s="8">
+        <v>180000</v>
+      </c>
       <c r="S42" s="8"/>
       <c r="T42" s="8"/>
       <c r="U42" s="8"/>
@@ -2548,13 +2622,14 @@
       <c r="AB42" s="8"/>
       <c r="AC42" s="8"/>
       <c r="AD42" s="8"/>
-      <c r="AE42" s="10">
+      <c r="AE42" s="8"/>
+      <c r="AF42" s="10">
         <v>600000</v>
       </c>
     </row>
-    <row r="43" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A43" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B43" s="10">
         <v>317648</v>
@@ -2572,13 +2647,15 @@
       <c r="M43" s="8"/>
       <c r="N43" s="8"/>
       <c r="O43" s="8">
-        <v>254118.40000000002</v>
+        <v>127059.20000000001</v>
       </c>
       <c r="P43" s="8">
+        <v>127059.20000000001</v>
+      </c>
+      <c r="Q43" s="8"/>
+      <c r="R43" s="8">
         <v>63529.600000000006</v>
       </c>
-      <c r="Q43" s="8"/>
-      <c r="R43" s="8"/>
       <c r="S43" s="8"/>
       <c r="T43" s="8"/>
       <c r="U43" s="8"/>
@@ -2591,13 +2668,14 @@
       <c r="AB43" s="8"/>
       <c r="AC43" s="8"/>
       <c r="AD43" s="8"/>
-      <c r="AE43" s="10">
+      <c r="AE43" s="8"/>
+      <c r="AF43" s="10">
         <v>317648</v>
       </c>
     </row>
-    <row r="44" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B44" s="10">
         <v>832813</v>
@@ -2620,35 +2698,40 @@
       <c r="R44" s="8"/>
       <c r="S44" s="8"/>
       <c r="T44" s="8">
-        <v>666250.4</v>
-      </c>
-      <c r="U44" s="8"/>
+        <v>333125.2</v>
+      </c>
+      <c r="U44" s="8">
+        <v>333125.2</v>
+      </c>
       <c r="V44" s="8"/>
-      <c r="W44" s="8">
+      <c r="W44" s="8"/>
+      <c r="X44" s="8"/>
+      <c r="Y44" s="8">
         <v>166562.6</v>
       </c>
-      <c r="X44" s="8"/>
-      <c r="Y44" s="8"/>
       <c r="Z44" s="8"/>
       <c r="AA44" s="8"/>
       <c r="AB44" s="8"/>
       <c r="AC44" s="8"/>
       <c r="AD44" s="8"/>
-      <c r="AE44" s="10">
+      <c r="AE44" s="8"/>
+      <c r="AF44" s="10">
         <v>832813</v>
       </c>
     </row>
-    <row r="45" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B45" s="10">
-        <v>341236.34</v>
+        <v>341236.34000000008</v>
       </c>
       <c r="C45" s="8">
-        <v>272989.07200000004</v>
-      </c>
-      <c r="D45" s="8"/>
+        <v>136494.53600000002</v>
+      </c>
+      <c r="D45" s="8">
+        <v>136494.53600000002</v>
+      </c>
       <c r="E45" s="8"/>
       <c r="F45" s="8"/>
       <c r="G45" s="8"/>
@@ -2664,10 +2747,10 @@
       <c r="Q45" s="8"/>
       <c r="R45" s="8"/>
       <c r="S45" s="8"/>
-      <c r="T45" s="8">
+      <c r="T45" s="8"/>
+      <c r="U45" s="8">
         <v>68247.268000000011</v>
       </c>
-      <c r="U45" s="8"/>
       <c r="V45" s="8"/>
       <c r="W45" s="8"/>
       <c r="X45" s="8"/>
@@ -2677,21 +2760,24 @@
       <c r="AB45" s="8"/>
       <c r="AC45" s="8"/>
       <c r="AD45" s="8"/>
-      <c r="AE45" s="10">
-        <v>341236.34</v>
-      </c>
-    </row>
-    <row r="46" spans="1:31" ht="69" x14ac:dyDescent="0.25">
+      <c r="AE45" s="8"/>
+      <c r="AF45" s="10">
+        <v>341236.34000000008</v>
+      </c>
+    </row>
+    <row r="46" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B46" s="10">
         <v>666700</v>
       </c>
       <c r="C46" s="8">
-        <v>533360</v>
-      </c>
-      <c r="D46" s="8"/>
+        <v>266680</v>
+      </c>
+      <c r="D46" s="8">
+        <v>266680</v>
+      </c>
       <c r="E46" s="8"/>
       <c r="F46" s="8"/>
       <c r="G46" s="8"/>
@@ -2708,11 +2794,11 @@
       <c r="R46" s="8"/>
       <c r="S46" s="8"/>
       <c r="T46" s="8"/>
-      <c r="U46" s="8">
+      <c r="U46" s="8"/>
+      <c r="V46" s="8"/>
+      <c r="W46" s="8">
         <v>133340</v>
       </c>
-      <c r="V46" s="8"/>
-      <c r="W46" s="8"/>
       <c r="X46" s="8"/>
       <c r="Y46" s="8"/>
       <c r="Z46" s="8"/>
@@ -2720,13 +2806,14 @@
       <c r="AB46" s="8"/>
       <c r="AC46" s="8"/>
       <c r="AD46" s="8"/>
-      <c r="AE46" s="10">
+      <c r="AE46" s="8"/>
+      <c r="AF46" s="10">
         <v>666700</v>
       </c>
     </row>
-    <row r="47" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B47" s="10">
         <v>460000</v>
@@ -2750,26 +2837,29 @@
       <c r="S47" s="8"/>
       <c r="T47" s="8"/>
       <c r="U47" s="8">
-        <v>368000</v>
+        <v>184000</v>
       </c>
       <c r="V47" s="8"/>
-      <c r="W47" s="8"/>
+      <c r="W47" s="8">
+        <v>184000</v>
+      </c>
       <c r="X47" s="8"/>
       <c r="Y47" s="8"/>
       <c r="Z47" s="8"/>
       <c r="AA47" s="8"/>
       <c r="AB47" s="8"/>
       <c r="AC47" s="8"/>
-      <c r="AD47" s="8">
+      <c r="AD47" s="8"/>
+      <c r="AE47" s="8">
         <v>92000</v>
       </c>
-      <c r="AE47" s="10">
+      <c r="AF47" s="10">
         <v>460000</v>
       </c>
     </row>
-    <row r="48" spans="1:31" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B48" s="10">
         <v>206880</v>
@@ -2790,13 +2880,11 @@
       <c r="P48" s="8"/>
       <c r="Q48" s="8"/>
       <c r="R48" s="8"/>
-      <c r="S48" s="8">
-        <v>82752</v>
-      </c>
-      <c r="T48" s="8">
-        <v>124128</v>
-      </c>
-      <c r="U48" s="8"/>
+      <c r="S48" s="8"/>
+      <c r="T48" s="8"/>
+      <c r="U48" s="8">
+        <v>206880</v>
+      </c>
       <c r="V48" s="8"/>
       <c r="W48" s="8"/>
       <c r="X48" s="8"/>
@@ -2806,13 +2894,14 @@
       <c r="AB48" s="8"/>
       <c r="AC48" s="8"/>
       <c r="AD48" s="8"/>
-      <c r="AE48" s="10">
+      <c r="AE48" s="8"/>
+      <c r="AF48" s="10">
         <v>206880</v>
       </c>
     </row>
-    <row r="49" spans="1:31" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B49" s="10">
         <v>799875</v>
@@ -2835,38 +2924,39 @@
       <c r="R49" s="8"/>
       <c r="S49" s="8"/>
       <c r="T49" s="8"/>
-      <c r="U49" s="8">
-        <v>319950</v>
-      </c>
+      <c r="U49" s="8"/>
       <c r="V49" s="8">
         <v>319950</v>
       </c>
-      <c r="W49" s="8"/>
+      <c r="W49" s="8">
+        <v>319950</v>
+      </c>
       <c r="X49" s="8"/>
       <c r="Y49" s="8"/>
       <c r="Z49" s="8"/>
-      <c r="AA49" s="8">
+      <c r="AA49" s="8"/>
+      <c r="AB49" s="8">
         <v>159975</v>
       </c>
-      <c r="AB49" s="8"/>
       <c r="AC49" s="8"/>
       <c r="AD49" s="8"/>
-      <c r="AE49" s="10">
+      <c r="AE49" s="8"/>
+      <c r="AF49" s="10">
         <v>799875</v>
       </c>
     </row>
-    <row r="50" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B50" s="12">
-        <v>11894263.719999999</v>
+        <v>11606149.915999999</v>
       </c>
       <c r="C50" s="12">
-        <v>806349.07200000004</v>
+        <v>403174.53600000002</v>
       </c>
       <c r="D50" s="12">
-        <v>0</v>
+        <v>403174.53600000002</v>
       </c>
       <c r="E50" s="12">
         <v>0</v>
@@ -2899,60 +2989,63 @@
         <v>0</v>
       </c>
       <c r="O50" s="12">
-        <v>1325887.264</v>
+        <v>728300.9040000001</v>
       </c>
       <c r="P50" s="12">
-        <v>314244.14399999997</v>
+        <v>357586.36000000004</v>
       </c>
       <c r="Q50" s="12">
-        <v>199972.29600000003</v>
+        <v>180000</v>
       </c>
       <c r="R50" s="12">
-        <v>2149163.5279999999</v>
+        <v>1133379.7040000001</v>
       </c>
       <c r="S50" s="12">
-        <v>880851.18000000017</v>
+        <v>1156584.5440000002</v>
       </c>
       <c r="T50" s="12">
-        <v>1527082.98</v>
+        <v>1637417.5379999999</v>
       </c>
       <c r="U50" s="12">
-        <v>2108937.7280000001</v>
+        <v>1973692.524</v>
       </c>
       <c r="V50" s="12">
-        <v>551172.23600000003</v>
+        <v>483789.85600000003</v>
       </c>
       <c r="W50" s="12">
-        <v>166562.6</v>
+        <v>1464107.362</v>
       </c>
       <c r="X50" s="12">
-        <v>797203.13199999998</v>
+        <v>0</v>
       </c>
       <c r="Y50" s="12">
-        <v>569915.91999999993</v>
+        <v>738375.80799999996</v>
       </c>
       <c r="Z50" s="12">
-        <v>244946.64</v>
+        <v>575768.44400000002</v>
       </c>
       <c r="AA50" s="12">
+        <v>118822.8</v>
+      </c>
+      <c r="AB50" s="12">
         <v>159975</v>
-      </c>
-      <c r="AB50" s="12">
-        <v>0</v>
       </c>
       <c r="AC50" s="12">
         <v>0</v>
       </c>
       <c r="AD50" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE50" s="12">
         <v>92000</v>
       </c>
-      <c r="AE50" s="12">
-        <v>11894263.719999999</v>
-      </c>
-    </row>
-    <row r="52" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF50" s="12">
+        <v>11606149.915999999</v>
+      </c>
+    </row>
+    <row r="52" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -2984,302 +3077,16 @@
       <c r="AC52" s="4"/>
       <c r="AD52" s="4"/>
       <c r="AE52" s="4"/>
+      <c r="AF52" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:AE1"/>
-    <mergeCell ref="A2:AE2"/>
-    <mergeCell ref="A52:AE52"/>
-    <mergeCell ref="A4:AE4"/>
-    <mergeCell ref="A28:AE28"/>
+    <mergeCell ref="A1:AF1"/>
+    <mergeCell ref="A2:AF2"/>
+    <mergeCell ref="A52:AF52"/>
+    <mergeCell ref="A4:AF4"/>
+    <mergeCell ref="A28:AF28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7BD3B104-9ADA-4665-A2A5-7653CB6F4F54}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98452712-719C-4C9F-829B-6D7F4742FDF2}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F270FCD-7F77-41D6-9446-9B8558CEA253}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-10 15:36)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Dashboard\.dashboard-repo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/.dashboard-repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{63E5A9AB-A611-4CCA-B02E-2FB82A0F6521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7A8A43A1-F232-45EB-8318-7C8EE3F2AD1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{3A182371-689F-4AB0-9027-60B39D162AFC}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{59F9A59C-4D69-45C6-BF8E-97C95CE32D2C}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C3620D9-DE81-4A50-ACC9-47BD8B542B35}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{009435BF-7FE5-4055-8CAB-0589FE975209}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-10 15:45)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/.dashboard-repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7A8A43A1-F232-45EB-8318-7C8EE3F2AD1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8CC2261-96B3-463B-9FA1-3DB9C2C77326}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{59F9A59C-4D69-45C6-BF8E-97C95CE32D2C}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{E4E4846D-8BF3-4158-8B6E-A4C7AEB9D7C6}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{009435BF-7FE5-4055-8CAB-0589FE975209}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79DA68A4-22F8-45B9-90B0-743686070225}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-10 15:48)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Dashboard/.dashboard-repo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8CC2261-96B3-463B-9FA1-3DB9C2C77326}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{89F0750A-0EBD-4C7D-B781-88AC7C5717F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{E4E4846D-8BF3-4158-8B6E-A4C7AEB9D7C6}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{5250133B-7256-43EC-891D-EC98ECD878E0}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79DA68A4-22F8-45B9-90B0-743686070225}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E7A8DD1-590D-4055-B238-1AE47BCEF52B}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-11 14:19)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{89F0750A-0EBD-4C7D-B781-88AC7C5717F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B866564-0525-4F56-A116-25E3E7D7BF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{5250133B-7256-43EC-891D-EC98ECD878E0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{12261E18-3F7B-4358-9B41-D37D82B3ADD8}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (20 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-10</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-11</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E7A8DD1-590D-4055-B238-1AE47BCEF52B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8766A8A0-92BB-49F7-93D8-12681C7FB49C}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-11 14:46)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B866564-0525-4F56-A116-25E3E7D7BF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{722FFE7C-4074-4135-AECA-DF167AE6FAED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{12261E18-3F7B-4358-9B41-D37D82B3ADD8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{11345C40-2092-40CC-93D0-0BA3AC63CA8E}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8766A8A0-92BB-49F7-93D8-12681C7FB49C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F74DCAD8-5B67-4B04-83B4-C3F40D30B369}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-11 16:17)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{722FFE7C-4074-4135-AECA-DF167AE6FAED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{39ED99AB-2B54-45D5-8063-8BD1064DCF53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{11345C40-2092-40CC-93D0-0BA3AC63CA8E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{37A3F414-C974-4B2C-8BB7-B56E231F6693}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F74DCAD8-5B67-4B04-83B4-C3F40D30B369}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EE643F4-FD77-4D76-B0FB-E0C9C307A65C}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 10:43)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{39ED99AB-2B54-45D5-8063-8BD1064DCF53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8BD8572A-0BCA-4ED0-9BAD-C944C3D53EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{37A3F414-C974-4B2C-8BB7-B56E231F6693}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{133E4B20-F238-4514-A849-99FEA01558CD}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (20 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-11</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-19</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EE643F4-FD77-4D76-B0FB-E0C9C307A65C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7F662D2-BFFC-4562-9B2E-D9A44A6182C8}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1676,7 +1676,7 @@
         <v>52</v>
       </c>
       <c r="B23" s="10">
-        <v>215000</v>
+        <v>218000</v>
       </c>
       <c r="C23" s="8"/>
       <c r="D23" s="8"/>
@@ -1697,11 +1697,11 @@
       <c r="S23" s="8"/>
       <c r="T23" s="8"/>
       <c r="U23" s="8">
-        <v>64500</v>
+        <v>65400</v>
       </c>
       <c r="V23" s="8"/>
       <c r="W23" s="8">
-        <v>107500</v>
+        <v>109000</v>
       </c>
       <c r="X23" s="8"/>
       <c r="Y23" s="8"/>
@@ -1710,11 +1710,11 @@
       <c r="AB23" s="8"/>
       <c r="AC23" s="8"/>
       <c r="AD23" s="8">
-        <v>43000</v>
+        <v>43600</v>
       </c>
       <c r="AE23" s="8"/>
       <c r="AF23" s="10">
-        <v>215000</v>
+        <v>218000</v>
       </c>
     </row>
     <row r="24" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
@@ -1810,7 +1810,7 @@
         <v>55</v>
       </c>
       <c r="B26" s="12">
-        <v>4294064.93</v>
+        <v>4297064.93</v>
       </c>
       <c r="C26" s="12">
         <v>139012.5</v>
@@ -1867,13 +1867,13 @@
         <v>739675.321</v>
       </c>
       <c r="U26" s="12">
-        <v>551333.80000000005</v>
+        <v>552233.80000000005</v>
       </c>
       <c r="V26" s="12">
         <v>264840.8</v>
       </c>
       <c r="W26" s="12">
-        <v>633127.19999999995</v>
+        <v>634627.19999999995</v>
       </c>
       <c r="X26" s="12">
         <v>24000</v>
@@ -1894,13 +1894,13 @@
         <v>0</v>
       </c>
       <c r="AD26" s="12">
-        <v>43000</v>
+        <v>43600</v>
       </c>
       <c r="AE26" s="12">
         <v>0</v>
       </c>
       <c r="AF26" s="12">
-        <v>4294064.93</v>
+        <v>4297064.93</v>
       </c>
     </row>
     <row r="28" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 11:58)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8BD8572A-0BCA-4ED0-9BAD-C944C3D53EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8AC90B2-582F-46BD-A5A8-133CA387F650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{133E4B20-F238-4514-A849-99FEA01558CD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EA9C86E0-4C41-4DBF-8158-ACB5CB419B7A}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7F662D2-BFFC-4562-9B2E-D9A44A6182C8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D54EBAA-6B67-4182-9206-310BC24EA404}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 13:17)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3089,4 +3089,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9885388A-B769-437A-9566-208F7848350B}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EDCD3665-3368-46BF-98A0-F486F86D7C8C}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE005799-E01F-4258-95EA-F97D5F51B4D5}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 15:02)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8AC90B2-582F-46BD-A5A8-133CA387F650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{525B5CB0-EBE8-408C-96E8-D84402E19EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EA9C86E0-4C41-4DBF-8158-ACB5CB419B7A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9FC3AFA8-FC69-46FC-888E-A26E4167C67C}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D54EBAA-6B67-4182-9206-310BC24EA404}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECB90456-C045-4FB4-97D3-030D0D3210F8}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3089,291 +3089,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9885388A-B769-437A-9566-208F7848350B}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EDCD3665-3368-46BF-98A0-F486F86D7C8C}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE005799-E01F-4258-95EA-F97D5F51B4D5}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 15:11)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3089,4 +3089,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7154FAE0-DD75-4CCE-AF39-B4EF54011774}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FE27EFD-8FD6-482F-B626-ACD61B360817}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5C637C7-942F-44A8-9D2F-CBC9AA98C9E4}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 15:40)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{525B5CB0-EBE8-408C-96E8-D84402E19EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{004D163F-4DAC-4F61-8EFB-7CB7291F639D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9FC3AFA8-FC69-46FC-888E-A26E4167C67C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{384D2250-13E7-437F-A1A7-A8A33CF6C3D5}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECB90456-C045-4FB4-97D3-030D0D3210F8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E21F58AB-E135-43AA-940D-F276E50B337C}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2042,7 +2042,7 @@
         <v>35</v>
       </c>
       <c r="B30" s="10">
-        <v>326786.36</v>
+        <v>313714.9056</v>
       </c>
       <c r="C30" s="8"/>
       <c r="D30" s="8"/>
@@ -2064,7 +2064,7 @@
       <c r="R30" s="8"/>
       <c r="S30" s="8"/>
       <c r="T30" s="8">
-        <v>130714.54399999999</v>
+        <v>117643.08959999999</v>
       </c>
       <c r="U30" s="8">
         <v>65357.271999999997</v>
@@ -2080,7 +2080,7 @@
       <c r="AD30" s="8"/>
       <c r="AE30" s="8"/>
       <c r="AF30" s="10">
-        <v>326786.36</v>
+        <v>313714.9056</v>
       </c>
     </row>
     <row r="31" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
@@ -2950,7 +2950,7 @@
         <v>55</v>
       </c>
       <c r="B50" s="12">
-        <v>11606149.915999999</v>
+        <v>11593078.4616</v>
       </c>
       <c r="C50" s="12">
         <v>403174.53600000002</v>
@@ -3004,7 +3004,7 @@
         <v>1156584.5440000002</v>
       </c>
       <c r="T50" s="12">
-        <v>1637417.5379999999</v>
+        <v>1624346.0836</v>
       </c>
       <c r="U50" s="12">
         <v>1973692.524</v>
@@ -3040,7 +3040,7 @@
         <v>92000</v>
       </c>
       <c r="AF50" s="12">
-        <v>11606149.915999999</v>
+        <v>11593078.4616</v>
       </c>
     </row>
     <row r="52" spans="1:32" x14ac:dyDescent="0.2">
@@ -3089,291 +3089,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7154FAE0-DD75-4CCE-AF39-B4EF54011774}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FE27EFD-8FD6-482F-B626-ACD61B360817}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5C637C7-942F-44A8-9D2F-CBC9AA98C9E4}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 15:47)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{004D163F-4DAC-4F61-8EFB-7CB7291F639D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{07D3D9FE-ED68-41CB-B02D-1D148F8EAC28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{384D2250-13E7-437F-A1A7-A8A33CF6C3D5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{600F2457-756F-459F-9FD7-A1EA956F7312}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E21F58AB-E135-43AA-940D-F276E50B337C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8D1A248-2ED8-4E62-87AB-E69FFD11FC24}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 16:08)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{07D3D9FE-ED68-41CB-B02D-1D148F8EAC28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C157F54-0B23-4BB6-B949-6F1318938A15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{600F2457-756F-459F-9FD7-A1EA956F7312}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D0722C64-791C-48BA-A177-3EE093663B81}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8D1A248-2ED8-4E62-87AB-E69FFD11FC24}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{802244DB-D362-495C-90AA-ED4444B9B7C9}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 16:29)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C157F54-0B23-4BB6-B949-6F1318938A15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4BA75A9-0DBD-4044-BE3F-8A731193BD5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D0722C64-791C-48BA-A177-3EE093663B81}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EBE7008A-66D7-4F96-B1D3-F7152AD3E4EC}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{802244DB-D362-495C-90AA-ED4444B9B7C9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7989D3C-D3F5-41EA-888B-C6C433BA11EC}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1722,7 +1722,7 @@
         <v>53</v>
       </c>
       <c r="B24" s="10">
-        <v>116000</v>
+        <v>58000</v>
       </c>
       <c r="C24" s="8"/>
       <c r="D24" s="8"/>
@@ -1743,7 +1743,7 @@
       <c r="S24" s="8"/>
       <c r="T24" s="8"/>
       <c r="U24" s="8">
-        <v>116000</v>
+        <v>58000</v>
       </c>
       <c r="V24" s="8"/>
       <c r="W24" s="8"/>
@@ -1756,7 +1756,7 @@
       <c r="AD24" s="8"/>
       <c r="AE24" s="8"/>
       <c r="AF24" s="10">
-        <v>116000</v>
+        <v>58000</v>
       </c>
     </row>
     <row r="25" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
@@ -1810,7 +1810,7 @@
         <v>55</v>
       </c>
       <c r="B26" s="12">
-        <v>4297064.93</v>
+        <v>4239064.93</v>
       </c>
       <c r="C26" s="12">
         <v>139012.5</v>
@@ -1867,7 +1867,7 @@
         <v>739675.321</v>
       </c>
       <c r="U26" s="12">
-        <v>552233.80000000005</v>
+        <v>494233.8</v>
       </c>
       <c r="V26" s="12">
         <v>264840.8</v>
@@ -1900,7 +1900,7 @@
         <v>0</v>
       </c>
       <c r="AF26" s="12">
-        <v>4297064.93</v>
+        <v>4239064.93</v>
       </c>
     </row>
     <row r="28" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 16:56)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4BA75A9-0DBD-4044-BE3F-8A731193BD5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D73E8F29-59D2-4261-BE1C-A0969FF21135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EBE7008A-66D7-4F96-B1D3-F7152AD3E4EC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2A6D8F2B-5260-46C8-8709-8AC6D1D823D9}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7989D3C-D3F5-41EA-888B-C6C433BA11EC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{145E89C1-0D68-458D-8A7E-EE11654687F2}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2042,7 +2042,7 @@
         <v>35</v>
       </c>
       <c r="B30" s="10">
-        <v>313714.9056</v>
+        <v>326786.36</v>
       </c>
       <c r="C30" s="8"/>
       <c r="D30" s="8"/>
@@ -2064,7 +2064,7 @@
       <c r="R30" s="8"/>
       <c r="S30" s="8"/>
       <c r="T30" s="8">
-        <v>117643.08959999999</v>
+        <v>130714.54399999999</v>
       </c>
       <c r="U30" s="8">
         <v>65357.271999999997</v>
@@ -2080,7 +2080,7 @@
       <c r="AD30" s="8"/>
       <c r="AE30" s="8"/>
       <c r="AF30" s="10">
-        <v>313714.9056</v>
+        <v>326786.36</v>
       </c>
     </row>
     <row r="31" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
@@ -2134,7 +2134,7 @@
         <v>37</v>
       </c>
       <c r="B32" s="10">
-        <v>537273.12000000011</v>
+        <v>576317.9</v>
       </c>
       <c r="C32" s="8"/>
       <c r="D32" s="8"/>
@@ -2158,7 +2158,7 @@
       <c r="R32" s="8"/>
       <c r="S32" s="8"/>
       <c r="T32" s="8">
-        <v>76218.8</v>
+        <v>115263.58</v>
       </c>
       <c r="U32" s="8"/>
       <c r="V32" s="8"/>
@@ -2172,7 +2172,7 @@
       <c r="AD32" s="8"/>
       <c r="AE32" s="8"/>
       <c r="AF32" s="10">
-        <v>537273.12000000011</v>
+        <v>576317.9</v>
       </c>
     </row>
     <row r="33" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
@@ -2180,7 +2180,7 @@
         <v>38</v>
       </c>
       <c r="B33" s="10">
-        <v>387553.29600000003</v>
+        <v>322961.08</v>
       </c>
       <c r="C33" s="8"/>
       <c r="D33" s="8"/>
@@ -2201,7 +2201,7 @@
         <v>129184.43200000002</v>
       </c>
       <c r="S33" s="8">
-        <v>258368.86400000003</v>
+        <v>193776.64800000002</v>
       </c>
       <c r="T33" s="8"/>
       <c r="U33" s="8"/>
@@ -2216,7 +2216,7 @@
       <c r="AD33" s="8"/>
       <c r="AE33" s="8"/>
       <c r="AF33" s="10">
-        <v>387553.29600000003</v>
+        <v>322961.08</v>
       </c>
     </row>
     <row r="34" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
@@ -2404,7 +2404,7 @@
         <v>43</v>
       </c>
       <c r="B38" s="10">
-        <v>359813.07999999996</v>
+        <v>327102.8</v>
       </c>
       <c r="C38" s="8"/>
       <c r="D38" s="8"/>
@@ -2434,7 +2434,7 @@
       <c r="X38" s="8"/>
       <c r="Y38" s="8"/>
       <c r="Z38" s="8">
-        <v>98130.84</v>
+        <v>65420.56</v>
       </c>
       <c r="AA38" s="8"/>
       <c r="AB38" s="8"/>
@@ -2442,7 +2442,7 @@
       <c r="AD38" s="8"/>
       <c r="AE38" s="8"/>
       <c r="AF38" s="10">
-        <v>359813.07999999996</v>
+        <v>327102.8</v>
       </c>
     </row>
     <row r="39" spans="1:32" ht="69" x14ac:dyDescent="0.25">
@@ -2496,7 +2496,7 @@
         <v>45</v>
       </c>
       <c r="B40" s="10">
-        <v>112000</v>
+        <v>80000</v>
       </c>
       <c r="C40" s="8"/>
       <c r="D40" s="8"/>
@@ -2517,7 +2517,7 @@
         <v>32000</v>
       </c>
       <c r="S40" s="8">
-        <v>80000</v>
+        <v>48000</v>
       </c>
       <c r="T40" s="8"/>
       <c r="U40" s="8"/>
@@ -2532,7 +2532,7 @@
       <c r="AD40" s="8"/>
       <c r="AE40" s="8"/>
       <c r="AF40" s="10">
-        <v>112000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="41" spans="1:32" ht="69" x14ac:dyDescent="0.25">
@@ -2950,7 +2950,7 @@
         <v>55</v>
       </c>
       <c r="B50" s="12">
-        <v>11593078.4616</v>
+        <v>11515892.199999999</v>
       </c>
       <c r="C50" s="12">
         <v>403174.53600000002</v>
@@ -3001,10 +3001,10 @@
         <v>1133379.7040000001</v>
       </c>
       <c r="S50" s="12">
-        <v>1156584.5440000002</v>
+        <v>1059992.3280000002</v>
       </c>
       <c r="T50" s="12">
-        <v>1624346.0836</v>
+        <v>1676462.318</v>
       </c>
       <c r="U50" s="12">
         <v>1973692.524</v>
@@ -3022,7 +3022,7 @@
         <v>738375.80799999996</v>
       </c>
       <c r="Z50" s="12">
-        <v>575768.44400000002</v>
+        <v>543058.16400000011</v>
       </c>
       <c r="AA50" s="12">
         <v>118822.8</v>
@@ -3040,7 +3040,7 @@
         <v>92000</v>
       </c>
       <c r="AF50" s="12">
-        <v>11593078.4616</v>
+        <v>11515892.199999999</v>
       </c>
     </row>
     <row r="52" spans="1:32" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 17:18)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D73E8F29-59D2-4261-BE1C-A0969FF21135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA8E7F21-9693-4168-A89D-FFB63BFBA022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2A6D8F2B-5260-46C8-8709-8AC6D1D823D9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FCE46536-3DF7-4A7F-943B-6AB69D172CCF}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{145E89C1-0D68-458D-8A7E-EE11654687F2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD92B91B-8EF7-4DE0-9C5E-7FD344987B3C}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 17:25)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA8E7F21-9693-4168-A89D-FFB63BFBA022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A2281275-03E2-4B2C-BDD2-BA8E0ABEEBC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FCE46536-3DF7-4A7F-943B-6AB69D172CCF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A084BCD2-64B5-44A9-A181-63204CA7FE22}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD92B91B-8EF7-4DE0-9C5E-7FD344987B3C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB736235-2DDD-47CF-9A97-7FD0EF4A886F}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -916,7 +916,7 @@
         <v>35</v>
       </c>
       <c r="B6" s="10">
-        <v>117000</v>
+        <v>130000</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
@@ -939,7 +939,7 @@
       </c>
       <c r="R6" s="8"/>
       <c r="S6" s="8">
-        <v>13000</v>
+        <v>26000</v>
       </c>
       <c r="T6" s="8"/>
       <c r="U6" s="8"/>
@@ -954,7 +954,7 @@
       <c r="AD6" s="8"/>
       <c r="AE6" s="8"/>
       <c r="AF6" s="10">
-        <v>117000</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="7" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
@@ -1810,7 +1810,7 @@
         <v>55</v>
       </c>
       <c r="B26" s="12">
-        <v>4239064.93</v>
+        <v>4252064.93</v>
       </c>
       <c r="C26" s="12">
         <v>139012.5</v>
@@ -1861,7 +1861,7 @@
         <v>272600</v>
       </c>
       <c r="S26" s="12">
-        <v>324403.70900000003</v>
+        <v>337403.70900000003</v>
       </c>
       <c r="T26" s="12">
         <v>739675.321</v>
@@ -1900,7 +1900,7 @@
         <v>0</v>
       </c>
       <c r="AF26" s="12">
-        <v>4239064.93</v>
+        <v>4252064.93</v>
       </c>
     </row>
     <row r="28" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 17:31)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A2281275-03E2-4B2C-BDD2-BA8E0ABEEBC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1DFFFE1B-A3E5-4B37-912B-7EABCCE55373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A084BCD2-64B5-44A9-A181-63204CA7FE22}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4F69D4C6-7F1B-4FD2-8612-43C843175D0E}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB736235-2DDD-47CF-9A97-7FD0EF4A886F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1FD67A5-CB78-437C-A5CA-9B74D598794E}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 17:35)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1DFFFE1B-A3E5-4B37-912B-7EABCCE55373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7FFC8F2D-84F8-4577-919A-7E0EBE049D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4F69D4C6-7F1B-4FD2-8612-43C843175D0E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9EADEDD1-F42B-42BD-A54F-FDD682EA4C29}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1FD67A5-CB78-437C-A5CA-9B74D598794E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7C58372-4FBF-4F8E-9BC1-CE8F15D61F47}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 17:51)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7FFC8F2D-84F8-4577-919A-7E0EBE049D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{91718976-3E12-4F78-9CBD-27CA987531C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9EADEDD1-F42B-42BD-A54F-FDD682EA4C29}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{33F00C75-0455-4294-9A4B-D7A3E6548A65}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7C58372-4FBF-4F8E-9BC1-CE8F15D61F47}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96430325-1C18-4B7E-BC04-3802AA2F03D5}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 18:00)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{91718976-3E12-4F78-9CBD-27CA987531C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2254811C-CC9E-4B64-890D-21B2D2EFF920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{33F00C75-0455-4294-9A4B-D7A3E6548A65}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EEA53C07-79A6-4C5E-8ACA-B6EEA73A1EB8}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96430325-1C18-4B7E-BC04-3802AA2F03D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{792798D8-F2ED-4647-80E3-56931337233A}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -983,13 +983,13 @@
       <c r="S7" s="8"/>
       <c r="T7" s="8"/>
       <c r="U7" s="8">
-        <v>41833.799999999996</v>
+        <v>41834</v>
       </c>
       <c r="V7" s="8">
         <v>69723</v>
       </c>
       <c r="W7" s="8">
-        <v>27889.200000000001</v>
+        <v>27889</v>
       </c>
       <c r="X7" s="8"/>
       <c r="Y7" s="8"/>
@@ -1228,7 +1228,7 @@
         <v>42</v>
       </c>
       <c r="B13" s="10">
-        <v>233247.9</v>
+        <v>233248</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
@@ -1253,10 +1253,10 @@
       <c r="W13" s="8"/>
       <c r="X13" s="8"/>
       <c r="Y13" s="8">
-        <v>69974.37</v>
+        <v>69974</v>
       </c>
       <c r="Z13" s="8">
-        <v>163273.53</v>
+        <v>163274</v>
       </c>
       <c r="AA13" s="8"/>
       <c r="AB13" s="8"/>
@@ -1264,7 +1264,7 @@
       <c r="AD13" s="8"/>
       <c r="AE13" s="8"/>
       <c r="AF13" s="10">
-        <v>233247.9</v>
+        <v>233248</v>
       </c>
     </row>
     <row r="14" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
@@ -1318,7 +1318,7 @@
         <v>44</v>
       </c>
       <c r="B15" s="10">
-        <v>656679.03</v>
+        <v>656680</v>
       </c>
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
@@ -1337,10 +1337,10 @@
       <c r="Q15" s="8"/>
       <c r="R15" s="8"/>
       <c r="S15" s="8">
-        <v>197003.709</v>
+        <v>197004</v>
       </c>
       <c r="T15" s="8">
-        <v>459675.321</v>
+        <v>459676</v>
       </c>
       <c r="U15" s="8"/>
       <c r="V15" s="8"/>
@@ -1354,7 +1354,7 @@
       <c r="AD15" s="8"/>
       <c r="AE15" s="8"/>
       <c r="AF15" s="10">
-        <v>656679.03</v>
+        <v>656680</v>
       </c>
     </row>
     <row r="16" spans="1:32" ht="69" x14ac:dyDescent="0.25">
@@ -1450,7 +1450,7 @@
         <v>47</v>
       </c>
       <c r="B18" s="10">
-        <v>234861</v>
+        <v>234860</v>
       </c>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -1465,11 +1465,11 @@
       <c r="M18" s="8"/>
       <c r="N18" s="8"/>
       <c r="O18" s="8">
-        <v>70458.3</v>
+        <v>70458</v>
       </c>
       <c r="P18" s="8"/>
       <c r="Q18" s="8">
-        <v>164402.70000000001</v>
+        <v>164402</v>
       </c>
       <c r="R18" s="8"/>
       <c r="S18" s="8"/>
@@ -1486,7 +1486,7 @@
       <c r="AD18" s="8"/>
       <c r="AE18" s="8"/>
       <c r="AF18" s="10">
-        <v>234861</v>
+        <v>234860</v>
       </c>
     </row>
     <row r="19" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
@@ -1587,7 +1587,7 @@
         <v>239148</v>
       </c>
       <c r="C21" s="8">
-        <v>71744.399999999994</v>
+        <v>71744</v>
       </c>
       <c r="D21" s="8">
         <v>119574</v>
@@ -1610,7 +1610,7 @@
       <c r="T21" s="8"/>
       <c r="U21" s="8"/>
       <c r="V21" s="8">
-        <v>47829.600000000006</v>
+        <v>47830</v>
       </c>
       <c r="W21" s="8"/>
       <c r="X21" s="8"/>
@@ -1630,13 +1630,13 @@
         <v>51</v>
       </c>
       <c r="B22" s="10">
-        <v>224226.99999999997</v>
+        <v>224227</v>
       </c>
       <c r="C22" s="8">
-        <v>67268.099999999991</v>
+        <v>67268</v>
       </c>
       <c r="D22" s="8">
-        <v>112113.5</v>
+        <v>112114</v>
       </c>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
@@ -1656,7 +1656,7 @@
       <c r="T22" s="8"/>
       <c r="U22" s="8"/>
       <c r="V22" s="8">
-        <v>44845.4</v>
+        <v>44845</v>
       </c>
       <c r="W22" s="8"/>
       <c r="X22" s="8"/>
@@ -1668,7 +1668,7 @@
       <c r="AD22" s="8"/>
       <c r="AE22" s="8"/>
       <c r="AF22" s="10">
-        <v>224226.99999999997</v>
+        <v>224227</v>
       </c>
     </row>
     <row r="23" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
@@ -1786,7 +1786,7 @@
       <c r="T25" s="8"/>
       <c r="U25" s="8"/>
       <c r="V25" s="8">
-        <v>102442.8</v>
+        <v>102443</v>
       </c>
       <c r="W25" s="8">
         <v>170738</v>
@@ -1795,7 +1795,7 @@
       <c r="Y25" s="8"/>
       <c r="Z25" s="8"/>
       <c r="AA25" s="8">
-        <v>68295.199999999997</v>
+        <v>68295</v>
       </c>
       <c r="AB25" s="8"/>
       <c r="AC25" s="8"/>
@@ -1810,13 +1810,13 @@
         <v>55</v>
       </c>
       <c r="B26" s="12">
-        <v>4252064.93</v>
+        <v>4252065</v>
       </c>
       <c r="C26" s="12">
-        <v>139012.5</v>
+        <v>139012</v>
       </c>
       <c r="D26" s="12">
-        <v>231687.5</v>
+        <v>231688</v>
       </c>
       <c r="E26" s="12">
         <v>0</v>
@@ -1849,43 +1849,43 @@
         <v>0</v>
       </c>
       <c r="O26" s="12">
-        <v>229452.3</v>
+        <v>229452</v>
       </c>
       <c r="P26" s="12">
         <v>223986</v>
       </c>
       <c r="Q26" s="12">
-        <v>229402.7</v>
+        <v>229402</v>
       </c>
       <c r="R26" s="12">
         <v>272600</v>
       </c>
       <c r="S26" s="12">
-        <v>337403.70900000003</v>
+        <v>337404</v>
       </c>
       <c r="T26" s="12">
-        <v>739675.321</v>
+        <v>739676</v>
       </c>
       <c r="U26" s="12">
-        <v>494233.8</v>
+        <v>494234</v>
       </c>
       <c r="V26" s="12">
-        <v>264840.8</v>
+        <v>264841</v>
       </c>
       <c r="W26" s="12">
-        <v>634627.19999999995</v>
+        <v>634627</v>
       </c>
       <c r="X26" s="12">
         <v>24000</v>
       </c>
       <c r="Y26" s="12">
-        <v>155974.37</v>
+        <v>155974</v>
       </c>
       <c r="Z26" s="12">
-        <v>163273.53</v>
+        <v>163274</v>
       </c>
       <c r="AA26" s="12">
-        <v>68295.199999999997</v>
+        <v>68295</v>
       </c>
       <c r="AB26" s="12">
         <v>0</v>
@@ -1900,7 +1900,7 @@
         <v>0</v>
       </c>
       <c r="AF26" s="12">
-        <v>4252064.93</v>
+        <v>4252065</v>
       </c>
     </row>
     <row r="28" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2042,7 +2042,7 @@
         <v>35</v>
       </c>
       <c r="B30" s="10">
-        <v>326786.36</v>
+        <v>326787</v>
       </c>
       <c r="C30" s="8"/>
       <c r="D30" s="8"/>
@@ -2057,17 +2057,17 @@
       <c r="M30" s="8"/>
       <c r="N30" s="8"/>
       <c r="O30" s="8">
-        <v>130714.54399999999</v>
+        <v>130715</v>
       </c>
       <c r="P30" s="8"/>
       <c r="Q30" s="8"/>
       <c r="R30" s="8"/>
       <c r="S30" s="8"/>
       <c r="T30" s="8">
-        <v>130714.54399999999</v>
+        <v>130715</v>
       </c>
       <c r="U30" s="8">
-        <v>65357.271999999997</v>
+        <v>65357</v>
       </c>
       <c r="V30" s="8"/>
       <c r="W30" s="8"/>
@@ -2080,7 +2080,7 @@
       <c r="AD30" s="8"/>
       <c r="AE30" s="8"/>
       <c r="AF30" s="10">
-        <v>326786.36</v>
+        <v>326787</v>
       </c>
     </row>
     <row r="31" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
@@ -2088,7 +2088,7 @@
         <v>36</v>
       </c>
       <c r="B31" s="10">
-        <v>409599.64000000007</v>
+        <v>409600</v>
       </c>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
@@ -2109,15 +2109,15 @@
       <c r="S31" s="8"/>
       <c r="T31" s="8"/>
       <c r="U31" s="8">
-        <v>163839.85600000003</v>
+        <v>163840</v>
       </c>
       <c r="V31" s="8">
-        <v>163839.85600000003</v>
+        <v>163840</v>
       </c>
       <c r="W31" s="8"/>
       <c r="X31" s="8"/>
       <c r="Y31" s="8">
-        <v>81919.928000000014</v>
+        <v>81920</v>
       </c>
       <c r="Z31" s="8"/>
       <c r="AA31" s="8"/>
@@ -2126,7 +2126,7 @@
       <c r="AD31" s="8"/>
       <c r="AE31" s="8"/>
       <c r="AF31" s="10">
-        <v>409599.64000000007</v>
+        <v>409600</v>
       </c>
     </row>
     <row r="32" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
@@ -2134,7 +2134,7 @@
         <v>37</v>
       </c>
       <c r="B32" s="10">
-        <v>576317.9</v>
+        <v>576318</v>
       </c>
       <c r="C32" s="8"/>
       <c r="D32" s="8"/>
@@ -2149,16 +2149,16 @@
       <c r="M32" s="8"/>
       <c r="N32" s="8"/>
       <c r="O32" s="8">
-        <v>230527.16000000003</v>
+        <v>230527</v>
       </c>
       <c r="P32" s="8">
-        <v>230527.16000000003</v>
+        <v>230527</v>
       </c>
       <c r="Q32" s="8"/>
       <c r="R32" s="8"/>
       <c r="S32" s="8"/>
       <c r="T32" s="8">
-        <v>115263.58</v>
+        <v>115264</v>
       </c>
       <c r="U32" s="8"/>
       <c r="V32" s="8"/>
@@ -2172,7 +2172,7 @@
       <c r="AD32" s="8"/>
       <c r="AE32" s="8"/>
       <c r="AF32" s="10">
-        <v>576317.9</v>
+        <v>576318</v>
       </c>
     </row>
     <row r="33" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
@@ -2180,7 +2180,7 @@
         <v>38</v>
       </c>
       <c r="B33" s="10">
-        <v>322961.08</v>
+        <v>322960</v>
       </c>
       <c r="C33" s="8"/>
       <c r="D33" s="8"/>
@@ -2198,10 +2198,10 @@
       <c r="P33" s="8"/>
       <c r="Q33" s="8"/>
       <c r="R33" s="8">
-        <v>129184.43200000002</v>
+        <v>129184</v>
       </c>
       <c r="S33" s="8">
-        <v>193776.64800000002</v>
+        <v>193776</v>
       </c>
       <c r="T33" s="8"/>
       <c r="U33" s="8"/>
@@ -2216,7 +2216,7 @@
       <c r="AD33" s="8"/>
       <c r="AE33" s="8"/>
       <c r="AF33" s="10">
-        <v>322961.08</v>
+        <v>322960</v>
       </c>
     </row>
     <row r="34" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
@@ -2224,7 +2224,7 @@
         <v>39</v>
       </c>
       <c r="B34" s="10">
-        <v>252247.67999999999</v>
+        <v>252248</v>
       </c>
       <c r="C34" s="8"/>
       <c r="D34" s="8"/>
@@ -2249,7 +2249,7 @@
       <c r="W34" s="8"/>
       <c r="X34" s="8"/>
       <c r="Y34" s="8">
-        <v>252247.67999999999</v>
+        <v>252248</v>
       </c>
       <c r="Z34" s="8"/>
       <c r="AA34" s="8"/>
@@ -2258,7 +2258,7 @@
       <c r="AD34" s="8"/>
       <c r="AE34" s="8"/>
       <c r="AF34" s="10">
-        <v>252247.67999999999</v>
+        <v>252248</v>
       </c>
     </row>
     <row r="35" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
@@ -2266,7 +2266,7 @@
         <v>40</v>
       </c>
       <c r="B35" s="10">
-        <v>338450.20000000007</v>
+        <v>338450</v>
       </c>
       <c r="C35" s="8"/>
       <c r="D35" s="8"/>
@@ -2284,13 +2284,13 @@
       <c r="P35" s="8"/>
       <c r="Q35" s="8"/>
       <c r="R35" s="8">
-        <v>135380.08000000002</v>
+        <v>135380</v>
       </c>
       <c r="S35" s="8">
-        <v>135380.08000000002</v>
+        <v>135380</v>
       </c>
       <c r="T35" s="8">
-        <v>67690.040000000008</v>
+        <v>67690</v>
       </c>
       <c r="U35" s="8"/>
       <c r="V35" s="8"/>
@@ -2304,7 +2304,7 @@
       <c r="AD35" s="8"/>
       <c r="AE35" s="8"/>
       <c r="AF35" s="10">
-        <v>338450.20000000007</v>
+        <v>338450</v>
       </c>
     </row>
     <row r="36" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
@@ -2312,7 +2312,7 @@
         <v>41</v>
       </c>
       <c r="B36" s="10">
-        <v>1156111.18</v>
+        <v>1156110</v>
       </c>
       <c r="C36" s="8"/>
       <c r="D36" s="8"/>
@@ -2330,16 +2330,16 @@
       <c r="P36" s="8"/>
       <c r="Q36" s="8"/>
       <c r="R36" s="8">
-        <v>462444.47200000001</v>
+        <v>462444</v>
       </c>
       <c r="S36" s="8"/>
       <c r="T36" s="8">
-        <v>346833.35399999999</v>
+        <v>346833</v>
       </c>
       <c r="U36" s="8"/>
       <c r="V36" s="8"/>
       <c r="W36" s="8">
-        <v>346833.35399999999</v>
+        <v>346833</v>
       </c>
       <c r="X36" s="8"/>
       <c r="Y36" s="8"/>
@@ -2350,7 +2350,7 @@
       <c r="AD36" s="8"/>
       <c r="AE36" s="8"/>
       <c r="AF36" s="10">
-        <v>1156111.18</v>
+        <v>1156110</v>
       </c>
     </row>
     <row r="37" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
@@ -2358,7 +2358,7 @@
         <v>42</v>
       </c>
       <c r="B37" s="10">
-        <v>594114</v>
+        <v>594115</v>
       </c>
       <c r="C37" s="8"/>
       <c r="D37" s="8"/>
@@ -2383,20 +2383,20 @@
       <c r="W37" s="8"/>
       <c r="X37" s="8"/>
       <c r="Y37" s="8">
-        <v>237645.6</v>
+        <v>237646</v>
       </c>
       <c r="Z37" s="8">
-        <v>237645.6</v>
+        <v>237646</v>
       </c>
       <c r="AA37" s="8">
-        <v>118822.8</v>
+        <v>118823</v>
       </c>
       <c r="AB37" s="8"/>
       <c r="AC37" s="8"/>
       <c r="AD37" s="8"/>
       <c r="AE37" s="8"/>
       <c r="AF37" s="10">
-        <v>594114</v>
+        <v>594115</v>
       </c>
     </row>
     <row r="38" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
@@ -2404,7 +2404,7 @@
         <v>43</v>
       </c>
       <c r="B38" s="10">
-        <v>327102.8</v>
+        <v>327103</v>
       </c>
       <c r="C38" s="8"/>
       <c r="D38" s="8"/>
@@ -2422,19 +2422,19 @@
       <c r="P38" s="8"/>
       <c r="Q38" s="8"/>
       <c r="R38" s="8">
-        <v>130841.12</v>
+        <v>130841</v>
       </c>
       <c r="S38" s="8"/>
       <c r="T38" s="8"/>
       <c r="U38" s="8">
-        <v>130841.12</v>
+        <v>130841</v>
       </c>
       <c r="V38" s="8"/>
       <c r="W38" s="8"/>
       <c r="X38" s="8"/>
       <c r="Y38" s="8"/>
       <c r="Z38" s="8">
-        <v>65420.56</v>
+        <v>65421</v>
       </c>
       <c r="AA38" s="8"/>
       <c r="AB38" s="8"/>
@@ -2442,7 +2442,7 @@
       <c r="AD38" s="8"/>
       <c r="AE38" s="8"/>
       <c r="AF38" s="10">
-        <v>327102.8</v>
+        <v>327103</v>
       </c>
     </row>
     <row r="39" spans="1:32" ht="69" x14ac:dyDescent="0.25">
@@ -2450,7 +2450,7 @@
         <v>44</v>
       </c>
       <c r="B39" s="10">
-        <v>1707089.0000000002</v>
+        <v>1707090</v>
       </c>
       <c r="C39" s="8"/>
       <c r="D39" s="8"/>
@@ -2469,13 +2469,13 @@
       <c r="Q39" s="8"/>
       <c r="R39" s="8"/>
       <c r="S39" s="8">
-        <v>682835.60000000009</v>
+        <v>682836</v>
       </c>
       <c r="T39" s="8">
-        <v>682835.60000000009</v>
+        <v>682836</v>
       </c>
       <c r="U39" s="8">
-        <v>341417.80000000005</v>
+        <v>341418</v>
       </c>
       <c r="V39" s="8"/>
       <c r="W39" s="8"/>
@@ -2488,7 +2488,7 @@
       <c r="AD39" s="8"/>
       <c r="AE39" s="8"/>
       <c r="AF39" s="10">
-        <v>1707089.0000000002</v>
+        <v>1707090</v>
       </c>
     </row>
     <row r="40" spans="1:32" ht="69" x14ac:dyDescent="0.25">
@@ -2540,7 +2540,7 @@
         <v>46</v>
       </c>
       <c r="B41" s="10">
-        <v>1199960.02</v>
+        <v>1199960</v>
       </c>
       <c r="C41" s="8"/>
       <c r="D41" s="8"/>
@@ -2561,16 +2561,16 @@
       <c r="S41" s="8"/>
       <c r="T41" s="8"/>
       <c r="U41" s="8">
-        <v>479984.00800000003</v>
+        <v>479984</v>
       </c>
       <c r="V41" s="8"/>
       <c r="W41" s="8">
-        <v>479984.00800000003</v>
+        <v>479984</v>
       </c>
       <c r="X41" s="8"/>
       <c r="Y41" s="8"/>
       <c r="Z41" s="8">
-        <v>239992.00400000002</v>
+        <v>239992</v>
       </c>
       <c r="AA41" s="8"/>
       <c r="AB41" s="8"/>
@@ -2578,7 +2578,7 @@
       <c r="AD41" s="8"/>
       <c r="AE41" s="8"/>
       <c r="AF41" s="10">
-        <v>1199960.02</v>
+        <v>1199960</v>
       </c>
     </row>
     <row r="42" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
@@ -2647,14 +2647,14 @@
       <c r="M43" s="8"/>
       <c r="N43" s="8"/>
       <c r="O43" s="8">
-        <v>127059.20000000001</v>
+        <v>127059</v>
       </c>
       <c r="P43" s="8">
-        <v>127059.20000000001</v>
+        <v>127059</v>
       </c>
       <c r="Q43" s="8"/>
       <c r="R43" s="8">
-        <v>63529.600000000006</v>
+        <v>63530</v>
       </c>
       <c r="S43" s="8"/>
       <c r="T43" s="8"/>
@@ -2698,16 +2698,16 @@
       <c r="R44" s="8"/>
       <c r="S44" s="8"/>
       <c r="T44" s="8">
-        <v>333125.2</v>
+        <v>333125</v>
       </c>
       <c r="U44" s="8">
-        <v>333125.2</v>
+        <v>333125</v>
       </c>
       <c r="V44" s="8"/>
       <c r="W44" s="8"/>
       <c r="X44" s="8"/>
       <c r="Y44" s="8">
-        <v>166562.6</v>
+        <v>166563</v>
       </c>
       <c r="Z44" s="8"/>
       <c r="AA44" s="8"/>
@@ -2724,13 +2724,13 @@
         <v>50</v>
       </c>
       <c r="B45" s="10">
-        <v>341236.34000000008</v>
+        <v>341237</v>
       </c>
       <c r="C45" s="8">
-        <v>136494.53600000002</v>
+        <v>136495</v>
       </c>
       <c r="D45" s="8">
-        <v>136494.53600000002</v>
+        <v>136495</v>
       </c>
       <c r="E45" s="8"/>
       <c r="F45" s="8"/>
@@ -2749,7 +2749,7 @@
       <c r="S45" s="8"/>
       <c r="T45" s="8"/>
       <c r="U45" s="8">
-        <v>68247.268000000011</v>
+        <v>68247</v>
       </c>
       <c r="V45" s="8"/>
       <c r="W45" s="8"/>
@@ -2762,7 +2762,7 @@
       <c r="AD45" s="8"/>
       <c r="AE45" s="8"/>
       <c r="AF45" s="10">
-        <v>341236.34000000008</v>
+        <v>341237</v>
       </c>
     </row>
     <row r="46" spans="1:32" ht="69" x14ac:dyDescent="0.25">
@@ -2950,13 +2950,13 @@
         <v>55</v>
       </c>
       <c r="B50" s="12">
-        <v>11515892.199999999</v>
+        <v>11515894</v>
       </c>
       <c r="C50" s="12">
-        <v>403174.53600000002</v>
+        <v>403175</v>
       </c>
       <c r="D50" s="12">
-        <v>403174.53600000002</v>
+        <v>403175</v>
       </c>
       <c r="E50" s="12">
         <v>0</v>
@@ -2989,43 +2989,43 @@
         <v>0</v>
       </c>
       <c r="O50" s="12">
-        <v>728300.9040000001</v>
+        <v>728301</v>
       </c>
       <c r="P50" s="12">
-        <v>357586.36000000004</v>
+        <v>357586</v>
       </c>
       <c r="Q50" s="12">
         <v>180000</v>
       </c>
       <c r="R50" s="12">
-        <v>1133379.7040000001</v>
+        <v>1133379</v>
       </c>
       <c r="S50" s="12">
-        <v>1059992.3280000002</v>
+        <v>1059992</v>
       </c>
       <c r="T50" s="12">
-        <v>1676462.318</v>
+        <v>1676463</v>
       </c>
       <c r="U50" s="12">
-        <v>1973692.524</v>
+        <v>1973692</v>
       </c>
       <c r="V50" s="12">
-        <v>483789.85600000003</v>
+        <v>483790</v>
       </c>
       <c r="W50" s="12">
-        <v>1464107.362</v>
+        <v>1464107</v>
       </c>
       <c r="X50" s="12">
         <v>0</v>
       </c>
       <c r="Y50" s="12">
-        <v>738375.80799999996</v>
+        <v>738377</v>
       </c>
       <c r="Z50" s="12">
-        <v>543058.16400000011</v>
+        <v>543059</v>
       </c>
       <c r="AA50" s="12">
-        <v>118822.8</v>
+        <v>118823</v>
       </c>
       <c r="AB50" s="12">
         <v>159975</v>
@@ -3040,7 +3040,7 @@
         <v>92000</v>
       </c>
       <c r="AF50" s="12">
-        <v>11515892.199999999</v>
+        <v>11515894</v>
       </c>
     </row>
     <row r="52" spans="1:32" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 18:04)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2254811C-CC9E-4B64-890D-21B2D2EFF920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{96F797A0-30BB-488C-AAE1-C4E70A2A883B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EEA53C07-79A6-4C5E-8ACA-B6EEA73A1EB8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DA10D142-047D-4BD5-A562-BF52EC78E440}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{792798D8-F2ED-4647-80E3-56931337233A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB72E3D4-5F02-42D6-A1B6-B4D3C6663E34}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-19 18:19)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{96F797A0-30BB-488C-AAE1-C4E70A2A883B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C7DE438-D9F7-4785-B559-C6B558D35FE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DA10D142-047D-4BD5-A562-BF52EC78E440}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F94F09D8-6E66-4B2D-9E6F-3D0E6FE6FDDA}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB72E3D4-5F02-42D6-A1B6-B4D3C6663E34}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFB958DD-455B-41AC-B822-89D509A87BB7}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2042,7 +2042,7 @@
         <v>35</v>
       </c>
       <c r="B30" s="10">
-        <v>326787</v>
+        <v>294109</v>
       </c>
       <c r="C30" s="8"/>
       <c r="D30" s="8"/>
@@ -2066,10 +2066,10 @@
       <c r="T30" s="8">
         <v>130715</v>
       </c>
-      <c r="U30" s="8">
-        <v>65357</v>
-      </c>
-      <c r="V30" s="8"/>
+      <c r="U30" s="8"/>
+      <c r="V30" s="8">
+        <v>32679</v>
+      </c>
       <c r="W30" s="8"/>
       <c r="X30" s="8"/>
       <c r="Y30" s="8"/>
@@ -2080,7 +2080,7 @@
       <c r="AD30" s="8"/>
       <c r="AE30" s="8"/>
       <c r="AF30" s="10">
-        <v>326787</v>
+        <v>294109</v>
       </c>
     </row>
     <row r="31" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
@@ -2950,7 +2950,7 @@
         <v>55</v>
       </c>
       <c r="B50" s="12">
-        <v>11515894</v>
+        <v>11483216</v>
       </c>
       <c r="C50" s="12">
         <v>403175</v>
@@ -3007,10 +3007,10 @@
         <v>1676463</v>
       </c>
       <c r="U50" s="12">
-        <v>1973692</v>
+        <v>1908335</v>
       </c>
       <c r="V50" s="12">
-        <v>483790</v>
+        <v>516469</v>
       </c>
       <c r="W50" s="12">
         <v>1464107</v>
@@ -3040,7 +3040,7 @@
         <v>92000</v>
       </c>
       <c r="AF50" s="12">
-        <v>11515894</v>
+        <v>11483216</v>
       </c>
     </row>
     <row r="52" spans="1:32" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 09:23)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C7DE438-D9F7-4785-B559-C6B558D35FE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CEA0FEC-6901-4F2D-A09F-DF003853557A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F94F09D8-6E66-4B2D-9E6F-3D0E6FE6FDDA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C9719E04-8F2D-44C4-A69A-B191511A15C9}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (20 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-19</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-20</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFB958DD-455B-41AC-B822-89D509A87BB7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB5EB1B6-E4D6-4C54-9C63-363BCFC1216B}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 09:33)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3089,4 +3089,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D74681E8-D658-496D-BAE0-85C36138804E}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD577756-2B72-487C-BB25-2A4ADE1A5DBE}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C160286-9597-4E9D-8AF6-6AC7C74A7352}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 14:42)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CEA0FEC-6901-4F2D-A09F-DF003853557A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9A0E94A-41C7-414A-8C78-A44C21DA42AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C9719E04-8F2D-44C4-A69A-B191511A15C9}"/>
+    <workbookView xWindow="4344" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{EA0A9D51-CFF6-4DC7-ABA9-9F0460A05FFE}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB5EB1B6-E4D6-4C54-9C63-363BCFC1216B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F6CEE63-19AE-475A-B02E-1865544E4DA7}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3089,291 +3089,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D74681E8-D658-496D-BAE0-85C36138804E}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD577756-2B72-487C-BB25-2A4ADE1A5DBE}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C160286-9597-4E9D-8AF6-6AC7C74A7352}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 14:44)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3089,4 +3089,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADC05F6C-D979-49C7-8096-59669AE7A897}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48D0C14A-6921-4875-896F-A7DE7E3B9C90}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AFFC27C-97E6-45F0-9188-9DCBF4909796}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 15:04)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9A0E94A-41C7-414A-8C78-A44C21DA42AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8C24E67A-14CE-4D5C-AD00-EBA8485FA61D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4344" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{EA0A9D51-CFF6-4DC7-ABA9-9F0460A05FFE}"/>
+    <workbookView xWindow="4344" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{6C542ECD-AC66-47F8-A39E-251C5AB3F650}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F6CEE63-19AE-475A-B02E-1865544E4DA7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{217DFADA-54C6-46EE-8CB5-2E2638D04DC8}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3089,291 +3089,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADC05F6C-D979-49C7-8096-59669AE7A897}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48D0C14A-6921-4875-896F-A7DE7E3B9C90}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AFFC27C-97E6-45F0-9188-9DCBF4909796}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 15:09)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3089,4 +3089,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C26F82B-8897-4BA5-9CC4-6677B31DED2C}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F7DFCBF-FFC7-483D-A9B3-32AB74AF8814}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C4EA68C-0958-49AF-B68C-E0BB1E0CACC9}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 15:31)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8C24E67A-14CE-4D5C-AD00-EBA8485FA61D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A314247-D4A8-45CD-9DA0-26B34DD6F295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4344" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{6C542ECD-AC66-47F8-A39E-251C5AB3F650}"/>
+    <workbookView xWindow="4344" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{F28E5B8C-6204-4176-88AC-3B87CFAC5E95}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{217DFADA-54C6-46EE-8CB5-2E2638D04DC8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24C81389-74C0-4E7B-8EB4-09E0A0D605EA}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3089,291 +3089,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C26F82B-8897-4BA5-9CC4-6677B31DED2C}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F7DFCBF-FFC7-483D-A9B3-32AB74AF8814}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C4EA68C-0958-49AF-B68C-E0BB1E0CACC9}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 15:34)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3089,4 +3089,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{536AA0F9-F691-437F-AD4B-9A942CD805A8}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6FBD581-BD06-46D2-96F0-90C4452F5919}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0EB7A9CE-94B8-4142-B453-A6F90124BD56}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 15:39)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A314247-D4A8-45CD-9DA0-26B34DD6F295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{195086F6-DAC7-4796-B457-D60A46577DCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4344" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{F28E5B8C-6204-4176-88AC-3B87CFAC5E95}"/>
+    <workbookView xWindow="4344" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{ED1B0027-59BB-486A-A417-5B2DB7741125}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24C81389-74C0-4E7B-8EB4-09E0A0D605EA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E632BA0-90F3-4523-9BEB-D577F9FBDA34}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3089,291 +3089,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{536AA0F9-F691-437F-AD4B-9A942CD805A8}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6FBD581-BD06-46D2-96F0-90C4452F5919}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0EB7A9CE-94B8-4142-B453-A6F90124BD56}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 15:48)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{195086F6-DAC7-4796-B457-D60A46577DCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{604EDF6F-63BA-4DF2-9CF1-A28129650BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4344" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{ED1B0027-59BB-486A-A417-5B2DB7741125}"/>
+    <workbookView xWindow="4344" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{06BA8071-01B0-4084-B512-01955A041940}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E632BA0-90F3-4523-9BEB-D577F9FBDA34}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E03CE84-58B4-4F51-B3B1-004DE81438EA}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 15:58)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{604EDF6F-63BA-4DF2-9CF1-A28129650BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE1894B8-A13D-44BB-911E-FCF8C2898A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4344" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{06BA8071-01B0-4084-B512-01955A041940}"/>
+    <workbookView xWindow="5040" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{D3EDF28F-9245-471C-8775-6D8E35B39311}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E03CE84-58B4-4F51-B3B1-004DE81438EA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E73F6323-06D6-4E74-96CB-C96A37D9584F}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 16:06)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE1894B8-A13D-44BB-911E-FCF8C2898A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3FB9E5EF-C488-48BE-919E-A4229596F373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5040" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{D3EDF28F-9245-471C-8775-6D8E35B39311}"/>
+    <workbookView xWindow="5040" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{4FCEDD1F-459B-42ED-BCFA-F2C721F18DED}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E73F6323-06D6-4E74-96CB-C96A37D9584F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C64BB69-9CEA-45F9-9A8C-2DC7D556D0F4}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 16:08)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3FB9E5EF-C488-48BE-919E-A4229596F373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{210188B8-45D4-43E8-91DF-EEB7238B8AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5040" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{4FCEDD1F-459B-42ED-BCFA-F2C721F18DED}"/>
+    <workbookView xWindow="5040" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{8F80F7E5-62C7-4027-B764-BC718253AA07}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C64BB69-9CEA-45F9-9A8C-2DC7D556D0F4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8426122-58BD-43E8-8E4D-A1E8F41ECF26}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 16:10)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{210188B8-45D4-43E8-91DF-EEB7238B8AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3AAC29B-D85F-4F73-AFCC-9001F440EAA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5040" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{8F80F7E5-62C7-4027-B764-BC718253AA07}"/>
+    <workbookView xWindow="5040" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{43C98709-D32B-42FE-AB4A-1EAB43F48A32}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8426122-58BD-43E8-8E4D-A1E8F41ECF26}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FB02DDB-8E81-479D-B4FB-8085B163FC73}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 16:20)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3089,4 +3089,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18DCB4B7-9264-4209-9356-155CD5A251CB}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{35E5132F-9CAB-4C6A-8C6E-96AFC9834EA9}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E83E0707-98D7-49E1-87CD-CCF9D0A6ED55}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 16:28)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3AAC29B-D85F-4F73-AFCC-9001F440EAA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C7517652-A93E-4E6F-B77B-4C2EC9D81910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5040" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{43C98709-D32B-42FE-AB4A-1EAB43F48A32}"/>
+    <workbookView xWindow="5040" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{BD290B1A-58A4-4B43-AB79-01B0D65FF07C}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FB02DDB-8E81-479D-B4FB-8085B163FC73}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25F84338-D9E0-41E3-BBD3-B6EC03278007}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3089,291 +3089,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18DCB4B7-9264-4209-9356-155CD5A251CB}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{35E5132F-9CAB-4C6A-8C6E-96AFC9834EA9}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E83E0707-98D7-49E1-87CD-CCF9D0A6ED55}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-20 16:48)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C7517652-A93E-4E6F-B77B-4C2EC9D81910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{34A3C07A-4613-48D3-BDB4-9B85862D8497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5040" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{BD290B1A-58A4-4B43-AB79-01B0D65FF07C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C1206866-7684-4577-9CB2-60B26A5294D8}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25F84338-D9E0-41E3-BBD3-B6EC03278007}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F583C52-02E3-4582-A4C3-6E5845FFF56E}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-21 09:16)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{34A3C07A-4613-48D3-BDB4-9B85862D8497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{251FD269-13C4-43B4-903B-B0AF1FDBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C1206866-7684-4577-9CB2-60B26A5294D8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{640B3BD5-3DDD-4895-8E4D-46031EB8A790}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (20 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-20</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-21</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F583C52-02E3-4582-A4C3-6E5845FFF56E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{546C5A41-925A-4B7C-BEB9-A8F8474ACC72}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-21 09:19)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3089,4 +3089,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53478990-52CF-4062-BB41-3DD46BED50B9}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D47FCCE3-A843-4099-B99F-E77651620F9F}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E48DDC36-D720-415D-A9BC-41A8FFE00D88}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{251FD269-13C4-43B4-903B-B0AF1FDBC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD2011ED-9048-419C-B78F-436F7F9C3D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{640B3BD5-3DDD-4895-8E4D-46031EB8A790}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EF824116-A05F-4D5E-8077-35BE0A2E9E39}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -39,12 +39,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="63">
   <si>
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (20 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-21</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-25</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -141,6 +141,21 @@
   </si>
   <si>
     <t>Jun-27</t>
+  </si>
+  <si>
+    <t>Jul-27</t>
+  </si>
+  <si>
+    <t>Aug-27</t>
+  </si>
+  <si>
+    <t>Sep-27</t>
+  </si>
+  <si>
+    <t>Oct-27</t>
+  </si>
+  <si>
+    <t>Nov-27</t>
   </si>
   <si>
     <t>รวม (฿)</t>
@@ -694,18 +709,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{546C5A41-925A-4B7C-BEB9-A8F8474ACC72}">
-  <dimension ref="A1:AF52"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B63DBD54-766B-4C85-B422-6C5EA53B1660}">
+  <dimension ref="A1:AK52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
     <col min="2" max="2" width="15" style="1" customWidth="1"/>
-    <col min="3" max="31" width="11" style="1" customWidth="1"/>
-    <col min="32" max="32" width="15" style="1" customWidth="1"/>
-    <col min="33" max="16384" width="8.88671875" style="1"/>
+    <col min="3" max="36" width="11" style="1" customWidth="1"/>
+    <col min="37" max="37" width="15" style="1" customWidth="1"/>
+    <col min="38" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:37" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -740,8 +755,13 @@
       <c r="AD1" s="2"/>
       <c r="AE1" s="2"/>
       <c r="AF1" s="2"/>
-    </row>
-    <row r="2" spans="1:32" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AG1" s="2"/>
+      <c r="AH1" s="2"/>
+      <c r="AI1" s="2"/>
+      <c r="AJ1" s="2"/>
+      <c r="AK1" s="2"/>
+    </row>
+    <row r="2" spans="1:37" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -776,8 +796,13 @@
       <c r="AD2" s="3"/>
       <c r="AE2" s="3"/>
       <c r="AF2" s="3"/>
-    </row>
-    <row r="4" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AG2" s="3"/>
+      <c r="AH2" s="3"/>
+      <c r="AI2" s="3"/>
+      <c r="AJ2" s="3"/>
+      <c r="AK2" s="3"/>
+    </row>
+    <row r="4" spans="1:37" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -812,8 +837,13 @@
       <c r="AD4" s="5"/>
       <c r="AE4" s="5"/>
       <c r="AF4" s="5"/>
-    </row>
-    <row r="5" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AG4" s="5"/>
+      <c r="AH4" s="5"/>
+      <c r="AI4" s="5"/>
+      <c r="AJ4" s="5"/>
+      <c r="AK4" s="5"/>
+    </row>
+    <row r="5" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
@@ -907,13 +937,28 @@
       <c r="AE5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="AF5" s="6" t="s">
+      <c r="AF5" s="7" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="6" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="AG5" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="AH5" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="AI5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="AJ5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK5" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B6" s="10">
         <v>130000</v>
@@ -953,13 +998,18 @@
       <c r="AC6" s="8"/>
       <c r="AD6" s="8"/>
       <c r="AE6" s="8"/>
-      <c r="AF6" s="10">
+      <c r="AF6" s="8"/>
+      <c r="AG6" s="8"/>
+      <c r="AH6" s="8"/>
+      <c r="AI6" s="8"/>
+      <c r="AJ6" s="8"/>
+      <c r="AK6" s="10">
         <v>130000</v>
       </c>
     </row>
-    <row r="7" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B7" s="10">
         <v>139446</v>
@@ -982,16 +1032,16 @@
       <c r="R7" s="8"/>
       <c r="S7" s="8"/>
       <c r="T7" s="8"/>
-      <c r="U7" s="8">
+      <c r="U7" s="8"/>
+      <c r="V7" s="8">
         <v>41834</v>
       </c>
-      <c r="V7" s="8">
+      <c r="W7" s="8">
         <v>69723</v>
       </c>
-      <c r="W7" s="8">
+      <c r="X7" s="8">
         <v>27889</v>
       </c>
-      <c r="X7" s="8"/>
       <c r="Y7" s="8"/>
       <c r="Z7" s="8"/>
       <c r="AA7" s="8"/>
@@ -999,13 +1049,18 @@
       <c r="AC7" s="8"/>
       <c r="AD7" s="8"/>
       <c r="AE7" s="8"/>
-      <c r="AF7" s="10">
+      <c r="AF7" s="8"/>
+      <c r="AG7" s="8"/>
+      <c r="AH7" s="8"/>
+      <c r="AI7" s="8"/>
+      <c r="AJ7" s="8"/>
+      <c r="AK7" s="10">
         <v>139446</v>
       </c>
     </row>
-    <row r="8" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:37" ht="80.400000000000006" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B8" s="10">
         <v>280000</v>
@@ -1045,13 +1100,18 @@
       <c r="AC8" s="8"/>
       <c r="AD8" s="8"/>
       <c r="AE8" s="8"/>
-      <c r="AF8" s="10">
+      <c r="AF8" s="8"/>
+      <c r="AG8" s="8"/>
+      <c r="AH8" s="8"/>
+      <c r="AI8" s="8"/>
+      <c r="AJ8" s="8"/>
+      <c r="AK8" s="10">
         <v>280000</v>
       </c>
     </row>
-    <row r="9" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B9" s="10">
         <v>89000</v>
@@ -1089,13 +1149,18 @@
       <c r="AC9" s="8"/>
       <c r="AD9" s="8"/>
       <c r="AE9" s="8"/>
-      <c r="AF9" s="10">
+      <c r="AF9" s="8"/>
+      <c r="AG9" s="8"/>
+      <c r="AH9" s="8"/>
+      <c r="AI9" s="8"/>
+      <c r="AJ9" s="8"/>
+      <c r="AK9" s="10">
         <v>89000</v>
       </c>
     </row>
-    <row r="10" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B10" s="10">
         <v>0</v>
@@ -1129,13 +1194,18 @@
       <c r="AC10" s="8"/>
       <c r="AD10" s="8"/>
       <c r="AE10" s="8"/>
-      <c r="AF10" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="AF10" s="8"/>
+      <c r="AG10" s="8"/>
+      <c r="AH10" s="8"/>
+      <c r="AI10" s="8"/>
+      <c r="AJ10" s="8"/>
+      <c r="AK10" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B11" s="10">
         <v>138000</v>
@@ -1173,13 +1243,18 @@
       <c r="AC11" s="8"/>
       <c r="AD11" s="8"/>
       <c r="AE11" s="8"/>
-      <c r="AF11" s="10">
+      <c r="AF11" s="8"/>
+      <c r="AG11" s="8"/>
+      <c r="AH11" s="8"/>
+      <c r="AI11" s="8"/>
+      <c r="AJ11" s="8"/>
+      <c r="AK11" s="10">
         <v>138000</v>
       </c>
     </row>
-    <row r="12" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B12" s="10">
         <v>280000</v>
@@ -1219,13 +1294,18 @@
       <c r="AC12" s="8"/>
       <c r="AD12" s="8"/>
       <c r="AE12" s="8"/>
-      <c r="AF12" s="10">
+      <c r="AF12" s="8"/>
+      <c r="AG12" s="8"/>
+      <c r="AH12" s="8"/>
+      <c r="AI12" s="8"/>
+      <c r="AJ12" s="8"/>
+      <c r="AK12" s="10">
         <v>280000</v>
       </c>
     </row>
-    <row r="13" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B13" s="10">
         <v>233248</v>
@@ -1263,13 +1343,18 @@
       <c r="AC13" s="8"/>
       <c r="AD13" s="8"/>
       <c r="AE13" s="8"/>
-      <c r="AF13" s="10">
+      <c r="AF13" s="8"/>
+      <c r="AG13" s="8"/>
+      <c r="AH13" s="8"/>
+      <c r="AI13" s="8"/>
+      <c r="AJ13" s="8"/>
+      <c r="AK13" s="10">
         <v>233248</v>
       </c>
     </row>
-    <row r="14" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B14" s="10">
         <v>120000</v>
@@ -1294,28 +1379,33 @@
       </c>
       <c r="S14" s="8"/>
       <c r="T14" s="8"/>
-      <c r="U14" s="8">
+      <c r="U14" s="8"/>
+      <c r="V14" s="8"/>
+      <c r="W14" s="8">
         <v>60000</v>
       </c>
-      <c r="V14" s="8"/>
-      <c r="W14" s="8"/>
-      <c r="X14" s="8">
+      <c r="X14" s="8"/>
+      <c r="Y14" s="8"/>
+      <c r="Z14" s="8">
         <v>24000</v>
       </c>
-      <c r="Y14" s="8"/>
-      <c r="Z14" s="8"/>
       <c r="AA14" s="8"/>
       <c r="AB14" s="8"/>
       <c r="AC14" s="8"/>
       <c r="AD14" s="8"/>
       <c r="AE14" s="8"/>
-      <c r="AF14" s="10">
+      <c r="AF14" s="8"/>
+      <c r="AG14" s="8"/>
+      <c r="AH14" s="8"/>
+      <c r="AI14" s="8"/>
+      <c r="AJ14" s="8"/>
+      <c r="AK14" s="10">
         <v>120000</v>
       </c>
     </row>
-    <row r="15" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B15" s="10">
         <v>656680</v>
@@ -1353,13 +1443,18 @@
       <c r="AC15" s="8"/>
       <c r="AD15" s="8"/>
       <c r="AE15" s="8"/>
-      <c r="AF15" s="10">
+      <c r="AF15" s="8"/>
+      <c r="AG15" s="8"/>
+      <c r="AH15" s="8"/>
+      <c r="AI15" s="8"/>
+      <c r="AJ15" s="8"/>
+      <c r="AK15" s="10">
         <v>656680</v>
       </c>
     </row>
-    <row r="16" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B16" s="10">
         <v>40000</v>
@@ -1395,13 +1490,18 @@
       <c r="AC16" s="8"/>
       <c r="AD16" s="8"/>
       <c r="AE16" s="8"/>
-      <c r="AF16" s="10">
+      <c r="AF16" s="8"/>
+      <c r="AG16" s="8"/>
+      <c r="AH16" s="8"/>
+      <c r="AI16" s="8"/>
+      <c r="AJ16" s="8"/>
+      <c r="AK16" s="10">
         <v>40000</v>
       </c>
     </row>
-    <row r="17" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B17" s="10">
         <v>430000</v>
@@ -1441,13 +1541,18 @@
       <c r="AC17" s="8"/>
       <c r="AD17" s="8"/>
       <c r="AE17" s="8"/>
-      <c r="AF17" s="10">
+      <c r="AF17" s="8"/>
+      <c r="AG17" s="8"/>
+      <c r="AH17" s="8"/>
+      <c r="AI17" s="8"/>
+      <c r="AJ17" s="8"/>
+      <c r="AK17" s="10">
         <v>430000</v>
       </c>
     </row>
-    <row r="18" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B18" s="10">
         <v>234860</v>
@@ -1485,13 +1590,18 @@
       <c r="AC18" s="8"/>
       <c r="AD18" s="8"/>
       <c r="AE18" s="8"/>
-      <c r="AF18" s="10">
+      <c r="AF18" s="8"/>
+      <c r="AG18" s="8"/>
+      <c r="AH18" s="8"/>
+      <c r="AI18" s="8"/>
+      <c r="AJ18" s="8"/>
+      <c r="AK18" s="10">
         <v>234860</v>
       </c>
     </row>
-    <row r="19" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B19" s="10">
         <v>119980</v>
@@ -1529,13 +1639,18 @@
       <c r="AC19" s="8"/>
       <c r="AD19" s="8"/>
       <c r="AE19" s="8"/>
-      <c r="AF19" s="10">
+      <c r="AF19" s="8"/>
+      <c r="AG19" s="8"/>
+      <c r="AH19" s="8"/>
+      <c r="AI19" s="8"/>
+      <c r="AJ19" s="8"/>
+      <c r="AK19" s="10">
         <v>119980</v>
       </c>
     </row>
-    <row r="20" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B20" s="10">
         <v>280000</v>
@@ -1575,13 +1690,18 @@
       <c r="AC20" s="8"/>
       <c r="AD20" s="8"/>
       <c r="AE20" s="8"/>
-      <c r="AF20" s="10">
+      <c r="AF20" s="8"/>
+      <c r="AG20" s="8"/>
+      <c r="AH20" s="8"/>
+      <c r="AI20" s="8"/>
+      <c r="AJ20" s="8"/>
+      <c r="AK20" s="10">
         <v>280000</v>
       </c>
     </row>
-    <row r="21" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B21" s="10">
         <v>239148</v>
@@ -1621,13 +1741,18 @@
       <c r="AC21" s="8"/>
       <c r="AD21" s="8"/>
       <c r="AE21" s="8"/>
-      <c r="AF21" s="10">
+      <c r="AF21" s="8"/>
+      <c r="AG21" s="8"/>
+      <c r="AH21" s="8"/>
+      <c r="AI21" s="8"/>
+      <c r="AJ21" s="8"/>
+      <c r="AK21" s="10">
         <v>239148</v>
       </c>
     </row>
-    <row r="22" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B22" s="10">
         <v>224227</v>
@@ -1667,13 +1792,18 @@
       <c r="AC22" s="8"/>
       <c r="AD22" s="8"/>
       <c r="AE22" s="8"/>
-      <c r="AF22" s="10">
+      <c r="AF22" s="8"/>
+      <c r="AG22" s="8"/>
+      <c r="AH22" s="8"/>
+      <c r="AI22" s="8"/>
+      <c r="AJ22" s="8"/>
+      <c r="AK22" s="10">
         <v>224227</v>
       </c>
     </row>
-    <row r="23" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B23" s="10">
         <v>218000</v>
@@ -1713,13 +1843,18 @@
         <v>43600</v>
       </c>
       <c r="AE23" s="8"/>
-      <c r="AF23" s="10">
+      <c r="AF23" s="8"/>
+      <c r="AG23" s="8"/>
+      <c r="AH23" s="8"/>
+      <c r="AI23" s="8"/>
+      <c r="AJ23" s="8"/>
+      <c r="AK23" s="10">
         <v>218000</v>
       </c>
     </row>
-    <row r="24" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B24" s="10">
         <v>58000</v>
@@ -1755,13 +1890,18 @@
       <c r="AC24" s="8"/>
       <c r="AD24" s="8"/>
       <c r="AE24" s="8"/>
-      <c r="AF24" s="10">
+      <c r="AF24" s="8"/>
+      <c r="AG24" s="8"/>
+      <c r="AH24" s="8"/>
+      <c r="AI24" s="8"/>
+      <c r="AJ24" s="8"/>
+      <c r="AK24" s="10">
         <v>58000</v>
       </c>
     </row>
-    <row r="25" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B25" s="10">
         <v>341476</v>
@@ -1788,26 +1928,31 @@
       <c r="V25" s="8">
         <v>102443</v>
       </c>
-      <c r="W25" s="8">
+      <c r="W25" s="8"/>
+      <c r="X25" s="8">
         <v>170738</v>
       </c>
-      <c r="X25" s="8"/>
       <c r="Y25" s="8"/>
       <c r="Z25" s="8"/>
-      <c r="AA25" s="8">
-        <v>68295</v>
-      </c>
+      <c r="AA25" s="8"/>
       <c r="AB25" s="8"/>
       <c r="AC25" s="8"/>
       <c r="AD25" s="8"/>
       <c r="AE25" s="8"/>
-      <c r="AF25" s="10">
+      <c r="AF25" s="8"/>
+      <c r="AG25" s="8"/>
+      <c r="AH25" s="8"/>
+      <c r="AI25" s="8"/>
+      <c r="AJ25" s="8">
+        <v>68295</v>
+      </c>
+      <c r="AK25" s="10">
         <v>341476</v>
       </c>
     </row>
-    <row r="26" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B26" s="12">
         <v>4252065</v>
@@ -1867,25 +2012,25 @@
         <v>739676</v>
       </c>
       <c r="U26" s="12">
-        <v>494234</v>
+        <v>392400</v>
       </c>
       <c r="V26" s="12">
-        <v>264841</v>
+        <v>236952</v>
       </c>
       <c r="W26" s="12">
-        <v>634627</v>
+        <v>565723</v>
       </c>
       <c r="X26" s="12">
-        <v>24000</v>
+        <v>198627</v>
       </c>
       <c r="Y26" s="12">
         <v>155974</v>
       </c>
       <c r="Z26" s="12">
-        <v>163274</v>
+        <v>187274</v>
       </c>
       <c r="AA26" s="12">
-        <v>68295</v>
+        <v>0</v>
       </c>
       <c r="AB26" s="12">
         <v>0</v>
@@ -1900,12 +2045,27 @@
         <v>0</v>
       </c>
       <c r="AF26" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG26" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH26" s="12">
+        <v>0</v>
+      </c>
+      <c r="AI26" s="12">
+        <v>0</v>
+      </c>
+      <c r="AJ26" s="12">
+        <v>68295</v>
+      </c>
+      <c r="AK26" s="12">
         <v>4252065</v>
       </c>
     </row>
-    <row r="28" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:37" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -1938,8 +2098,13 @@
       <c r="AD28" s="5"/>
       <c r="AE28" s="5"/>
       <c r="AF28" s="5"/>
-    </row>
-    <row r="29" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AG28" s="5"/>
+      <c r="AH28" s="5"/>
+      <c r="AI28" s="5"/>
+      <c r="AJ28" s="5"/>
+      <c r="AK28" s="5"/>
+    </row>
+    <row r="29" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>3</v>
       </c>
@@ -2033,13 +2198,28 @@
       <c r="AE29" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="AF29" s="6" t="s">
+      <c r="AF29" s="7" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="30" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="AG29" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="AH29" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="AI29" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="AJ29" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK29" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="30" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B30" s="10">
         <v>294109</v>
@@ -2079,13 +2259,18 @@
       <c r="AC30" s="8"/>
       <c r="AD30" s="8"/>
       <c r="AE30" s="8"/>
-      <c r="AF30" s="10">
+      <c r="AF30" s="8"/>
+      <c r="AG30" s="8"/>
+      <c r="AH30" s="8"/>
+      <c r="AI30" s="8"/>
+      <c r="AJ30" s="8"/>
+      <c r="AK30" s="10">
         <v>294109</v>
       </c>
     </row>
-    <row r="31" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B31" s="10">
         <v>409600</v>
@@ -2108,13 +2293,13 @@
       <c r="R31" s="8"/>
       <c r="S31" s="8"/>
       <c r="T31" s="8"/>
-      <c r="U31" s="8">
-        <v>163840</v>
-      </c>
+      <c r="U31" s="8"/>
       <c r="V31" s="8">
         <v>163840</v>
       </c>
-      <c r="W31" s="8"/>
+      <c r="W31" s="8">
+        <v>163840</v>
+      </c>
       <c r="X31" s="8"/>
       <c r="Y31" s="8">
         <v>81920</v>
@@ -2125,13 +2310,18 @@
       <c r="AC31" s="8"/>
       <c r="AD31" s="8"/>
       <c r="AE31" s="8"/>
-      <c r="AF31" s="10">
+      <c r="AF31" s="8"/>
+      <c r="AG31" s="8"/>
+      <c r="AH31" s="8"/>
+      <c r="AI31" s="8"/>
+      <c r="AJ31" s="8"/>
+      <c r="AK31" s="10">
         <v>409600</v>
       </c>
     </row>
-    <row r="32" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:37" ht="80.400000000000006" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B32" s="10">
         <v>576318</v>
@@ -2171,13 +2361,18 @@
       <c r="AC32" s="8"/>
       <c r="AD32" s="8"/>
       <c r="AE32" s="8"/>
-      <c r="AF32" s="10">
+      <c r="AF32" s="8"/>
+      <c r="AG32" s="8"/>
+      <c r="AH32" s="8"/>
+      <c r="AI32" s="8"/>
+      <c r="AJ32" s="8"/>
+      <c r="AK32" s="10">
         <v>576318</v>
       </c>
     </row>
-    <row r="33" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B33" s="10">
         <v>322960</v>
@@ -2215,13 +2410,18 @@
       <c r="AC33" s="8"/>
       <c r="AD33" s="8"/>
       <c r="AE33" s="8"/>
-      <c r="AF33" s="10">
+      <c r="AF33" s="8"/>
+      <c r="AG33" s="8"/>
+      <c r="AH33" s="8"/>
+      <c r="AI33" s="8"/>
+      <c r="AJ33" s="8"/>
+      <c r="AK33" s="10">
         <v>322960</v>
       </c>
     </row>
-    <row r="34" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B34" s="10">
         <v>252248</v>
@@ -2257,13 +2457,18 @@
       <c r="AC34" s="8"/>
       <c r="AD34" s="8"/>
       <c r="AE34" s="8"/>
-      <c r="AF34" s="10">
+      <c r="AF34" s="8"/>
+      <c r="AG34" s="8"/>
+      <c r="AH34" s="8"/>
+      <c r="AI34" s="8"/>
+      <c r="AJ34" s="8"/>
+      <c r="AK34" s="10">
         <v>252248</v>
       </c>
     </row>
-    <row r="35" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B35" s="10">
         <v>338450</v>
@@ -2303,13 +2508,18 @@
       <c r="AC35" s="8"/>
       <c r="AD35" s="8"/>
       <c r="AE35" s="8"/>
-      <c r="AF35" s="10">
+      <c r="AF35" s="8"/>
+      <c r="AG35" s="8"/>
+      <c r="AH35" s="8"/>
+      <c r="AI35" s="8"/>
+      <c r="AJ35" s="8"/>
+      <c r="AK35" s="10">
         <v>338450</v>
       </c>
     </row>
-    <row r="36" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B36" s="10">
         <v>1156110</v>
@@ -2349,13 +2559,18 @@
       <c r="AC36" s="8"/>
       <c r="AD36" s="8"/>
       <c r="AE36" s="8"/>
-      <c r="AF36" s="10">
+      <c r="AF36" s="8"/>
+      <c r="AG36" s="8"/>
+      <c r="AH36" s="8"/>
+      <c r="AI36" s="8"/>
+      <c r="AJ36" s="8"/>
+      <c r="AK36" s="10">
         <v>1156110</v>
       </c>
     </row>
-    <row r="37" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B37" s="10">
         <v>594115</v>
@@ -2395,13 +2610,18 @@
       <c r="AC37" s="8"/>
       <c r="AD37" s="8"/>
       <c r="AE37" s="8"/>
-      <c r="AF37" s="10">
+      <c r="AF37" s="8"/>
+      <c r="AG37" s="8"/>
+      <c r="AH37" s="8"/>
+      <c r="AI37" s="8"/>
+      <c r="AJ37" s="8"/>
+      <c r="AK37" s="10">
         <v>594115</v>
       </c>
     </row>
-    <row r="38" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B38" s="10">
         <v>327103</v>
@@ -2426,28 +2646,33 @@
       </c>
       <c r="S38" s="8"/>
       <c r="T38" s="8"/>
-      <c r="U38" s="8">
+      <c r="U38" s="8"/>
+      <c r="V38" s="8"/>
+      <c r="W38" s="8">
         <v>130841</v>
       </c>
-      <c r="V38" s="8"/>
-      <c r="W38" s="8"/>
       <c r="X38" s="8"/>
       <c r="Y38" s="8"/>
-      <c r="Z38" s="8">
+      <c r="Z38" s="8"/>
+      <c r="AA38" s="8">
         <v>65421</v>
       </c>
-      <c r="AA38" s="8"/>
       <c r="AB38" s="8"/>
       <c r="AC38" s="8"/>
       <c r="AD38" s="8"/>
       <c r="AE38" s="8"/>
-      <c r="AF38" s="10">
+      <c r="AF38" s="8"/>
+      <c r="AG38" s="8"/>
+      <c r="AH38" s="8"/>
+      <c r="AI38" s="8"/>
+      <c r="AJ38" s="8"/>
+      <c r="AK38" s="10">
         <v>327103</v>
       </c>
     </row>
-    <row r="39" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B39" s="10">
         <v>1707090</v>
@@ -2487,13 +2712,18 @@
       <c r="AC39" s="8"/>
       <c r="AD39" s="8"/>
       <c r="AE39" s="8"/>
-      <c r="AF39" s="10">
+      <c r="AF39" s="8"/>
+      <c r="AG39" s="8"/>
+      <c r="AH39" s="8"/>
+      <c r="AI39" s="8"/>
+      <c r="AJ39" s="8"/>
+      <c r="AK39" s="10">
         <v>1707090</v>
       </c>
     </row>
-    <row r="40" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B40" s="10">
         <v>80000</v>
@@ -2531,13 +2761,18 @@
       <c r="AC40" s="8"/>
       <c r="AD40" s="8"/>
       <c r="AE40" s="8"/>
-      <c r="AF40" s="10">
+      <c r="AF40" s="8"/>
+      <c r="AG40" s="8"/>
+      <c r="AH40" s="8"/>
+      <c r="AI40" s="8"/>
+      <c r="AJ40" s="8"/>
+      <c r="AK40" s="10">
         <v>80000</v>
       </c>
     </row>
-    <row r="41" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B41" s="10">
         <v>1199960</v>
@@ -2577,13 +2812,18 @@
       <c r="AC41" s="8"/>
       <c r="AD41" s="8"/>
       <c r="AE41" s="8"/>
-      <c r="AF41" s="10">
+      <c r="AF41" s="8"/>
+      <c r="AG41" s="8"/>
+      <c r="AH41" s="8"/>
+      <c r="AI41" s="8"/>
+      <c r="AJ41" s="8"/>
+      <c r="AK41" s="10">
         <v>1199960</v>
       </c>
     </row>
-    <row r="42" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B42" s="10">
         <v>600000</v>
@@ -2623,13 +2863,18 @@
       <c r="AC42" s="8"/>
       <c r="AD42" s="8"/>
       <c r="AE42" s="8"/>
-      <c r="AF42" s="10">
+      <c r="AF42" s="8"/>
+      <c r="AG42" s="8"/>
+      <c r="AH42" s="8"/>
+      <c r="AI42" s="8"/>
+      <c r="AJ42" s="8"/>
+      <c r="AK42" s="10">
         <v>600000</v>
       </c>
     </row>
-    <row r="43" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A43" s="9" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B43" s="10">
         <v>317648</v>
@@ -2669,13 +2914,18 @@
       <c r="AC43" s="8"/>
       <c r="AD43" s="8"/>
       <c r="AE43" s="8"/>
-      <c r="AF43" s="10">
+      <c r="AF43" s="8"/>
+      <c r="AG43" s="8"/>
+      <c r="AH43" s="8"/>
+      <c r="AI43" s="8"/>
+      <c r="AJ43" s="8"/>
+      <c r="AK43" s="10">
         <v>317648</v>
       </c>
     </row>
-    <row r="44" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B44" s="10">
         <v>832813</v>
@@ -2715,13 +2965,18 @@
       <c r="AC44" s="8"/>
       <c r="AD44" s="8"/>
       <c r="AE44" s="8"/>
-      <c r="AF44" s="10">
+      <c r="AF44" s="8"/>
+      <c r="AG44" s="8"/>
+      <c r="AH44" s="8"/>
+      <c r="AI44" s="8"/>
+      <c r="AJ44" s="8"/>
+      <c r="AK44" s="10">
         <v>832813</v>
       </c>
     </row>
-    <row r="45" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B45" s="10">
         <v>341237</v>
@@ -2761,13 +3016,18 @@
       <c r="AC45" s="8"/>
       <c r="AD45" s="8"/>
       <c r="AE45" s="8"/>
-      <c r="AF45" s="10">
+      <c r="AF45" s="8"/>
+      <c r="AG45" s="8"/>
+      <c r="AH45" s="8"/>
+      <c r="AI45" s="8"/>
+      <c r="AJ45" s="8"/>
+      <c r="AK45" s="10">
         <v>341237</v>
       </c>
     </row>
-    <row r="46" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B46" s="10">
         <v>666700</v>
@@ -2807,13 +3067,18 @@
       <c r="AC46" s="8"/>
       <c r="AD46" s="8"/>
       <c r="AE46" s="8"/>
-      <c r="AF46" s="10">
+      <c r="AF46" s="8"/>
+      <c r="AG46" s="8"/>
+      <c r="AH46" s="8"/>
+      <c r="AI46" s="8"/>
+      <c r="AJ46" s="8"/>
+      <c r="AK46" s="10">
         <v>666700</v>
       </c>
     </row>
-    <row r="47" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B47" s="10">
         <v>460000</v>
@@ -2853,13 +3118,18 @@
       <c r="AE47" s="8">
         <v>92000</v>
       </c>
-      <c r="AF47" s="10">
+      <c r="AF47" s="8"/>
+      <c r="AG47" s="8"/>
+      <c r="AH47" s="8"/>
+      <c r="AI47" s="8"/>
+      <c r="AJ47" s="8"/>
+      <c r="AK47" s="10">
         <v>460000</v>
       </c>
     </row>
-    <row r="48" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B48" s="10">
         <v>206880</v>
@@ -2895,13 +3165,18 @@
       <c r="AC48" s="8"/>
       <c r="AD48" s="8"/>
       <c r="AE48" s="8"/>
-      <c r="AF48" s="10">
+      <c r="AF48" s="8"/>
+      <c r="AG48" s="8"/>
+      <c r="AH48" s="8"/>
+      <c r="AI48" s="8"/>
+      <c r="AJ48" s="8"/>
+      <c r="AK48" s="10">
         <v>206880</v>
       </c>
     </row>
-    <row r="49" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B49" s="10">
         <v>799875</v>
@@ -2928,10 +3203,10 @@
       <c r="V49" s="8">
         <v>319950</v>
       </c>
-      <c r="W49" s="8">
+      <c r="W49" s="8"/>
+      <c r="X49" s="8">
         <v>319950</v>
       </c>
-      <c r="X49" s="8"/>
       <c r="Y49" s="8"/>
       <c r="Z49" s="8"/>
       <c r="AA49" s="8"/>
@@ -2941,13 +3216,18 @@
       <c r="AC49" s="8"/>
       <c r="AD49" s="8"/>
       <c r="AE49" s="8"/>
-      <c r="AF49" s="10">
+      <c r="AF49" s="8"/>
+      <c r="AG49" s="8"/>
+      <c r="AH49" s="8"/>
+      <c r="AI49" s="8"/>
+      <c r="AJ49" s="8"/>
+      <c r="AK49" s="10">
         <v>799875</v>
       </c>
     </row>
-    <row r="50" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B50" s="12">
         <v>11483216</v>
@@ -3007,25 +3287,25 @@
         <v>1676463</v>
       </c>
       <c r="U50" s="12">
-        <v>1908335</v>
+        <v>1613654</v>
       </c>
       <c r="V50" s="12">
         <v>516469</v>
       </c>
       <c r="W50" s="12">
-        <v>1464107</v>
+        <v>1438838</v>
       </c>
       <c r="X50" s="12">
-        <v>0</v>
+        <v>319950</v>
       </c>
       <c r="Y50" s="12">
         <v>738377</v>
       </c>
       <c r="Z50" s="12">
-        <v>543059</v>
+        <v>477638</v>
       </c>
       <c r="AA50" s="12">
-        <v>118823</v>
+        <v>184244</v>
       </c>
       <c r="AB50" s="12">
         <v>159975</v>
@@ -3040,12 +3320,27 @@
         <v>92000</v>
       </c>
       <c r="AF50" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG50" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH50" s="12">
+        <v>0</v>
+      </c>
+      <c r="AI50" s="12">
+        <v>0</v>
+      </c>
+      <c r="AJ50" s="12">
+        <v>0</v>
+      </c>
+      <c r="AK50" s="12">
         <v>11483216</v>
       </c>
     </row>
-    <row r="52" spans="1:32" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -3078,14 +3373,19 @@
       <c r="AD52" s="4"/>
       <c r="AE52" s="4"/>
       <c r="AF52" s="4"/>
+      <c r="AG52" s="4"/>
+      <c r="AH52" s="4"/>
+      <c r="AI52" s="4"/>
+      <c r="AJ52" s="4"/>
+      <c r="AK52" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:AF1"/>
-    <mergeCell ref="A2:AF2"/>
-    <mergeCell ref="A52:AF52"/>
-    <mergeCell ref="A4:AF4"/>
-    <mergeCell ref="A28:AF28"/>
+    <mergeCell ref="A1:AK1"/>
+    <mergeCell ref="A2:AK2"/>
+    <mergeCell ref="A52:AK52"/>
+    <mergeCell ref="A4:AK4"/>
+    <mergeCell ref="A28:AK28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3367,13 +3667,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53478990-52CF-4062-BB41-3DD46BED50B9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C00B9C26-D045-493A-BE6E-63C09BC1CBAA}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D47FCCE3-A843-4099-B99F-E77651620F9F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05173B43-544D-42D0-8336-EB2EC8CE5A13}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E48DDC36-D720-415D-A9BC-41A8FFE00D88}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{324F0E58-FEAF-4649-8120-D7A1A3CD0F16}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-25 15:54)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD2011ED-9048-419C-B78F-436F7F9C3D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9990DB78-8636-4E57-8079-32F628F8C7B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EF824116-A05F-4D5E-8077-35BE0A2E9E39}"/>
+    <workbookView xWindow="4260" yWindow="1008" windowWidth="17280" windowHeight="8880" xr2:uid="{EE619DE5-EDBD-43A5-A551-3C67CF44E62F}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -227,7 +227,7 @@
     <t>② Forecast Revenue รายเดือน (฿)  —  รับงวด 1-3 ตามวันที่จริง</t>
   </si>
   <si>
-    <t>หมายเหตุ: ตัวเลขชุดเดียวกับกราฟ Financial Forecast บน Dashboard · Cost = เงินจ่ายผู้รับเหมา คอลัมน์ K/N/P ลงตามวันที่ L/O/Q · Forecast = รับงวด 1 (Sale Price x 40% ลงวันที่ L) + งวด 2 (คอลัมน์ S วันที่ T) + งวด 3 (คอลัมน์ U วันที่ V) · นับเฉพาะรายการที่มีวันที่ในชีต</t>
+    <t>หมายเหตุ: ตัวเลขชุดเดียวกับกราฟ Financial Forecast บน Dashboard · Cost = เงินจ่ายผู้รับเหมา คอลัมน์ K/N/P ลงตามวันที่ L/O/Q · Forecast = รับงวด 1 (Sale Price x 40% ลงวันที่ X ถ้ามี มิฉะนั้นใช้ L) + งวด 2 (คอลัมน์ S วันที่ T) + งวด 3 (คอลัมน์ U วันที่ V) · นับเฉพาะรายการที่มีวันที่ในชีต</t>
   </si>
 </sst>
 </file>
@@ -709,7 +709,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B63DBD54-766B-4C85-B422-6C5EA53B1660}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8178116-99C2-4FBE-A2C8-552C2CE95738}">
   <dimension ref="A1:AK52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2291,12 +2291,12 @@
       <c r="P31" s="8"/>
       <c r="Q31" s="8"/>
       <c r="R31" s="8"/>
-      <c r="S31" s="8"/>
+      <c r="S31" s="8">
+        <v>163840</v>
+      </c>
       <c r="T31" s="8"/>
       <c r="U31" s="8"/>
-      <c r="V31" s="8">
-        <v>163840</v>
-      </c>
+      <c r="V31" s="8"/>
       <c r="W31" s="8">
         <v>163840</v>
       </c>
@@ -3281,7 +3281,7 @@
         <v>1133379</v>
       </c>
       <c r="S50" s="12">
-        <v>1059992</v>
+        <v>1223832</v>
       </c>
       <c r="T50" s="12">
         <v>1676463</v>
@@ -3290,7 +3290,7 @@
         <v>1613654</v>
       </c>
       <c r="V50" s="12">
-        <v>516469</v>
+        <v>352629</v>
       </c>
       <c r="W50" s="12">
         <v>1438838</v>
@@ -3389,291 +3389,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C00B9C26-D045-493A-BE6E-63C09BC1CBAA}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05173B43-544D-42D0-8336-EB2EC8CE5A13}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{324F0E58-FEAF-4649-8120-D7A1A3CD0F16}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-25 15:56)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9990DB78-8636-4E57-8079-32F628F8C7B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6583FDE-21FB-49BB-9113-0380E3781378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4260" yWindow="1008" windowWidth="17280" windowHeight="8880" xr2:uid="{EE619DE5-EDBD-43A5-A551-3C67CF44E62F}"/>
+    <workbookView xWindow="4260" yWindow="1008" windowWidth="17280" windowHeight="8880" xr2:uid="{BAB356DC-42FA-45C9-AB98-07B61D8D6AAA}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -709,7 +709,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8178116-99C2-4FBE-A2C8-552C2CE95738}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8B91C3A-9211-4541-9D08-18BCBEEEDBDE}">
   <dimension ref="A1:AK52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2291,12 +2291,12 @@
       <c r="P31" s="8"/>
       <c r="Q31" s="8"/>
       <c r="R31" s="8"/>
-      <c r="S31" s="8">
-        <v>163840</v>
-      </c>
+      <c r="S31" s="8"/>
       <c r="T31" s="8"/>
       <c r="U31" s="8"/>
-      <c r="V31" s="8"/>
+      <c r="V31" s="8">
+        <v>163840</v>
+      </c>
       <c r="W31" s="8">
         <v>163840</v>
       </c>
@@ -3281,7 +3281,7 @@
         <v>1133379</v>
       </c>
       <c r="S50" s="12">
-        <v>1223832</v>
+        <v>1059992</v>
       </c>
       <c r="T50" s="12">
         <v>1676463</v>
@@ -3290,7 +3290,7 @@
         <v>1613654</v>
       </c>
       <c r="V50" s="12">
-        <v>352629</v>
+        <v>516469</v>
       </c>
       <c r="W50" s="12">
         <v>1438838</v>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-25 17:15)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6583FDE-21FB-49BB-9113-0380E3781378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{344D1C7A-1F79-4B71-BF96-91BC36688255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4260" yWindow="1008" windowWidth="17280" windowHeight="8880" xr2:uid="{BAB356DC-42FA-45C9-AB98-07B61D8D6AAA}"/>
+    <workbookView xWindow="4260" yWindow="1008" windowWidth="17280" windowHeight="8880" xr2:uid="{E95C1914-8A79-4345-9700-E44435DB7F02}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -709,7 +709,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8B91C3A-9211-4541-9D08-18BCBEEEDBDE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D6F4E31-F35F-49EB-8D85-2BE98755E9C7}">
   <dimension ref="A1:AK52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-27 09:23)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{344D1C7A-1F79-4B71-BF96-91BC36688255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{641C3744-3BA9-4D40-8ECF-535E65BC3FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4260" yWindow="1008" windowWidth="17280" windowHeight="8880" xr2:uid="{E95C1914-8A79-4345-9700-E44435DB7F02}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AFB5640D-9C78-4267-A0C6-46D24577AE27}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (20 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-25</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-27</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -709,7 +709,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D6F4E31-F35F-49EB-8D85-2BE98755E9C7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C243354F-B627-4413-96ED-4A1A650B74A2}">
   <dimension ref="A1:AK52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-27 09:32)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{641C3744-3BA9-4D40-8ECF-535E65BC3FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B91FA58-25C4-45D8-9A1C-3F191A53DB79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AFB5640D-9C78-4267-A0C6-46D24577AE27}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EA41CC95-99BC-45FF-8BBB-2B05A8F1AA4E}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -709,7 +709,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C243354F-B627-4413-96ED-4A1A650B74A2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DB72412-2AA6-4C6F-9BD7-ABAEDECB5AF4}">
   <dimension ref="A1:AK52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-27 09:41)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B91FA58-25C4-45D8-9A1C-3F191A53DB79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C02692F-A7D7-494E-9034-F63082F51395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EA41CC95-99BC-45FF-8BBB-2B05A8F1AA4E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{20AF644E-6E85-415C-8350-1CCABEA9464C}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -709,7 +709,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DB72412-2AA6-4C6F-9BD7-ABAEDECB5AF4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88D8A6E5-00F8-48CD-84F0-FE85EA09DD52}">
   <dimension ref="A1:AK52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2793,11 +2793,11 @@
       <c r="P41" s="8"/>
       <c r="Q41" s="8"/>
       <c r="R41" s="8"/>
-      <c r="S41" s="8"/>
+      <c r="S41" s="8">
+        <v>479984</v>
+      </c>
       <c r="T41" s="8"/>
-      <c r="U41" s="8">
-        <v>479984</v>
-      </c>
+      <c r="U41" s="8"/>
       <c r="V41" s="8"/>
       <c r="W41" s="8">
         <v>479984</v>
@@ -3151,9 +3151,11 @@
       <c r="Q48" s="8"/>
       <c r="R48" s="8"/>
       <c r="S48" s="8"/>
-      <c r="T48" s="8"/>
+      <c r="T48" s="8">
+        <v>82752</v>
+      </c>
       <c r="U48" s="8">
-        <v>206880</v>
+        <v>124128</v>
       </c>
       <c r="V48" s="8"/>
       <c r="W48" s="8"/>
@@ -3281,13 +3283,13 @@
         <v>1133379</v>
       </c>
       <c r="S50" s="12">
-        <v>1059992</v>
+        <v>1539976</v>
       </c>
       <c r="T50" s="12">
-        <v>1676463</v>
+        <v>1759215</v>
       </c>
       <c r="U50" s="12">
-        <v>1613654</v>
+        <v>1050918</v>
       </c>
       <c r="V50" s="12">
         <v>516469</v>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-27 09:44)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3391,4 +3391,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6424BC6-CE2C-4F8B-9DBB-B4BF2C456929}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14DED4A3-8405-4CC0-A91A-C66E3FF617A9}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{597EFCDE-F165-4A19-BBEA-F00E0EB4296F}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-27 09:48)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C02692F-A7D7-494E-9034-F63082F51395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{40225EA5-C0C0-466D-A904-437A6EF3E6D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{20AF644E-6E85-415C-8350-1CCABEA9464C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{03C8BB53-DE82-4A96-BBB8-288CF8B795E9}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -709,7 +709,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88D8A6E5-00F8-48CD-84F0-FE85EA09DD52}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56B618DE-E8E8-4EEF-8CB2-A9A5AA59B01E}">
   <dimension ref="A1:AK52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3391,291 +3391,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6424BC6-CE2C-4F8B-9DBB-B4BF2C456929}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14DED4A3-8405-4CC0-A91A-C66E3FF617A9}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{597EFCDE-F165-4A19-BBEA-F00E0EB4296F}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-27 09:50)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{40225EA5-C0C0-466D-A904-437A6EF3E6D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D44A482C-B998-4B96-AB61-7E81E5068DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{03C8BB53-DE82-4A96-BBB8-288CF8B795E9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9A8D9570-842E-4A5D-91D5-18CDA98F26C5}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -709,7 +709,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56B618DE-E8E8-4EEF-8CB2-A9A5AA59B01E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13A52BA2-70BD-42AA-BF60-699828282D7F}">
   <dimension ref="A1:AK52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2951,13 +2951,13 @@
         <v>333125</v>
       </c>
       <c r="U44" s="8">
-        <v>333125</v>
+        <v>249844</v>
       </c>
       <c r="V44" s="8"/>
       <c r="W44" s="8"/>
       <c r="X44" s="8"/>
       <c r="Y44" s="8">
-        <v>166563</v>
+        <v>249844</v>
       </c>
       <c r="Z44" s="8"/>
       <c r="AA44" s="8"/>
@@ -3289,7 +3289,7 @@
         <v>1759215</v>
       </c>
       <c r="U50" s="12">
-        <v>1050918</v>
+        <v>967637</v>
       </c>
       <c r="V50" s="12">
         <v>516469</v>
@@ -3301,7 +3301,7 @@
         <v>319950</v>
       </c>
       <c r="Y50" s="12">
-        <v>738377</v>
+        <v>821658</v>
       </c>
       <c r="Z50" s="12">
         <v>477638</v>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-27 09:57)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D44A482C-B998-4B96-AB61-7E81E5068DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C0EC0BA1-11BE-44BA-BF4B-E6168B07B4BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9A8D9570-842E-4A5D-91D5-18CDA98F26C5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B7FBEAE2-359D-4E27-BDD7-D1E435B9FF20}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -709,7 +709,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13A52BA2-70BD-42AA-BF60-699828282D7F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD833C28-E598-4B99-B370-447B6AA8E918}">
   <dimension ref="A1:AK52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-27 10:04)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3391,4 +3391,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C70931D-00E0-4C0E-A97F-00FC25B64D6D}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99859A7D-65E1-48AE-94F3-DB11CB4A7BA7}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1468BFC3-5B1E-4C8F-BF7C-0A37AE260061}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-27 10:09)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C0EC0BA1-11BE-44BA-BF4B-E6168B07B4BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5DD3D450-BBB0-47A2-8157-1FA657BFB0A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B7FBEAE2-359D-4E27-BDD7-D1E435B9FF20}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4DE18957-FD36-4757-A063-F3E72C77B50B}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -709,7 +709,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD833C28-E598-4B99-B370-447B6AA8E918}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2242E7CB-17C2-42D9-910D-CBB1CFD50070}">
   <dimension ref="A1:AK52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3100,10 +3100,10 @@
       <c r="Q47" s="8"/>
       <c r="R47" s="8"/>
       <c r="S47" s="8"/>
-      <c r="T47" s="8"/>
-      <c r="U47" s="8">
+      <c r="T47" s="8">
         <v>184000</v>
       </c>
+      <c r="U47" s="8"/>
       <c r="V47" s="8"/>
       <c r="W47" s="8">
         <v>184000</v>
@@ -3286,10 +3286,10 @@
         <v>1539976</v>
       </c>
       <c r="T50" s="12">
-        <v>1759215</v>
+        <v>1943215</v>
       </c>
       <c r="U50" s="12">
-        <v>967637</v>
+        <v>783637</v>
       </c>
       <c r="V50" s="12">
         <v>516469</v>
@@ -3391,291 +3391,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C70931D-00E0-4C0E-A97F-00FC25B64D6D}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99859A7D-65E1-48AE-94F3-DB11CB4A7BA7}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1468BFC3-5B1E-4C8F-BF7C-0A37AE260061}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-27 10:12)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5DD3D450-BBB0-47A2-8157-1FA657BFB0A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{82C1E68F-585A-4AD4-A3D5-BC64901B8583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4DE18957-FD36-4757-A063-F3E72C77B50B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AE87049D-145D-4E68-B4C9-D755D6ACAE1B}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -709,7 +709,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2242E7CB-17C2-42D9-910D-CBB1CFD50070}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A27843E-64F7-490D-B491-F63AAED60A65}">
   <dimension ref="A1:AK52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1826,10 +1826,10 @@
       <c r="R23" s="8"/>
       <c r="S23" s="8"/>
       <c r="T23" s="8"/>
-      <c r="U23" s="8">
+      <c r="U23" s="8"/>
+      <c r="V23" s="8">
         <v>65400</v>
       </c>
-      <c r="V23" s="8"/>
       <c r="W23" s="8">
         <v>109000</v>
       </c>
@@ -2012,10 +2012,10 @@
         <v>739676</v>
       </c>
       <c r="U26" s="12">
-        <v>392400</v>
+        <v>327000</v>
       </c>
       <c r="V26" s="12">
-        <v>236952</v>
+        <v>302352</v>
       </c>
       <c r="W26" s="12">
         <v>565723</v>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-27 10:14)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{82C1E68F-585A-4AD4-A3D5-BC64901B8583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C440238-1B89-4C6D-AB96-C79FFCAB6CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AE87049D-145D-4E68-B4C9-D755D6ACAE1B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D6888D61-B304-433D-B139-F3BE922C4F5D}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -709,7 +709,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A27843E-64F7-490D-B491-F63AAED60A65}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86B98B49-0539-42D3-87D0-364943F21A57}">
   <dimension ref="A1:AK52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-27 10:22)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C440238-1B89-4C6D-AB96-C79FFCAB6CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D40BA29F-D88C-4807-9371-437197E31665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D6888D61-B304-433D-B139-F3BE922C4F5D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DA7F9EC5-5C99-463B-849D-B83DEA854FB3}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="58">
   <si>
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (20 โครงการ PO)</t>
   </si>
@@ -141,21 +141,6 @@
   </si>
   <si>
     <t>Jun-27</t>
-  </si>
-  <si>
-    <t>Jul-27</t>
-  </si>
-  <si>
-    <t>Aug-27</t>
-  </si>
-  <si>
-    <t>Sep-27</t>
-  </si>
-  <si>
-    <t>Oct-27</t>
-  </si>
-  <si>
-    <t>Nov-27</t>
   </si>
   <si>
     <t>รวม (฿)</t>
@@ -709,18 +694,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86B98B49-0539-42D3-87D0-364943F21A57}">
-  <dimension ref="A1:AK52"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{331FE809-C83A-4E5B-977F-7C75901AA62D}">
+  <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
     <col min="2" max="2" width="15" style="1" customWidth="1"/>
-    <col min="3" max="36" width="11" style="1" customWidth="1"/>
-    <col min="37" max="37" width="15" style="1" customWidth="1"/>
-    <col min="38" max="16384" width="8.88671875" style="1"/>
+    <col min="3" max="31" width="11" style="1" customWidth="1"/>
+    <col min="32" max="32" width="15" style="1" customWidth="1"/>
+    <col min="33" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:32" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -755,13 +740,8 @@
       <c r="AD1" s="2"/>
       <c r="AE1" s="2"/>
       <c r="AF1" s="2"/>
-      <c r="AG1" s="2"/>
-      <c r="AH1" s="2"/>
-      <c r="AI1" s="2"/>
-      <c r="AJ1" s="2"/>
-      <c r="AK1" s="2"/>
-    </row>
-    <row r="2" spans="1:37" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:32" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -796,13 +776,8 @@
       <c r="AD2" s="3"/>
       <c r="AE2" s="3"/>
       <c r="AF2" s="3"/>
-      <c r="AG2" s="3"/>
-      <c r="AH2" s="3"/>
-      <c r="AI2" s="3"/>
-      <c r="AJ2" s="3"/>
-      <c r="AK2" s="3"/>
-    </row>
-    <row r="4" spans="1:37" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -837,13 +812,8 @@
       <c r="AD4" s="5"/>
       <c r="AE4" s="5"/>
       <c r="AF4" s="5"/>
-      <c r="AG4" s="5"/>
-      <c r="AH4" s="5"/>
-      <c r="AI4" s="5"/>
-      <c r="AJ4" s="5"/>
-      <c r="AK4" s="5"/>
-    </row>
-    <row r="5" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
@@ -937,28 +907,13 @@
       <c r="AE5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="AF5" s="7" t="s">
+      <c r="AF5" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="AG5" s="7" t="s">
+    </row>
+    <row r="6" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
         <v>35</v>
-      </c>
-      <c r="AH5" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="AI5" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="AJ5" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="AK5" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>40</v>
       </c>
       <c r="B6" s="10">
         <v>130000</v>
@@ -998,18 +953,13 @@
       <c r="AC6" s="8"/>
       <c r="AD6" s="8"/>
       <c r="AE6" s="8"/>
-      <c r="AF6" s="8"/>
-      <c r="AG6" s="8"/>
-      <c r="AH6" s="8"/>
-      <c r="AI6" s="8"/>
-      <c r="AJ6" s="8"/>
-      <c r="AK6" s="10">
+      <c r="AF6" s="10">
         <v>130000</v>
       </c>
     </row>
-    <row r="7" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B7" s="10">
         <v>139446</v>
@@ -1049,18 +999,13 @@
       <c r="AC7" s="8"/>
       <c r="AD7" s="8"/>
       <c r="AE7" s="8"/>
-      <c r="AF7" s="8"/>
-      <c r="AG7" s="8"/>
-      <c r="AH7" s="8"/>
-      <c r="AI7" s="8"/>
-      <c r="AJ7" s="8"/>
-      <c r="AK7" s="10">
+      <c r="AF7" s="10">
         <v>139446</v>
       </c>
     </row>
-    <row r="8" spans="1:37" ht="80.400000000000006" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B8" s="10">
         <v>280000</v>
@@ -1100,18 +1045,13 @@
       <c r="AC8" s="8"/>
       <c r="AD8" s="8"/>
       <c r="AE8" s="8"/>
-      <c r="AF8" s="8"/>
-      <c r="AG8" s="8"/>
-      <c r="AH8" s="8"/>
-      <c r="AI8" s="8"/>
-      <c r="AJ8" s="8"/>
-      <c r="AK8" s="10">
+      <c r="AF8" s="10">
         <v>280000</v>
       </c>
     </row>
-    <row r="9" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B9" s="10">
         <v>89000</v>
@@ -1149,18 +1089,13 @@
       <c r="AC9" s="8"/>
       <c r="AD9" s="8"/>
       <c r="AE9" s="8"/>
-      <c r="AF9" s="8"/>
-      <c r="AG9" s="8"/>
-      <c r="AH9" s="8"/>
-      <c r="AI9" s="8"/>
-      <c r="AJ9" s="8"/>
-      <c r="AK9" s="10">
+      <c r="AF9" s="10">
         <v>89000</v>
       </c>
     </row>
-    <row r="10" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B10" s="10">
         <v>0</v>
@@ -1194,18 +1129,13 @@
       <c r="AC10" s="8"/>
       <c r="AD10" s="8"/>
       <c r="AE10" s="8"/>
-      <c r="AF10" s="8"/>
-      <c r="AG10" s="8"/>
-      <c r="AH10" s="8"/>
-      <c r="AI10" s="8"/>
-      <c r="AJ10" s="8"/>
-      <c r="AK10" s="10">
+      <c r="AF10" s="10">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B11" s="10">
         <v>138000</v>
@@ -1243,18 +1173,13 @@
       <c r="AC11" s="8"/>
       <c r="AD11" s="8"/>
       <c r="AE11" s="8"/>
-      <c r="AF11" s="8"/>
-      <c r="AG11" s="8"/>
-      <c r="AH11" s="8"/>
-      <c r="AI11" s="8"/>
-      <c r="AJ11" s="8"/>
-      <c r="AK11" s="10">
+      <c r="AF11" s="10">
         <v>138000</v>
       </c>
     </row>
-    <row r="12" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B12" s="10">
         <v>280000</v>
@@ -1294,18 +1219,13 @@
       <c r="AC12" s="8"/>
       <c r="AD12" s="8"/>
       <c r="AE12" s="8"/>
-      <c r="AF12" s="8"/>
-      <c r="AG12" s="8"/>
-      <c r="AH12" s="8"/>
-      <c r="AI12" s="8"/>
-      <c r="AJ12" s="8"/>
-      <c r="AK12" s="10">
+      <c r="AF12" s="10">
         <v>280000</v>
       </c>
     </row>
-    <row r="13" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B13" s="10">
         <v>233248</v>
@@ -1343,18 +1263,13 @@
       <c r="AC13" s="8"/>
       <c r="AD13" s="8"/>
       <c r="AE13" s="8"/>
-      <c r="AF13" s="8"/>
-      <c r="AG13" s="8"/>
-      <c r="AH13" s="8"/>
-      <c r="AI13" s="8"/>
-      <c r="AJ13" s="8"/>
-      <c r="AK13" s="10">
+      <c r="AF13" s="10">
         <v>233248</v>
       </c>
     </row>
-    <row r="14" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B14" s="10">
         <v>120000</v>
@@ -1394,18 +1309,13 @@
       <c r="AC14" s="8"/>
       <c r="AD14" s="8"/>
       <c r="AE14" s="8"/>
-      <c r="AF14" s="8"/>
-      <c r="AG14" s="8"/>
-      <c r="AH14" s="8"/>
-      <c r="AI14" s="8"/>
-      <c r="AJ14" s="8"/>
-      <c r="AK14" s="10">
+      <c r="AF14" s="10">
         <v>120000</v>
       </c>
     </row>
-    <row r="15" spans="1:37" ht="69" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B15" s="10">
         <v>656680</v>
@@ -1443,18 +1353,13 @@
       <c r="AC15" s="8"/>
       <c r="AD15" s="8"/>
       <c r="AE15" s="8"/>
-      <c r="AF15" s="8"/>
-      <c r="AG15" s="8"/>
-      <c r="AH15" s="8"/>
-      <c r="AI15" s="8"/>
-      <c r="AJ15" s="8"/>
-      <c r="AK15" s="10">
+      <c r="AF15" s="10">
         <v>656680</v>
       </c>
     </row>
-    <row r="16" spans="1:37" ht="69" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B16" s="10">
         <v>40000</v>
@@ -1490,18 +1395,13 @@
       <c r="AC16" s="8"/>
       <c r="AD16" s="8"/>
       <c r="AE16" s="8"/>
-      <c r="AF16" s="8"/>
-      <c r="AG16" s="8"/>
-      <c r="AH16" s="8"/>
-      <c r="AI16" s="8"/>
-      <c r="AJ16" s="8"/>
-      <c r="AK16" s="10">
+      <c r="AF16" s="10">
         <v>40000</v>
       </c>
     </row>
-    <row r="17" spans="1:37" ht="69" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B17" s="10">
         <v>430000</v>
@@ -1541,18 +1441,13 @@
       <c r="AC17" s="8"/>
       <c r="AD17" s="8"/>
       <c r="AE17" s="8"/>
-      <c r="AF17" s="8"/>
-      <c r="AG17" s="8"/>
-      <c r="AH17" s="8"/>
-      <c r="AI17" s="8"/>
-      <c r="AJ17" s="8"/>
-      <c r="AK17" s="10">
+      <c r="AF17" s="10">
         <v>430000</v>
       </c>
     </row>
-    <row r="18" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B18" s="10">
         <v>234860</v>
@@ -1590,18 +1485,13 @@
       <c r="AC18" s="8"/>
       <c r="AD18" s="8"/>
       <c r="AE18" s="8"/>
-      <c r="AF18" s="8"/>
-      <c r="AG18" s="8"/>
-      <c r="AH18" s="8"/>
-      <c r="AI18" s="8"/>
-      <c r="AJ18" s="8"/>
-      <c r="AK18" s="10">
+      <c r="AF18" s="10">
         <v>234860</v>
       </c>
     </row>
-    <row r="19" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B19" s="10">
         <v>119980</v>
@@ -1639,18 +1529,13 @@
       <c r="AC19" s="8"/>
       <c r="AD19" s="8"/>
       <c r="AE19" s="8"/>
-      <c r="AF19" s="8"/>
-      <c r="AG19" s="8"/>
-      <c r="AH19" s="8"/>
-      <c r="AI19" s="8"/>
-      <c r="AJ19" s="8"/>
-      <c r="AK19" s="10">
+      <c r="AF19" s="10">
         <v>119980</v>
       </c>
     </row>
-    <row r="20" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B20" s="10">
         <v>280000</v>
@@ -1690,18 +1575,13 @@
       <c r="AC20" s="8"/>
       <c r="AD20" s="8"/>
       <c r="AE20" s="8"/>
-      <c r="AF20" s="8"/>
-      <c r="AG20" s="8"/>
-      <c r="AH20" s="8"/>
-      <c r="AI20" s="8"/>
-      <c r="AJ20" s="8"/>
-      <c r="AK20" s="10">
+      <c r="AF20" s="10">
         <v>280000</v>
       </c>
     </row>
-    <row r="21" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B21" s="10">
         <v>239148</v>
@@ -1741,18 +1621,13 @@
       <c r="AC21" s="8"/>
       <c r="AD21" s="8"/>
       <c r="AE21" s="8"/>
-      <c r="AF21" s="8"/>
-      <c r="AG21" s="8"/>
-      <c r="AH21" s="8"/>
-      <c r="AI21" s="8"/>
-      <c r="AJ21" s="8"/>
-      <c r="AK21" s="10">
+      <c r="AF21" s="10">
         <v>239148</v>
       </c>
     </row>
-    <row r="22" spans="1:37" ht="69" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B22" s="10">
         <v>224227</v>
@@ -1792,18 +1667,13 @@
       <c r="AC22" s="8"/>
       <c r="AD22" s="8"/>
       <c r="AE22" s="8"/>
-      <c r="AF22" s="8"/>
-      <c r="AG22" s="8"/>
-      <c r="AH22" s="8"/>
-      <c r="AI22" s="8"/>
-      <c r="AJ22" s="8"/>
-      <c r="AK22" s="10">
+      <c r="AF22" s="10">
         <v>224227</v>
       </c>
     </row>
-    <row r="23" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B23" s="10">
         <v>218000</v>
@@ -1843,18 +1713,13 @@
         <v>43600</v>
       </c>
       <c r="AE23" s="8"/>
-      <c r="AF23" s="8"/>
-      <c r="AG23" s="8"/>
-      <c r="AH23" s="8"/>
-      <c r="AI23" s="8"/>
-      <c r="AJ23" s="8"/>
-      <c r="AK23" s="10">
+      <c r="AF23" s="10">
         <v>218000</v>
       </c>
     </row>
-    <row r="24" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B24" s="10">
         <v>58000</v>
@@ -1890,18 +1755,13 @@
       <c r="AC24" s="8"/>
       <c r="AD24" s="8"/>
       <c r="AE24" s="8"/>
-      <c r="AF24" s="8"/>
-      <c r="AG24" s="8"/>
-      <c r="AH24" s="8"/>
-      <c r="AI24" s="8"/>
-      <c r="AJ24" s="8"/>
-      <c r="AK24" s="10">
+      <c r="AF24" s="10">
         <v>58000</v>
       </c>
     </row>
-    <row r="25" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B25" s="10">
         <v>341476</v>
@@ -1930,7 +1790,7 @@
       </c>
       <c r="W25" s="8"/>
       <c r="X25" s="8">
-        <v>170738</v>
+        <v>239033</v>
       </c>
       <c r="Y25" s="8"/>
       <c r="Z25" s="8"/>
@@ -1939,20 +1799,13 @@
       <c r="AC25" s="8"/>
       <c r="AD25" s="8"/>
       <c r="AE25" s="8"/>
-      <c r="AF25" s="8"/>
-      <c r="AG25" s="8"/>
-      <c r="AH25" s="8"/>
-      <c r="AI25" s="8"/>
-      <c r="AJ25" s="8">
-        <v>68295</v>
-      </c>
-      <c r="AK25" s="10">
+      <c r="AF25" s="10">
         <v>341476</v>
       </c>
     </row>
-    <row r="26" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B26" s="12">
         <v>4252065</v>
@@ -2021,7 +1874,7 @@
         <v>565723</v>
       </c>
       <c r="X26" s="12">
-        <v>198627</v>
+        <v>266922</v>
       </c>
       <c r="Y26" s="12">
         <v>155974</v>
@@ -2045,27 +1898,12 @@
         <v>0</v>
       </c>
       <c r="AF26" s="12">
-        <v>0</v>
-      </c>
-      <c r="AG26" s="12">
-        <v>0</v>
-      </c>
-      <c r="AH26" s="12">
-        <v>0</v>
-      </c>
-      <c r="AI26" s="12">
-        <v>0</v>
-      </c>
-      <c r="AJ26" s="12">
-        <v>68295</v>
-      </c>
-      <c r="AK26" s="12">
         <v>4252065</v>
       </c>
     </row>
-    <row r="28" spans="1:37" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -2098,13 +1936,8 @@
       <c r="AD28" s="5"/>
       <c r="AE28" s="5"/>
       <c r="AF28" s="5"/>
-      <c r="AG28" s="5"/>
-      <c r="AH28" s="5"/>
-      <c r="AI28" s="5"/>
-      <c r="AJ28" s="5"/>
-      <c r="AK28" s="5"/>
-    </row>
-    <row r="29" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>3</v>
       </c>
@@ -2198,28 +2031,13 @@
       <c r="AE29" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="AF29" s="7" t="s">
+      <c r="AF29" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="AG29" s="7" t="s">
+    </row>
+    <row r="30" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A30" s="9" t="s">
         <v>35</v>
-      </c>
-      <c r="AH29" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="AI29" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="AJ29" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="AK29" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="30" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A30" s="9" t="s">
-        <v>40</v>
       </c>
       <c r="B30" s="10">
         <v>294109</v>
@@ -2259,18 +2077,13 @@
       <c r="AC30" s="8"/>
       <c r="AD30" s="8"/>
       <c r="AE30" s="8"/>
-      <c r="AF30" s="8"/>
-      <c r="AG30" s="8"/>
-      <c r="AH30" s="8"/>
-      <c r="AI30" s="8"/>
-      <c r="AJ30" s="8"/>
-      <c r="AK30" s="10">
+      <c r="AF30" s="10">
         <v>294109</v>
       </c>
     </row>
-    <row r="31" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B31" s="10">
         <v>409600</v>
@@ -2310,18 +2123,13 @@
       <c r="AC31" s="8"/>
       <c r="AD31" s="8"/>
       <c r="AE31" s="8"/>
-      <c r="AF31" s="8"/>
-      <c r="AG31" s="8"/>
-      <c r="AH31" s="8"/>
-      <c r="AI31" s="8"/>
-      <c r="AJ31" s="8"/>
-      <c r="AK31" s="10">
+      <c r="AF31" s="10">
         <v>409600</v>
       </c>
     </row>
-    <row r="32" spans="1:37" ht="80.400000000000006" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B32" s="10">
         <v>576318</v>
@@ -2361,18 +2169,13 @@
       <c r="AC32" s="8"/>
       <c r="AD32" s="8"/>
       <c r="AE32" s="8"/>
-      <c r="AF32" s="8"/>
-      <c r="AG32" s="8"/>
-      <c r="AH32" s="8"/>
-      <c r="AI32" s="8"/>
-      <c r="AJ32" s="8"/>
-      <c r="AK32" s="10">
+      <c r="AF32" s="10">
         <v>576318</v>
       </c>
     </row>
-    <row r="33" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B33" s="10">
         <v>322960</v>
@@ -2410,18 +2213,13 @@
       <c r="AC33" s="8"/>
       <c r="AD33" s="8"/>
       <c r="AE33" s="8"/>
-      <c r="AF33" s="8"/>
-      <c r="AG33" s="8"/>
-      <c r="AH33" s="8"/>
-      <c r="AI33" s="8"/>
-      <c r="AJ33" s="8"/>
-      <c r="AK33" s="10">
+      <c r="AF33" s="10">
         <v>322960</v>
       </c>
     </row>
-    <row r="34" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B34" s="10">
         <v>252248</v>
@@ -2457,18 +2255,13 @@
       <c r="AC34" s="8"/>
       <c r="AD34" s="8"/>
       <c r="AE34" s="8"/>
-      <c r="AF34" s="8"/>
-      <c r="AG34" s="8"/>
-      <c r="AH34" s="8"/>
-      <c r="AI34" s="8"/>
-      <c r="AJ34" s="8"/>
-      <c r="AK34" s="10">
+      <c r="AF34" s="10">
         <v>252248</v>
       </c>
     </row>
-    <row r="35" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B35" s="10">
         <v>338450</v>
@@ -2508,18 +2301,13 @@
       <c r="AC35" s="8"/>
       <c r="AD35" s="8"/>
       <c r="AE35" s="8"/>
-      <c r="AF35" s="8"/>
-      <c r="AG35" s="8"/>
-      <c r="AH35" s="8"/>
-      <c r="AI35" s="8"/>
-      <c r="AJ35" s="8"/>
-      <c r="AK35" s="10">
+      <c r="AF35" s="10">
         <v>338450</v>
       </c>
     </row>
-    <row r="36" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B36" s="10">
         <v>1156110</v>
@@ -2559,18 +2347,13 @@
       <c r="AC36" s="8"/>
       <c r="AD36" s="8"/>
       <c r="AE36" s="8"/>
-      <c r="AF36" s="8"/>
-      <c r="AG36" s="8"/>
-      <c r="AH36" s="8"/>
-      <c r="AI36" s="8"/>
-      <c r="AJ36" s="8"/>
-      <c r="AK36" s="10">
+      <c r="AF36" s="10">
         <v>1156110</v>
       </c>
     </row>
-    <row r="37" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B37" s="10">
         <v>594115</v>
@@ -2610,18 +2393,13 @@
       <c r="AC37" s="8"/>
       <c r="AD37" s="8"/>
       <c r="AE37" s="8"/>
-      <c r="AF37" s="8"/>
-      <c r="AG37" s="8"/>
-      <c r="AH37" s="8"/>
-      <c r="AI37" s="8"/>
-      <c r="AJ37" s="8"/>
-      <c r="AK37" s="10">
+      <c r="AF37" s="10">
         <v>594115</v>
       </c>
     </row>
-    <row r="38" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B38" s="10">
         <v>327103</v>
@@ -2661,18 +2439,13 @@
       <c r="AC38" s="8"/>
       <c r="AD38" s="8"/>
       <c r="AE38" s="8"/>
-      <c r="AF38" s="8"/>
-      <c r="AG38" s="8"/>
-      <c r="AH38" s="8"/>
-      <c r="AI38" s="8"/>
-      <c r="AJ38" s="8"/>
-      <c r="AK38" s="10">
+      <c r="AF38" s="10">
         <v>327103</v>
       </c>
     </row>
-    <row r="39" spans="1:37" ht="69" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B39" s="10">
         <v>1707090</v>
@@ -2712,18 +2485,13 @@
       <c r="AC39" s="8"/>
       <c r="AD39" s="8"/>
       <c r="AE39" s="8"/>
-      <c r="AF39" s="8"/>
-      <c r="AG39" s="8"/>
-      <c r="AH39" s="8"/>
-      <c r="AI39" s="8"/>
-      <c r="AJ39" s="8"/>
-      <c r="AK39" s="10">
+      <c r="AF39" s="10">
         <v>1707090</v>
       </c>
     </row>
-    <row r="40" spans="1:37" ht="69" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B40" s="10">
         <v>80000</v>
@@ -2761,18 +2529,13 @@
       <c r="AC40" s="8"/>
       <c r="AD40" s="8"/>
       <c r="AE40" s="8"/>
-      <c r="AF40" s="8"/>
-      <c r="AG40" s="8"/>
-      <c r="AH40" s="8"/>
-      <c r="AI40" s="8"/>
-      <c r="AJ40" s="8"/>
-      <c r="AK40" s="10">
+      <c r="AF40" s="10">
         <v>80000</v>
       </c>
     </row>
-    <row r="41" spans="1:37" ht="69" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B41" s="10">
         <v>1199960</v>
@@ -2812,18 +2575,13 @@
       <c r="AC41" s="8"/>
       <c r="AD41" s="8"/>
       <c r="AE41" s="8"/>
-      <c r="AF41" s="8"/>
-      <c r="AG41" s="8"/>
-      <c r="AH41" s="8"/>
-      <c r="AI41" s="8"/>
-      <c r="AJ41" s="8"/>
-      <c r="AK41" s="10">
+      <c r="AF41" s="10">
         <v>1199960</v>
       </c>
     </row>
-    <row r="42" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B42" s="10">
         <v>600000</v>
@@ -2863,18 +2621,13 @@
       <c r="AC42" s="8"/>
       <c r="AD42" s="8"/>
       <c r="AE42" s="8"/>
-      <c r="AF42" s="8"/>
-      <c r="AG42" s="8"/>
-      <c r="AH42" s="8"/>
-      <c r="AI42" s="8"/>
-      <c r="AJ42" s="8"/>
-      <c r="AK42" s="10">
+      <c r="AF42" s="10">
         <v>600000</v>
       </c>
     </row>
-    <row r="43" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A43" s="9" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B43" s="10">
         <v>317648</v>
@@ -2914,18 +2667,13 @@
       <c r="AC43" s="8"/>
       <c r="AD43" s="8"/>
       <c r="AE43" s="8"/>
-      <c r="AF43" s="8"/>
-      <c r="AG43" s="8"/>
-      <c r="AH43" s="8"/>
-      <c r="AI43" s="8"/>
-      <c r="AJ43" s="8"/>
-      <c r="AK43" s="10">
+      <c r="AF43" s="10">
         <v>317648</v>
       </c>
     </row>
-    <row r="44" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B44" s="10">
         <v>832813</v>
@@ -2965,18 +2713,13 @@
       <c r="AC44" s="8"/>
       <c r="AD44" s="8"/>
       <c r="AE44" s="8"/>
-      <c r="AF44" s="8"/>
-      <c r="AG44" s="8"/>
-      <c r="AH44" s="8"/>
-      <c r="AI44" s="8"/>
-      <c r="AJ44" s="8"/>
-      <c r="AK44" s="10">
+      <c r="AF44" s="10">
         <v>832813</v>
       </c>
     </row>
-    <row r="45" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B45" s="10">
         <v>341237</v>
@@ -3016,18 +2759,13 @@
       <c r="AC45" s="8"/>
       <c r="AD45" s="8"/>
       <c r="AE45" s="8"/>
-      <c r="AF45" s="8"/>
-      <c r="AG45" s="8"/>
-      <c r="AH45" s="8"/>
-      <c r="AI45" s="8"/>
-      <c r="AJ45" s="8"/>
-      <c r="AK45" s="10">
+      <c r="AF45" s="10">
         <v>341237</v>
       </c>
     </row>
-    <row r="46" spans="1:37" ht="69" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B46" s="10">
         <v>666700</v>
@@ -3067,18 +2805,13 @@
       <c r="AC46" s="8"/>
       <c r="AD46" s="8"/>
       <c r="AE46" s="8"/>
-      <c r="AF46" s="8"/>
-      <c r="AG46" s="8"/>
-      <c r="AH46" s="8"/>
-      <c r="AI46" s="8"/>
-      <c r="AJ46" s="8"/>
-      <c r="AK46" s="10">
+      <c r="AF46" s="10">
         <v>666700</v>
       </c>
     </row>
-    <row r="47" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B47" s="10">
         <v>460000</v>
@@ -3118,18 +2851,13 @@
       <c r="AE47" s="8">
         <v>92000</v>
       </c>
-      <c r="AF47" s="8"/>
-      <c r="AG47" s="8"/>
-      <c r="AH47" s="8"/>
-      <c r="AI47" s="8"/>
-      <c r="AJ47" s="8"/>
-      <c r="AK47" s="10">
+      <c r="AF47" s="10">
         <v>460000</v>
       </c>
     </row>
-    <row r="48" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B48" s="10">
         <v>206880</v>
@@ -3167,18 +2895,13 @@
       <c r="AC48" s="8"/>
       <c r="AD48" s="8"/>
       <c r="AE48" s="8"/>
-      <c r="AF48" s="8"/>
-      <c r="AG48" s="8"/>
-      <c r="AH48" s="8"/>
-      <c r="AI48" s="8"/>
-      <c r="AJ48" s="8"/>
-      <c r="AK48" s="10">
+      <c r="AF48" s="10">
         <v>206880</v>
       </c>
     </row>
-    <row r="49" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B49" s="10">
         <v>799875</v>
@@ -3218,18 +2941,13 @@
       <c r="AC49" s="8"/>
       <c r="AD49" s="8"/>
       <c r="AE49" s="8"/>
-      <c r="AF49" s="8"/>
-      <c r="AG49" s="8"/>
-      <c r="AH49" s="8"/>
-      <c r="AI49" s="8"/>
-      <c r="AJ49" s="8"/>
-      <c r="AK49" s="10">
+      <c r="AF49" s="10">
         <v>799875</v>
       </c>
     </row>
-    <row r="50" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B50" s="12">
         <v>11483216</v>
@@ -3322,27 +3040,12 @@
         <v>92000</v>
       </c>
       <c r="AF50" s="12">
-        <v>0</v>
-      </c>
-      <c r="AG50" s="12">
-        <v>0</v>
-      </c>
-      <c r="AH50" s="12">
-        <v>0</v>
-      </c>
-      <c r="AI50" s="12">
-        <v>0</v>
-      </c>
-      <c r="AJ50" s="12">
-        <v>0</v>
-      </c>
-      <c r="AK50" s="12">
         <v>11483216</v>
       </c>
     </row>
-    <row r="52" spans="1:37" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -3375,19 +3078,14 @@
       <c r="AD52" s="4"/>
       <c r="AE52" s="4"/>
       <c r="AF52" s="4"/>
-      <c r="AG52" s="4"/>
-      <c r="AH52" s="4"/>
-      <c r="AI52" s="4"/>
-      <c r="AJ52" s="4"/>
-      <c r="AK52" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:AK1"/>
-    <mergeCell ref="A2:AK2"/>
-    <mergeCell ref="A52:AK52"/>
-    <mergeCell ref="A4:AK4"/>
-    <mergeCell ref="A28:AK28"/>
+    <mergeCell ref="A1:AF1"/>
+    <mergeCell ref="A2:AF2"/>
+    <mergeCell ref="A52:AF52"/>
+    <mergeCell ref="A4:AF4"/>
+    <mergeCell ref="A28:AF28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-27 11:10)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D40BA29F-D88C-4807-9371-437197E31665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1E2F13A-7487-4C27-9A21-5D81173D08C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DA7F9EC5-5C99-463B-849D-B83DEA854FB3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4374AAE7-999F-4BD4-B09F-6A149B9BA9D0}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{331FE809-C83A-4E5B-977F-7C75901AA62D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89DCAD69-D813-4F19-B3A6-7171C6B02FAE}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2746,10 +2746,10 @@
       <c r="R45" s="8"/>
       <c r="S45" s="8"/>
       <c r="T45" s="8"/>
-      <c r="U45" s="8">
+      <c r="U45" s="8"/>
+      <c r="V45" s="8">
         <v>68247</v>
       </c>
-      <c r="V45" s="8"/>
       <c r="W45" s="8"/>
       <c r="X45" s="8"/>
       <c r="Y45" s="8"/>
@@ -3007,10 +3007,10 @@
         <v>1943215</v>
       </c>
       <c r="U50" s="12">
-        <v>783637</v>
+        <v>715390</v>
       </c>
       <c r="V50" s="12">
-        <v>516469</v>
+        <v>584716</v>
       </c>
       <c r="W50" s="12">
         <v>1438838</v>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-27 13:09)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1E2F13A-7487-4C27-9A21-5D81173D08C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{95D0977E-6787-4CEE-B6D1-9822CD8E4036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4374AAE7-999F-4BD4-B09F-6A149B9BA9D0}"/>
+    <workbookView xWindow="16032" yWindow="960" windowWidth="6492" windowHeight="8880" xr2:uid="{4BD74E39-681A-4640-809D-7568BE912155}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89DCAD69-D813-4F19-B3A6-7171C6B02FAE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04EE38BE-B9CB-45FB-8E83-EB40FA505942}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-28 11:34)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{95D0977E-6787-4CEE-B6D1-9822CD8E4036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E0C8C11-5D38-4A3B-85CD-B008B6DB0B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16032" yWindow="960" windowWidth="6492" windowHeight="8880" xr2:uid="{4BD74E39-681A-4640-809D-7568BE912155}"/>
+    <workbookView xWindow="8520" yWindow="1392" windowWidth="14328" windowHeight="8880" xr2:uid="{06B71865-819E-4741-A7CE-C3A982BD0CEF}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (20 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-27</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-28</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04EE38BE-B9CB-45FB-8E83-EB40FA505942}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{637E9759-2039-43E7-BCE8-F47C10F1B166}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-31 09:10)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E0C8C11-5D38-4A3B-85CD-B008B6DB0B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{56BF79A2-DE1C-47F7-BDDE-57CD9656AFF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8520" yWindow="1392" windowWidth="14328" windowHeight="8880" xr2:uid="{06B71865-819E-4741-A7CE-C3A982BD0CEF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8CD568EF-2049-4BF9-BF0F-ED5163385586}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (20 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-28</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-31</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{637E9759-2039-43E7-BCE8-F47C10F1B166}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32B163C2-DCF6-485F-8680-48CB3ACCD1C5}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-31 09:14)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3089,4 +3089,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C1B16921-93CD-4DDC-AB78-0EF5BC603710}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22B71ED8-D99B-4572-BB5C-4A18D5A2A7AA}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3FCBDBB-DE6D-4CB0-BDD8-A057FDC580CB}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-31 09:16)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{56BF79A2-DE1C-47F7-BDDE-57CD9656AFF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AED41BFF-B871-47AB-8289-F46FE6052608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8CD568EF-2049-4BF9-BF0F-ED5163385586}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B406086F-4EA6-4639-BB29-424CC9181CF6}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32B163C2-DCF6-485F-8680-48CB3ACCD1C5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C737084E-7F07-4A35-906A-0B0945464F8A}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3089,291 +3089,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C1B16921-93CD-4DDC-AB78-0EF5BC603710}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22B71ED8-D99B-4572-BB5C-4A18D5A2A7AA}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3FCBDBB-DE6D-4CB0-BDD8-A057FDC580CB}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-31 10:19)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AED41BFF-B871-47AB-8289-F46FE6052608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B7DAE37-3BB0-444F-9147-BB98FEF0940B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B406086F-4EA6-4639-BB29-424CC9181CF6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{87C2C07D-8358-40CE-98B9-DEDA89BBE9F9}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C737084E-7F07-4A35-906A-0B0945464F8A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{591B81DF-B969-4FAF-8428-2032F3FDEFC2}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-31 10:25)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3089,4 +3089,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{400800F6-8A37-4F45-B9F6-61019D1A8A14}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94ED64C7-0CD5-43DD-9194-4196BA09D275}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9EE32FAA-358B-4F1A-B71F-965F0FA5B242}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-31 10:34)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B7DAE37-3BB0-444F-9147-BB98FEF0940B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{353AA814-F7EA-4914-843C-CC8A0E452079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{87C2C07D-8358-40CE-98B9-DEDA89BBE9F9}"/>
+    <workbookView xWindow="5928" yWindow="1668" windowWidth="14328" windowHeight="8880" xr2:uid="{A29608CB-4C02-43CC-B5A4-A4DDB5F24A28}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{591B81DF-B969-4FAF-8428-2032F3FDEFC2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{491E2E2A-6458-44DB-AE28-11D02E2BB1C0}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2924,10 +2924,10 @@
       <c r="R49" s="8"/>
       <c r="S49" s="8"/>
       <c r="T49" s="8"/>
-      <c r="U49" s="8"/>
-      <c r="V49" s="8">
+      <c r="U49" s="8">
         <v>319950</v>
       </c>
+      <c r="V49" s="8"/>
       <c r="W49" s="8"/>
       <c r="X49" s="8">
         <v>319950</v>
@@ -3007,10 +3007,10 @@
         <v>1943215</v>
       </c>
       <c r="U50" s="12">
-        <v>715390</v>
+        <v>1035340</v>
       </c>
       <c r="V50" s="12">
-        <v>584716</v>
+        <v>264766</v>
       </c>
       <c r="W50" s="12">
         <v>1438838</v>
@@ -3089,291 +3089,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{400800F6-8A37-4F45-B9F6-61019D1A8A14}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94ED64C7-0CD5-43DD-9194-4196BA09D275}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9EE32FAA-358B-4F1A-B71F-965F0FA5B242}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-31 10:37)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{353AA814-F7EA-4914-843C-CC8A0E452079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{217539F1-A18C-4833-98E8-5C7A7186A946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5928" yWindow="1668" windowWidth="14328" windowHeight="8880" xr2:uid="{A29608CB-4C02-43CC-B5A4-A4DDB5F24A28}"/>
+    <workbookView xWindow="5928" yWindow="1668" windowWidth="14328" windowHeight="8880" xr2:uid="{A1C8F763-B325-46CA-9232-3D6AA270B6DB}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{491E2E2A-6458-44DB-AE28-11D02E2BB1C0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD0387C0-44E8-4F96-A923-FE296B81DD6F}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2101,15 +2101,15 @@
       <c r="M31" s="8"/>
       <c r="N31" s="8"/>
       <c r="O31" s="8"/>
-      <c r="P31" s="8"/>
+      <c r="P31" s="8">
+        <v>163840</v>
+      </c>
       <c r="Q31" s="8"/>
       <c r="R31" s="8"/>
       <c r="S31" s="8"/>
       <c r="T31" s="8"/>
       <c r="U31" s="8"/>
-      <c r="V31" s="8">
-        <v>163840</v>
-      </c>
+      <c r="V31" s="8"/>
       <c r="W31" s="8">
         <v>163840</v>
       </c>
@@ -2992,7 +2992,7 @@
         <v>728301</v>
       </c>
       <c r="P50" s="12">
-        <v>357586</v>
+        <v>521426</v>
       </c>
       <c r="Q50" s="12">
         <v>180000</v>
@@ -3010,7 +3010,7 @@
         <v>1035340</v>
       </c>
       <c r="V50" s="12">
-        <v>264766</v>
+        <v>100926</v>
       </c>
       <c r="W50" s="12">
         <v>1438838</v>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-31 10:40)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{217539F1-A18C-4833-98E8-5C7A7186A946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0383EA28-511B-4AAF-9AD1-10DB1C700647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5928" yWindow="1668" windowWidth="14328" windowHeight="8880" xr2:uid="{A1C8F763-B325-46CA-9232-3D6AA270B6DB}"/>
+    <workbookView xWindow="5928" yWindow="1668" windowWidth="14328" windowHeight="8880" xr2:uid="{5D0F6AD3-2906-4874-BFCE-4D3EA3275C83}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD0387C0-44E8-4F96-A923-FE296B81DD6F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56CE0CE3-614E-42AD-BD58-362DC89C7A66}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1655,10 +1655,10 @@
       <c r="S22" s="8"/>
       <c r="T22" s="8"/>
       <c r="U22" s="8"/>
-      <c r="V22" s="8">
+      <c r="V22" s="8"/>
+      <c r="W22" s="8">
         <v>44845</v>
       </c>
-      <c r="W22" s="8"/>
       <c r="X22" s="8"/>
       <c r="Y22" s="8"/>
       <c r="Z22" s="8"/>
@@ -1868,10 +1868,10 @@
         <v>327000</v>
       </c>
       <c r="V26" s="12">
-        <v>302352</v>
+        <v>257507</v>
       </c>
       <c r="W26" s="12">
-        <v>565723</v>
+        <v>610568</v>
       </c>
       <c r="X26" s="12">
         <v>266922</v>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-31 10:48)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0383EA28-511B-4AAF-9AD1-10DB1C700647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D0DAF08-F134-46AC-9B50-677E289B79B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5928" yWindow="1668" windowWidth="14328" windowHeight="8880" xr2:uid="{5D0F6AD3-2906-4874-BFCE-4D3EA3275C83}"/>
+    <workbookView xWindow="5928" yWindow="1668" windowWidth="14328" windowHeight="8880" xr2:uid="{F9668CF8-C909-4957-BD32-AA5B0E5CC572}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56CE0CE3-614E-42AD-BD58-362DC89C7A66}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71306498-FACC-49A5-B04D-00D7A30A557A}">
   <dimension ref="A1:AF52"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1584,7 +1584,7 @@
         <v>50</v>
       </c>
       <c r="B21" s="10">
-        <v>239148</v>
+        <v>284858</v>
       </c>
       <c r="C21" s="8">
         <v>71744</v>
@@ -1610,7 +1610,7 @@
       <c r="T21" s="8"/>
       <c r="U21" s="8"/>
       <c r="V21" s="8">
-        <v>47830</v>
+        <v>93540</v>
       </c>
       <c r="W21" s="8"/>
       <c r="X21" s="8"/>
@@ -1622,7 +1622,7 @@
       <c r="AD21" s="8"/>
       <c r="AE21" s="8"/>
       <c r="AF21" s="10">
-        <v>239148</v>
+        <v>284858</v>
       </c>
     </row>
     <row r="22" spans="1:32" ht="69" x14ac:dyDescent="0.25">
@@ -1630,7 +1630,7 @@
         <v>51</v>
       </c>
       <c r="B22" s="10">
-        <v>224227</v>
+        <v>246650</v>
       </c>
       <c r="C22" s="8">
         <v>67268</v>
@@ -1657,7 +1657,7 @@
       <c r="U22" s="8"/>
       <c r="V22" s="8"/>
       <c r="W22" s="8">
-        <v>44845</v>
+        <v>67268</v>
       </c>
       <c r="X22" s="8"/>
       <c r="Y22" s="8"/>
@@ -1668,7 +1668,7 @@
       <c r="AD22" s="8"/>
       <c r="AE22" s="8"/>
       <c r="AF22" s="10">
-        <v>224227</v>
+        <v>246650</v>
       </c>
     </row>
     <row r="23" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
@@ -1808,7 +1808,7 @@
         <v>55</v>
       </c>
       <c r="B26" s="12">
-        <v>4252065</v>
+        <v>4320198</v>
       </c>
       <c r="C26" s="12">
         <v>139012</v>
@@ -1868,10 +1868,10 @@
         <v>327000</v>
       </c>
       <c r="V26" s="12">
-        <v>257507</v>
+        <v>303217</v>
       </c>
       <c r="W26" s="12">
-        <v>610568</v>
+        <v>632991</v>
       </c>
       <c r="X26" s="12">
         <v>266922</v>
@@ -1898,7 +1898,7 @@
         <v>0</v>
       </c>
       <c r="AF26" s="12">
-        <v>4252065</v>
+        <v>4320198</v>
       </c>
     </row>
     <row r="28" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-31 11:27)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D0DAF08-F134-46AC-9B50-677E289B79B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{05B320A9-604F-4C76-A34B-75425A592C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5928" yWindow="1668" windowWidth="14328" windowHeight="8880" xr2:uid="{F9668CF8-C909-4957-BD32-AA5B0E5CC572}"/>
+    <workbookView xWindow="5928" yWindow="1668" windowWidth="14328" windowHeight="8880" xr2:uid="{72E01C85-E361-44C9-8AD2-133DCDFE32D3}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -39,9 +39,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="58">
-  <si>
-    <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (20 โครงการ PO)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="59">
+  <si>
+    <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (21 โครงการ PO)</t>
   </si>
   <si>
     <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-31</t>
@@ -204,6 +204,9 @@
   </si>
   <si>
     <t>CRLEV-26-025  Achalaboon Residence</t>
+  </si>
+  <si>
+    <t>K'Ink &amp; K'Cody Residence</t>
   </si>
   <si>
     <t>รวมทั้งหมด (Total)</t>
@@ -694,8 +697,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71306498-FACC-49A5-B04D-00D7A30A557A}">
-  <dimension ref="A1:AF52"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33AF483C-E886-4AE5-A452-03ABB9A8EEE3}">
+  <dimension ref="A1:AF54"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -1803,290 +1806,290 @@
         <v>341476</v>
       </c>
     </row>
-    <row r="26" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="11" t="s">
+    <row r="26" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A26" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="12">
-        <v>4320198</v>
-      </c>
-      <c r="C26" s="12">
+      <c r="B26" s="10">
+        <v>150000</v>
+      </c>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="8"/>
+      <c r="M26" s="8"/>
+      <c r="N26" s="8"/>
+      <c r="O26" s="8"/>
+      <c r="P26" s="8"/>
+      <c r="Q26" s="8"/>
+      <c r="R26" s="8"/>
+      <c r="S26" s="8"/>
+      <c r="T26" s="8"/>
+      <c r="U26" s="8"/>
+      <c r="V26" s="8">
+        <v>45000</v>
+      </c>
+      <c r="W26" s="8"/>
+      <c r="X26" s="8">
+        <v>75000</v>
+      </c>
+      <c r="Y26" s="8">
+        <v>30000</v>
+      </c>
+      <c r="Z26" s="8"/>
+      <c r="AA26" s="8"/>
+      <c r="AB26" s="8"/>
+      <c r="AC26" s="8"/>
+      <c r="AD26" s="8"/>
+      <c r="AE26" s="8"/>
+      <c r="AF26" s="10">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" s="12">
+        <v>4470198</v>
+      </c>
+      <c r="C27" s="12">
         <v>139012</v>
       </c>
-      <c r="D26" s="12">
+      <c r="D27" s="12">
         <v>231688</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E27" s="12">
         <v>0</v>
       </c>
-      <c r="F26" s="12">
+      <c r="F27" s="12">
         <v>0</v>
       </c>
-      <c r="G26" s="12">
+      <c r="G27" s="12">
         <v>0</v>
       </c>
-      <c r="H26" s="12">
+      <c r="H27" s="12">
         <v>0</v>
       </c>
-      <c r="I26" s="12">
+      <c r="I27" s="12">
         <v>0</v>
       </c>
-      <c r="J26" s="12">
+      <c r="J27" s="12">
         <v>0</v>
       </c>
-      <c r="K26" s="12">
+      <c r="K27" s="12">
         <v>0</v>
       </c>
-      <c r="L26" s="12">
+      <c r="L27" s="12">
         <v>0</v>
       </c>
-      <c r="M26" s="12">
+      <c r="M27" s="12">
         <v>0</v>
       </c>
-      <c r="N26" s="12">
+      <c r="N27" s="12">
         <v>0</v>
       </c>
-      <c r="O26" s="12">
+      <c r="O27" s="12">
         <v>229452</v>
       </c>
-      <c r="P26" s="12">
+      <c r="P27" s="12">
         <v>223986</v>
       </c>
-      <c r="Q26" s="12">
+      <c r="Q27" s="12">
         <v>229402</v>
       </c>
-      <c r="R26" s="12">
+      <c r="R27" s="12">
         <v>272600</v>
       </c>
-      <c r="S26" s="12">
+      <c r="S27" s="12">
         <v>337404</v>
       </c>
-      <c r="T26" s="12">
+      <c r="T27" s="12">
         <v>739676</v>
       </c>
-      <c r="U26" s="12">
+      <c r="U27" s="12">
         <v>327000</v>
       </c>
-      <c r="V26" s="12">
-        <v>303217</v>
-      </c>
-      <c r="W26" s="12">
+      <c r="V27" s="12">
+        <v>348217</v>
+      </c>
+      <c r="W27" s="12">
         <v>632991</v>
       </c>
-      <c r="X26" s="12">
-        <v>266922</v>
-      </c>
-      <c r="Y26" s="12">
-        <v>155974</v>
-      </c>
-      <c r="Z26" s="12">
+      <c r="X27" s="12">
+        <v>341922</v>
+      </c>
+      <c r="Y27" s="12">
+        <v>185974</v>
+      </c>
+      <c r="Z27" s="12">
         <v>187274</v>
       </c>
-      <c r="AA26" s="12">
+      <c r="AA27" s="12">
         <v>0</v>
       </c>
-      <c r="AB26" s="12">
+      <c r="AB27" s="12">
         <v>0</v>
       </c>
-      <c r="AC26" s="12">
+      <c r="AC27" s="12">
         <v>0</v>
       </c>
-      <c r="AD26" s="12">
+      <c r="AD27" s="12">
         <v>43600</v>
       </c>
-      <c r="AE26" s="12">
+      <c r="AE27" s="12">
         <v>0</v>
       </c>
-      <c r="AF26" s="12">
-        <v>4320198</v>
-      </c>
-    </row>
-    <row r="28" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
-      <c r="K28" s="5"/>
-      <c r="L28" s="5"/>
-      <c r="M28" s="5"/>
-      <c r="N28" s="5"/>
-      <c r="O28" s="5"/>
-      <c r="P28" s="5"/>
-      <c r="Q28" s="5"/>
-      <c r="R28" s="5"/>
-      <c r="S28" s="5"/>
-      <c r="T28" s="5"/>
-      <c r="U28" s="5"/>
-      <c r="V28" s="5"/>
-      <c r="W28" s="5"/>
-      <c r="X28" s="5"/>
-      <c r="Y28" s="5"/>
-      <c r="Z28" s="5"/>
-      <c r="AA28" s="5"/>
-      <c r="AB28" s="5"/>
-      <c r="AC28" s="5"/>
-      <c r="AD28" s="5"/>
-      <c r="AE28" s="5"/>
-      <c r="AF28" s="5"/>
-    </row>
-    <row r="29" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
+      <c r="AF27" s="12">
+        <v>4470198</v>
+      </c>
+    </row>
+    <row r="29" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="5"/>
+      <c r="O29" s="5"/>
+      <c r="P29" s="5"/>
+      <c r="Q29" s="5"/>
+      <c r="R29" s="5"/>
+      <c r="S29" s="5"/>
+      <c r="T29" s="5"/>
+      <c r="U29" s="5"/>
+      <c r="V29" s="5"/>
+      <c r="W29" s="5"/>
+      <c r="X29" s="5"/>
+      <c r="Y29" s="5"/>
+      <c r="Z29" s="5"/>
+      <c r="AA29" s="5"/>
+      <c r="AB29" s="5"/>
+      <c r="AC29" s="5"/>
+      <c r="AD29" s="5"/>
+      <c r="AE29" s="5"/>
+      <c r="AF29" s="5"/>
+    </row>
+    <row r="30" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B30" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C30" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D30" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E29" s="7" t="s">
+      <c r="E30" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="F30" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G29" s="7" t="s">
+      <c r="G30" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="H29" s="7" t="s">
+      <c r="H30" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="I29" s="7" t="s">
+      <c r="I30" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="J29" s="7" t="s">
+      <c r="J30" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K29" s="7" t="s">
+      <c r="K30" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="L29" s="7" t="s">
+      <c r="L30" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="M29" s="7" t="s">
+      <c r="M30" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="N29" s="7" t="s">
+      <c r="N30" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="O29" s="7" t="s">
+      <c r="O30" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="P29" s="7" t="s">
+      <c r="P30" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="Q29" s="7" t="s">
+      <c r="Q30" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="R29" s="7" t="s">
+      <c r="R30" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="S29" s="7" t="s">
+      <c r="S30" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="T29" s="7" t="s">
+      <c r="T30" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="U29" s="7" t="s">
+      <c r="U30" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="V29" s="7" t="s">
+      <c r="V30" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="W29" s="7" t="s">
+      <c r="W30" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="X29" s="7" t="s">
+      <c r="X30" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="Y29" s="7" t="s">
+      <c r="Y30" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="Z29" s="7" t="s">
+      <c r="Z30" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="AA29" s="7" t="s">
+      <c r="AA30" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="AB29" s="7" t="s">
+      <c r="AB30" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="AC29" s="7" t="s">
+      <c r="AC30" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="AD29" s="7" t="s">
+      <c r="AD30" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="AE29" s="7" t="s">
+      <c r="AE30" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="AF29" s="6" t="s">
+      <c r="AF30" s="6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A30" s="9" t="s">
+    <row r="31" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A31" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B30" s="10">
+      <c r="B31" s="10">
         <v>294109</v>
-      </c>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="8"/>
-      <c r="I30" s="8"/>
-      <c r="J30" s="8"/>
-      <c r="K30" s="8"/>
-      <c r="L30" s="8"/>
-      <c r="M30" s="8"/>
-      <c r="N30" s="8"/>
-      <c r="O30" s="8">
-        <v>130715</v>
-      </c>
-      <c r="P30" s="8"/>
-      <c r="Q30" s="8"/>
-      <c r="R30" s="8"/>
-      <c r="S30" s="8"/>
-      <c r="T30" s="8">
-        <v>130715</v>
-      </c>
-      <c r="U30" s="8"/>
-      <c r="V30" s="8">
-        <v>32679</v>
-      </c>
-      <c r="W30" s="8"/>
-      <c r="X30" s="8"/>
-      <c r="Y30" s="8"/>
-      <c r="Z30" s="8"/>
-      <c r="AA30" s="8"/>
-      <c r="AB30" s="8"/>
-      <c r="AC30" s="8"/>
-      <c r="AD30" s="8"/>
-      <c r="AE30" s="8"/>
-      <c r="AF30" s="10">
-        <v>294109</v>
-      </c>
-    </row>
-    <row r="31" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A31" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B31" s="10">
-        <v>409600</v>
       </c>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
@@ -2100,23 +2103,23 @@
       <c r="L31" s="8"/>
       <c r="M31" s="8"/>
       <c r="N31" s="8"/>
-      <c r="O31" s="8"/>
-      <c r="P31" s="8">
-        <v>163840</v>
-      </c>
+      <c r="O31" s="8">
+        <v>130715</v>
+      </c>
+      <c r="P31" s="8"/>
       <c r="Q31" s="8"/>
       <c r="R31" s="8"/>
       <c r="S31" s="8"/>
-      <c r="T31" s="8"/>
+      <c r="T31" s="8">
+        <v>130715</v>
+      </c>
       <c r="U31" s="8"/>
-      <c r="V31" s="8"/>
-      <c r="W31" s="8">
-        <v>163840</v>
-      </c>
+      <c r="V31" s="8">
+        <v>32679</v>
+      </c>
+      <c r="W31" s="8"/>
       <c r="X31" s="8"/>
-      <c r="Y31" s="8">
-        <v>81920</v>
-      </c>
+      <c r="Y31" s="8"/>
       <c r="Z31" s="8"/>
       <c r="AA31" s="8"/>
       <c r="AB31" s="8"/>
@@ -2124,15 +2127,15 @@
       <c r="AD31" s="8"/>
       <c r="AE31" s="8"/>
       <c r="AF31" s="10">
+        <v>294109</v>
+      </c>
+    </row>
+    <row r="32" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A32" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" s="10">
         <v>409600</v>
-      </c>
-    </row>
-    <row r="32" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
-      <c r="A32" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B32" s="10">
-        <v>576318</v>
       </c>
       <c r="C32" s="8"/>
       <c r="D32" s="8"/>
@@ -2146,23 +2149,23 @@
       <c r="L32" s="8"/>
       <c r="M32" s="8"/>
       <c r="N32" s="8"/>
-      <c r="O32" s="8">
-        <v>230527</v>
-      </c>
+      <c r="O32" s="8"/>
       <c r="P32" s="8">
-        <v>230527</v>
+        <v>163840</v>
       </c>
       <c r="Q32" s="8"/>
       <c r="R32" s="8"/>
       <c r="S32" s="8"/>
-      <c r="T32" s="8">
-        <v>115264</v>
-      </c>
+      <c r="T32" s="8"/>
       <c r="U32" s="8"/>
       <c r="V32" s="8"/>
-      <c r="W32" s="8"/>
+      <c r="W32" s="8">
+        <v>163840</v>
+      </c>
       <c r="X32" s="8"/>
-      <c r="Y32" s="8"/>
+      <c r="Y32" s="8">
+        <v>81920</v>
+      </c>
       <c r="Z32" s="8"/>
       <c r="AA32" s="8"/>
       <c r="AB32" s="8"/>
@@ -2170,15 +2173,15 @@
       <c r="AD32" s="8"/>
       <c r="AE32" s="8"/>
       <c r="AF32" s="10">
+        <v>409600</v>
+      </c>
+    </row>
+    <row r="33" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A33" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B33" s="10">
         <v>576318</v>
-      </c>
-    </row>
-    <row r="33" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A33" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B33" s="10">
-        <v>322960</v>
       </c>
       <c r="C33" s="8"/>
       <c r="D33" s="8"/>
@@ -2192,16 +2195,18 @@
       <c r="L33" s="8"/>
       <c r="M33" s="8"/>
       <c r="N33" s="8"/>
-      <c r="O33" s="8"/>
-      <c r="P33" s="8"/>
+      <c r="O33" s="8">
+        <v>230527</v>
+      </c>
+      <c r="P33" s="8">
+        <v>230527</v>
+      </c>
       <c r="Q33" s="8"/>
-      <c r="R33" s="8">
-        <v>129184</v>
-      </c>
-      <c r="S33" s="8">
-        <v>193776</v>
-      </c>
-      <c r="T33" s="8"/>
+      <c r="R33" s="8"/>
+      <c r="S33" s="8"/>
+      <c r="T33" s="8">
+        <v>115264</v>
+      </c>
       <c r="U33" s="8"/>
       <c r="V33" s="8"/>
       <c r="W33" s="8"/>
@@ -2214,15 +2219,15 @@
       <c r="AD33" s="8"/>
       <c r="AE33" s="8"/>
       <c r="AF33" s="10">
+        <v>576318</v>
+      </c>
+    </row>
+    <row r="34" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A34" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B34" s="10">
         <v>322960</v>
-      </c>
-    </row>
-    <row r="34" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
-      <c r="A34" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B34" s="10">
-        <v>252248</v>
       </c>
       <c r="C34" s="8"/>
       <c r="D34" s="8"/>
@@ -2239,16 +2244,18 @@
       <c r="O34" s="8"/>
       <c r="P34" s="8"/>
       <c r="Q34" s="8"/>
-      <c r="R34" s="8"/>
-      <c r="S34" s="8"/>
+      <c r="R34" s="8">
+        <v>129184</v>
+      </c>
+      <c r="S34" s="8">
+        <v>193776</v>
+      </c>
       <c r="T34" s="8"/>
       <c r="U34" s="8"/>
       <c r="V34" s="8"/>
       <c r="W34" s="8"/>
       <c r="X34" s="8"/>
-      <c r="Y34" s="8">
-        <v>252248</v>
-      </c>
+      <c r="Y34" s="8"/>
       <c r="Z34" s="8"/>
       <c r="AA34" s="8"/>
       <c r="AB34" s="8"/>
@@ -2256,15 +2263,15 @@
       <c r="AD34" s="8"/>
       <c r="AE34" s="8"/>
       <c r="AF34" s="10">
-        <v>252248</v>
+        <v>322960</v>
       </c>
     </row>
     <row r="35" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B35" s="10">
-        <v>338450</v>
+        <v>252248</v>
       </c>
       <c r="C35" s="8"/>
       <c r="D35" s="8"/>
@@ -2281,20 +2288,16 @@
       <c r="O35" s="8"/>
       <c r="P35" s="8"/>
       <c r="Q35" s="8"/>
-      <c r="R35" s="8">
-        <v>135380</v>
-      </c>
-      <c r="S35" s="8">
-        <v>135380</v>
-      </c>
-      <c r="T35" s="8">
-        <v>67690</v>
-      </c>
+      <c r="R35" s="8"/>
+      <c r="S35" s="8"/>
+      <c r="T35" s="8"/>
       <c r="U35" s="8"/>
       <c r="V35" s="8"/>
       <c r="W35" s="8"/>
       <c r="X35" s="8"/>
-      <c r="Y35" s="8"/>
+      <c r="Y35" s="8">
+        <v>252248</v>
+      </c>
       <c r="Z35" s="8"/>
       <c r="AA35" s="8"/>
       <c r="AB35" s="8"/>
@@ -2302,15 +2305,15 @@
       <c r="AD35" s="8"/>
       <c r="AE35" s="8"/>
       <c r="AF35" s="10">
+        <v>252248</v>
+      </c>
+    </row>
+    <row r="36" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A36" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B36" s="10">
         <v>338450</v>
-      </c>
-    </row>
-    <row r="36" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A36" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B36" s="10">
-        <v>1156110</v>
       </c>
       <c r="C36" s="8"/>
       <c r="D36" s="8"/>
@@ -2328,17 +2331,17 @@
       <c r="P36" s="8"/>
       <c r="Q36" s="8"/>
       <c r="R36" s="8">
-        <v>462444</v>
-      </c>
-      <c r="S36" s="8"/>
+        <v>135380</v>
+      </c>
+      <c r="S36" s="8">
+        <v>135380</v>
+      </c>
       <c r="T36" s="8">
-        <v>346833</v>
+        <v>67690</v>
       </c>
       <c r="U36" s="8"/>
       <c r="V36" s="8"/>
-      <c r="W36" s="8">
-        <v>346833</v>
-      </c>
+      <c r="W36" s="8"/>
       <c r="X36" s="8"/>
       <c r="Y36" s="8"/>
       <c r="Z36" s="8"/>
@@ -2348,15 +2351,15 @@
       <c r="AD36" s="8"/>
       <c r="AE36" s="8"/>
       <c r="AF36" s="10">
+        <v>338450</v>
+      </c>
+    </row>
+    <row r="37" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A37" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B37" s="10">
         <v>1156110</v>
-      </c>
-    </row>
-    <row r="37" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
-      <c r="A37" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B37" s="10">
-        <v>594115</v>
       </c>
       <c r="C37" s="8"/>
       <c r="D37" s="8"/>
@@ -2373,36 +2376,36 @@
       <c r="O37" s="8"/>
       <c r="P37" s="8"/>
       <c r="Q37" s="8"/>
-      <c r="R37" s="8"/>
+      <c r="R37" s="8">
+        <v>462444</v>
+      </c>
       <c r="S37" s="8"/>
-      <c r="T37" s="8"/>
+      <c r="T37" s="8">
+        <v>346833</v>
+      </c>
       <c r="U37" s="8"/>
       <c r="V37" s="8"/>
-      <c r="W37" s="8"/>
+      <c r="W37" s="8">
+        <v>346833</v>
+      </c>
       <c r="X37" s="8"/>
-      <c r="Y37" s="8">
-        <v>237646</v>
-      </c>
-      <c r="Z37" s="8">
-        <v>237646</v>
-      </c>
-      <c r="AA37" s="8">
-        <v>118823</v>
-      </c>
+      <c r="Y37" s="8"/>
+      <c r="Z37" s="8"/>
+      <c r="AA37" s="8"/>
       <c r="AB37" s="8"/>
       <c r="AC37" s="8"/>
       <c r="AD37" s="8"/>
       <c r="AE37" s="8"/>
       <c r="AF37" s="10">
+        <v>1156110</v>
+      </c>
+    </row>
+    <row r="38" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A38" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B38" s="10">
         <v>594115</v>
-      </c>
-    </row>
-    <row r="38" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A38" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B38" s="10">
-        <v>327103</v>
       </c>
       <c r="C38" s="8"/>
       <c r="D38" s="8"/>
@@ -2419,36 +2422,36 @@
       <c r="O38" s="8"/>
       <c r="P38" s="8"/>
       <c r="Q38" s="8"/>
-      <c r="R38" s="8">
-        <v>130841</v>
-      </c>
+      <c r="R38" s="8"/>
       <c r="S38" s="8"/>
       <c r="T38" s="8"/>
       <c r="U38" s="8"/>
       <c r="V38" s="8"/>
-      <c r="W38" s="8">
-        <v>130841</v>
-      </c>
+      <c r="W38" s="8"/>
       <c r="X38" s="8"/>
-      <c r="Y38" s="8"/>
-      <c r="Z38" s="8"/>
+      <c r="Y38" s="8">
+        <v>237646</v>
+      </c>
+      <c r="Z38" s="8">
+        <v>237646</v>
+      </c>
       <c r="AA38" s="8">
-        <v>65421</v>
+        <v>118823</v>
       </c>
       <c r="AB38" s="8"/>
       <c r="AC38" s="8"/>
       <c r="AD38" s="8"/>
       <c r="AE38" s="8"/>
       <c r="AF38" s="10">
+        <v>594115</v>
+      </c>
+    </row>
+    <row r="39" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A39" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B39" s="10">
         <v>327103</v>
-      </c>
-    </row>
-    <row r="39" spans="1:32" ht="69" x14ac:dyDescent="0.25">
-      <c r="A39" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="B39" s="10">
-        <v>1707090</v>
       </c>
       <c r="C39" s="8"/>
       <c r="D39" s="8"/>
@@ -2465,36 +2468,36 @@
       <c r="O39" s="8"/>
       <c r="P39" s="8"/>
       <c r="Q39" s="8"/>
-      <c r="R39" s="8"/>
-      <c r="S39" s="8">
-        <v>682836</v>
-      </c>
-      <c r="T39" s="8">
-        <v>682836</v>
-      </c>
-      <c r="U39" s="8">
-        <v>341418</v>
-      </c>
+      <c r="R39" s="8">
+        <v>130841</v>
+      </c>
+      <c r="S39" s="8"/>
+      <c r="T39" s="8"/>
+      <c r="U39" s="8"/>
       <c r="V39" s="8"/>
-      <c r="W39" s="8"/>
+      <c r="W39" s="8">
+        <v>130841</v>
+      </c>
       <c r="X39" s="8"/>
       <c r="Y39" s="8"/>
       <c r="Z39" s="8"/>
-      <c r="AA39" s="8"/>
+      <c r="AA39" s="8">
+        <v>65421</v>
+      </c>
       <c r="AB39" s="8"/>
       <c r="AC39" s="8"/>
       <c r="AD39" s="8"/>
       <c r="AE39" s="8"/>
       <c r="AF39" s="10">
-        <v>1707090</v>
+        <v>327103</v>
       </c>
     </row>
     <row r="40" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B40" s="10">
-        <v>80000</v>
+        <v>1707090</v>
       </c>
       <c r="C40" s="8"/>
       <c r="D40" s="8"/>
@@ -2511,14 +2514,16 @@
       <c r="O40" s="8"/>
       <c r="P40" s="8"/>
       <c r="Q40" s="8"/>
-      <c r="R40" s="8">
-        <v>32000</v>
-      </c>
+      <c r="R40" s="8"/>
       <c r="S40" s="8">
-        <v>48000</v>
-      </c>
-      <c r="T40" s="8"/>
-      <c r="U40" s="8"/>
+        <v>682836</v>
+      </c>
+      <c r="T40" s="8">
+        <v>682836</v>
+      </c>
+      <c r="U40" s="8">
+        <v>341418</v>
+      </c>
       <c r="V40" s="8"/>
       <c r="W40" s="8"/>
       <c r="X40" s="8"/>
@@ -2530,15 +2535,15 @@
       <c r="AD40" s="8"/>
       <c r="AE40" s="8"/>
       <c r="AF40" s="10">
-        <v>80000</v>
+        <v>1707090</v>
       </c>
     </row>
     <row r="41" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B41" s="10">
-        <v>1199960</v>
+        <v>80000</v>
       </c>
       <c r="C41" s="8"/>
       <c r="D41" s="8"/>
@@ -2555,36 +2560,34 @@
       <c r="O41" s="8"/>
       <c r="P41" s="8"/>
       <c r="Q41" s="8"/>
-      <c r="R41" s="8"/>
+      <c r="R41" s="8">
+        <v>32000</v>
+      </c>
       <c r="S41" s="8">
-        <v>479984</v>
+        <v>48000</v>
       </c>
       <c r="T41" s="8"/>
       <c r="U41" s="8"/>
       <c r="V41" s="8"/>
-      <c r="W41" s="8">
-        <v>479984</v>
-      </c>
+      <c r="W41" s="8"/>
       <c r="X41" s="8"/>
       <c r="Y41" s="8"/>
-      <c r="Z41" s="8">
-        <v>239992</v>
-      </c>
+      <c r="Z41" s="8"/>
       <c r="AA41" s="8"/>
       <c r="AB41" s="8"/>
       <c r="AC41" s="8"/>
       <c r="AD41" s="8"/>
       <c r="AE41" s="8"/>
       <c r="AF41" s="10">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+      <c r="A42" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B42" s="10">
         <v>1199960</v>
-      </c>
-    </row>
-    <row r="42" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
-      <c r="A42" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B42" s="10">
-        <v>600000</v>
       </c>
       <c r="C42" s="8"/>
       <c r="D42" s="8"/>
@@ -2598,39 +2601,39 @@
       <c r="L42" s="8"/>
       <c r="M42" s="8"/>
       <c r="N42" s="8"/>
-      <c r="O42" s="8">
-        <v>240000</v>
-      </c>
+      <c r="O42" s="8"/>
       <c r="P42" s="8"/>
-      <c r="Q42" s="8">
-        <v>180000</v>
-      </c>
-      <c r="R42" s="8">
-        <v>180000</v>
-      </c>
-      <c r="S42" s="8"/>
+      <c r="Q42" s="8"/>
+      <c r="R42" s="8"/>
+      <c r="S42" s="8">
+        <v>479984</v>
+      </c>
       <c r="T42" s="8"/>
       <c r="U42" s="8"/>
       <c r="V42" s="8"/>
-      <c r="W42" s="8"/>
+      <c r="W42" s="8">
+        <v>479984</v>
+      </c>
       <c r="X42" s="8"/>
       <c r="Y42" s="8"/>
-      <c r="Z42" s="8"/>
+      <c r="Z42" s="8">
+        <v>239992</v>
+      </c>
       <c r="AA42" s="8"/>
       <c r="AB42" s="8"/>
       <c r="AC42" s="8"/>
       <c r="AD42" s="8"/>
       <c r="AE42" s="8"/>
       <c r="AF42" s="10">
+        <v>1199960</v>
+      </c>
+    </row>
+    <row r="43" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A43" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B43" s="10">
         <v>600000</v>
-      </c>
-    </row>
-    <row r="43" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A43" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B43" s="10">
-        <v>317648</v>
       </c>
       <c r="C43" s="8"/>
       <c r="D43" s="8"/>
@@ -2645,14 +2648,14 @@
       <c r="M43" s="8"/>
       <c r="N43" s="8"/>
       <c r="O43" s="8">
-        <v>127059</v>
-      </c>
-      <c r="P43" s="8">
-        <v>127059</v>
-      </c>
-      <c r="Q43" s="8"/>
+        <v>240000</v>
+      </c>
+      <c r="P43" s="8"/>
+      <c r="Q43" s="8">
+        <v>180000</v>
+      </c>
       <c r="R43" s="8">
-        <v>63530</v>
+        <v>180000</v>
       </c>
       <c r="S43" s="8"/>
       <c r="T43" s="8"/>
@@ -2668,15 +2671,15 @@
       <c r="AD43" s="8"/>
       <c r="AE43" s="8"/>
       <c r="AF43" s="10">
+        <v>600000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A44" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B44" s="10">
         <v>317648</v>
-      </c>
-    </row>
-    <row r="44" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A44" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B44" s="10">
-        <v>832813</v>
       </c>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -2690,23 +2693,23 @@
       <c r="L44" s="8"/>
       <c r="M44" s="8"/>
       <c r="N44" s="8"/>
-      <c r="O44" s="8"/>
-      <c r="P44" s="8"/>
+      <c r="O44" s="8">
+        <v>127059</v>
+      </c>
+      <c r="P44" s="8">
+        <v>127059</v>
+      </c>
       <c r="Q44" s="8"/>
-      <c r="R44" s="8"/>
+      <c r="R44" s="8">
+        <v>63530</v>
+      </c>
       <c r="S44" s="8"/>
-      <c r="T44" s="8">
-        <v>333125</v>
-      </c>
-      <c r="U44" s="8">
-        <v>249844</v>
-      </c>
+      <c r="T44" s="8"/>
+      <c r="U44" s="8"/>
       <c r="V44" s="8"/>
       <c r="W44" s="8"/>
       <c r="X44" s="8"/>
-      <c r="Y44" s="8">
-        <v>249844</v>
-      </c>
+      <c r="Y44" s="8"/>
       <c r="Z44" s="8"/>
       <c r="AA44" s="8"/>
       <c r="AB44" s="8"/>
@@ -2714,22 +2717,18 @@
       <c r="AD44" s="8"/>
       <c r="AE44" s="8"/>
       <c r="AF44" s="10">
+        <v>317648</v>
+      </c>
+    </row>
+    <row r="45" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A45" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B45" s="10">
         <v>832813</v>
       </c>
-    </row>
-    <row r="45" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A45" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="B45" s="10">
-        <v>341237</v>
-      </c>
-      <c r="C45" s="8">
-        <v>136495</v>
-      </c>
-      <c r="D45" s="8">
-        <v>136495</v>
-      </c>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
       <c r="E45" s="8"/>
       <c r="F45" s="8"/>
       <c r="G45" s="8"/>
@@ -2745,14 +2744,18 @@
       <c r="Q45" s="8"/>
       <c r="R45" s="8"/>
       <c r="S45" s="8"/>
-      <c r="T45" s="8"/>
-      <c r="U45" s="8"/>
-      <c r="V45" s="8">
-        <v>68247</v>
-      </c>
+      <c r="T45" s="8">
+        <v>333125</v>
+      </c>
+      <c r="U45" s="8">
+        <v>249844</v>
+      </c>
+      <c r="V45" s="8"/>
       <c r="W45" s="8"/>
       <c r="X45" s="8"/>
-      <c r="Y45" s="8"/>
+      <c r="Y45" s="8">
+        <v>249844</v>
+      </c>
       <c r="Z45" s="8"/>
       <c r="AA45" s="8"/>
       <c r="AB45" s="8"/>
@@ -2760,21 +2763,21 @@
       <c r="AD45" s="8"/>
       <c r="AE45" s="8"/>
       <c r="AF45" s="10">
+        <v>832813</v>
+      </c>
+    </row>
+    <row r="46" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A46" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B46" s="10">
         <v>341237</v>
       </c>
-    </row>
-    <row r="46" spans="1:32" ht="69" x14ac:dyDescent="0.25">
-      <c r="A46" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="B46" s="10">
-        <v>666700</v>
-      </c>
       <c r="C46" s="8">
-        <v>266680</v>
+        <v>136495</v>
       </c>
       <c r="D46" s="8">
-        <v>266680</v>
+        <v>136495</v>
       </c>
       <c r="E46" s="8"/>
       <c r="F46" s="8"/>
@@ -2793,10 +2796,10 @@
       <c r="S46" s="8"/>
       <c r="T46" s="8"/>
       <c r="U46" s="8"/>
-      <c r="V46" s="8"/>
-      <c r="W46" s="8">
-        <v>133340</v>
-      </c>
+      <c r="V46" s="8">
+        <v>68247</v>
+      </c>
+      <c r="W46" s="8"/>
       <c r="X46" s="8"/>
       <c r="Y46" s="8"/>
       <c r="Z46" s="8"/>
@@ -2806,18 +2809,22 @@
       <c r="AD46" s="8"/>
       <c r="AE46" s="8"/>
       <c r="AF46" s="10">
+        <v>341237</v>
+      </c>
+    </row>
+    <row r="47" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+      <c r="A47" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B47" s="10">
         <v>666700</v>
       </c>
-    </row>
-    <row r="47" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A47" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="B47" s="10">
-        <v>460000</v>
-      </c>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
+      <c r="C47" s="8">
+        <v>266680</v>
+      </c>
+      <c r="D47" s="8">
+        <v>266680</v>
+      </c>
       <c r="E47" s="8"/>
       <c r="F47" s="8"/>
       <c r="G47" s="8"/>
@@ -2833,13 +2840,11 @@
       <c r="Q47" s="8"/>
       <c r="R47" s="8"/>
       <c r="S47" s="8"/>
-      <c r="T47" s="8">
-        <v>184000</v>
-      </c>
+      <c r="T47" s="8"/>
       <c r="U47" s="8"/>
       <c r="V47" s="8"/>
       <c r="W47" s="8">
-        <v>184000</v>
+        <v>133340</v>
       </c>
       <c r="X47" s="8"/>
       <c r="Y47" s="8"/>
@@ -2848,19 +2853,17 @@
       <c r="AB47" s="8"/>
       <c r="AC47" s="8"/>
       <c r="AD47" s="8"/>
-      <c r="AE47" s="8">
-        <v>92000</v>
-      </c>
+      <c r="AE47" s="8"/>
       <c r="AF47" s="10">
-        <v>460000</v>
+        <v>666700</v>
       </c>
     </row>
     <row r="48" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B48" s="10">
-        <v>206880</v>
+        <v>460000</v>
       </c>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
@@ -2880,13 +2883,13 @@
       <c r="R48" s="8"/>
       <c r="S48" s="8"/>
       <c r="T48" s="8">
-        <v>82752</v>
-      </c>
-      <c r="U48" s="8">
-        <v>124128</v>
-      </c>
+        <v>184000</v>
+      </c>
+      <c r="U48" s="8"/>
       <c r="V48" s="8"/>
-      <c r="W48" s="8"/>
+      <c r="W48" s="8">
+        <v>184000</v>
+      </c>
       <c r="X48" s="8"/>
       <c r="Y48" s="8"/>
       <c r="Z48" s="8"/>
@@ -2894,17 +2897,19 @@
       <c r="AB48" s="8"/>
       <c r="AC48" s="8"/>
       <c r="AD48" s="8"/>
-      <c r="AE48" s="8"/>
+      <c r="AE48" s="8">
+        <v>92000</v>
+      </c>
       <c r="AF48" s="10">
+        <v>460000</v>
+      </c>
+    </row>
+    <row r="49" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A49" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B49" s="10">
         <v>206880</v>
-      </c>
-    </row>
-    <row r="49" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A49" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B49" s="10">
-        <v>799875</v>
       </c>
       <c r="C49" s="8"/>
       <c r="D49" s="8"/>
@@ -2923,169 +2928,257 @@
       <c r="Q49" s="8"/>
       <c r="R49" s="8"/>
       <c r="S49" s="8"/>
-      <c r="T49" s="8"/>
+      <c r="T49" s="8">
+        <v>82752</v>
+      </c>
       <c r="U49" s="8">
-        <v>319950</v>
+        <v>124128</v>
       </c>
       <c r="V49" s="8"/>
       <c r="W49" s="8"/>
-      <c r="X49" s="8">
-        <v>319950</v>
-      </c>
+      <c r="X49" s="8"/>
       <c r="Y49" s="8"/>
       <c r="Z49" s="8"/>
       <c r="AA49" s="8"/>
-      <c r="AB49" s="8">
-        <v>159975</v>
-      </c>
+      <c r="AB49" s="8"/>
       <c r="AC49" s="8"/>
       <c r="AD49" s="8"/>
       <c r="AE49" s="8"/>
       <c r="AF49" s="10">
+        <v>206880</v>
+      </c>
+    </row>
+    <row r="50" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A50" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B50" s="10">
         <v>799875</v>
       </c>
-    </row>
-    <row r="50" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="11" t="s">
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="8"/>
+      <c r="G50" s="8"/>
+      <c r="H50" s="8"/>
+      <c r="I50" s="8"/>
+      <c r="J50" s="8"/>
+      <c r="K50" s="8"/>
+      <c r="L50" s="8"/>
+      <c r="M50" s="8"/>
+      <c r="N50" s="8"/>
+      <c r="O50" s="8"/>
+      <c r="P50" s="8"/>
+      <c r="Q50" s="8"/>
+      <c r="R50" s="8"/>
+      <c r="S50" s="8"/>
+      <c r="T50" s="8"/>
+      <c r="U50" s="8">
+        <v>319950</v>
+      </c>
+      <c r="V50" s="8"/>
+      <c r="W50" s="8"/>
+      <c r="X50" s="8">
+        <v>319950</v>
+      </c>
+      <c r="Y50" s="8"/>
+      <c r="Z50" s="8"/>
+      <c r="AA50" s="8"/>
+      <c r="AB50" s="8">
+        <v>159975</v>
+      </c>
+      <c r="AC50" s="8"/>
+      <c r="AD50" s="8"/>
+      <c r="AE50" s="8"/>
+      <c r="AF50" s="10">
+        <v>799875</v>
+      </c>
+    </row>
+    <row r="51" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A51" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B50" s="12">
-        <v>11483216</v>
-      </c>
-      <c r="C50" s="12">
+      <c r="B51" s="10">
+        <v>90000</v>
+      </c>
+      <c r="C51" s="8"/>
+      <c r="D51" s="8"/>
+      <c r="E51" s="8"/>
+      <c r="F51" s="8"/>
+      <c r="G51" s="8"/>
+      <c r="H51" s="8"/>
+      <c r="I51" s="8"/>
+      <c r="J51" s="8"/>
+      <c r="K51" s="8"/>
+      <c r="L51" s="8"/>
+      <c r="M51" s="8"/>
+      <c r="N51" s="8"/>
+      <c r="O51" s="8"/>
+      <c r="P51" s="8"/>
+      <c r="Q51" s="8"/>
+      <c r="R51" s="8"/>
+      <c r="S51" s="8"/>
+      <c r="T51" s="8"/>
+      <c r="U51" s="8"/>
+      <c r="V51" s="8"/>
+      <c r="W51" s="8"/>
+      <c r="X51" s="8">
+        <v>60000</v>
+      </c>
+      <c r="Y51" s="8">
+        <v>30000</v>
+      </c>
+      <c r="Z51" s="8"/>
+      <c r="AA51" s="8"/>
+      <c r="AB51" s="8"/>
+      <c r="AC51" s="8"/>
+      <c r="AD51" s="8"/>
+      <c r="AE51" s="8"/>
+      <c r="AF51" s="10">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B52" s="12">
+        <v>11573216</v>
+      </c>
+      <c r="C52" s="12">
         <v>403175</v>
       </c>
-      <c r="D50" s="12">
+      <c r="D52" s="12">
         <v>403175</v>
       </c>
-      <c r="E50" s="12">
+      <c r="E52" s="12">
         <v>0</v>
       </c>
-      <c r="F50" s="12">
+      <c r="F52" s="12">
         <v>0</v>
       </c>
-      <c r="G50" s="12">
+      <c r="G52" s="12">
         <v>0</v>
       </c>
-      <c r="H50" s="12">
+      <c r="H52" s="12">
         <v>0</v>
       </c>
-      <c r="I50" s="12">
+      <c r="I52" s="12">
         <v>0</v>
       </c>
-      <c r="J50" s="12">
+      <c r="J52" s="12">
         <v>0</v>
       </c>
-      <c r="K50" s="12">
+      <c r="K52" s="12">
         <v>0</v>
       </c>
-      <c r="L50" s="12">
+      <c r="L52" s="12">
         <v>0</v>
       </c>
-      <c r="M50" s="12">
+      <c r="M52" s="12">
         <v>0</v>
       </c>
-      <c r="N50" s="12">
+      <c r="N52" s="12">
         <v>0</v>
       </c>
-      <c r="O50" s="12">
+      <c r="O52" s="12">
         <v>728301</v>
       </c>
-      <c r="P50" s="12">
+      <c r="P52" s="12">
         <v>521426</v>
       </c>
-      <c r="Q50" s="12">
+      <c r="Q52" s="12">
         <v>180000</v>
       </c>
-      <c r="R50" s="12">
+      <c r="R52" s="12">
         <v>1133379</v>
       </c>
-      <c r="S50" s="12">
+      <c r="S52" s="12">
         <v>1539976</v>
       </c>
-      <c r="T50" s="12">
+      <c r="T52" s="12">
         <v>1943215</v>
       </c>
-      <c r="U50" s="12">
+      <c r="U52" s="12">
         <v>1035340</v>
       </c>
-      <c r="V50" s="12">
+      <c r="V52" s="12">
         <v>100926</v>
       </c>
-      <c r="W50" s="12">
+      <c r="W52" s="12">
         <v>1438838</v>
       </c>
-      <c r="X50" s="12">
-        <v>319950</v>
-      </c>
-      <c r="Y50" s="12">
-        <v>821658</v>
-      </c>
-      <c r="Z50" s="12">
+      <c r="X52" s="12">
+        <v>379950</v>
+      </c>
+      <c r="Y52" s="12">
+        <v>851658</v>
+      </c>
+      <c r="Z52" s="12">
         <v>477638</v>
       </c>
-      <c r="AA50" s="12">
+      <c r="AA52" s="12">
         <v>184244</v>
       </c>
-      <c r="AB50" s="12">
+      <c r="AB52" s="12">
         <v>159975</v>
       </c>
-      <c r="AC50" s="12">
+      <c r="AC52" s="12">
         <v>0</v>
       </c>
-      <c r="AD50" s="12">
+      <c r="AD52" s="12">
         <v>0</v>
       </c>
-      <c r="AE50" s="12">
+      <c r="AE52" s="12">
         <v>92000</v>
       </c>
-      <c r="AF50" s="12">
-        <v>11483216</v>
-      </c>
-    </row>
-    <row r="52" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A52" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B52" s="4"/>
-      <c r="C52" s="4"/>
-      <c r="D52" s="4"/>
-      <c r="E52" s="4"/>
-      <c r="F52" s="4"/>
-      <c r="G52" s="4"/>
-      <c r="H52" s="4"/>
-      <c r="I52" s="4"/>
-      <c r="J52" s="4"/>
-      <c r="K52" s="4"/>
-      <c r="L52" s="4"/>
-      <c r="M52" s="4"/>
-      <c r="N52" s="4"/>
-      <c r="O52" s="4"/>
-      <c r="P52" s="4"/>
-      <c r="Q52" s="4"/>
-      <c r="R52" s="4"/>
-      <c r="S52" s="4"/>
-      <c r="T52" s="4"/>
-      <c r="U52" s="4"/>
-      <c r="V52" s="4"/>
-      <c r="W52" s="4"/>
-      <c r="X52" s="4"/>
-      <c r="Y52" s="4"/>
-      <c r="Z52" s="4"/>
-      <c r="AA52" s="4"/>
-      <c r="AB52" s="4"/>
-      <c r="AC52" s="4"/>
-      <c r="AD52" s="4"/>
-      <c r="AE52" s="4"/>
-      <c r="AF52" s="4"/>
+      <c r="AF52" s="12">
+        <v>11573216</v>
+      </c>
+    </row>
+    <row r="54" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A54" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B54" s="4"/>
+      <c r="C54" s="4"/>
+      <c r="D54" s="4"/>
+      <c r="E54" s="4"/>
+      <c r="F54" s="4"/>
+      <c r="G54" s="4"/>
+      <c r="H54" s="4"/>
+      <c r="I54" s="4"/>
+      <c r="J54" s="4"/>
+      <c r="K54" s="4"/>
+      <c r="L54" s="4"/>
+      <c r="M54" s="4"/>
+      <c r="N54" s="4"/>
+      <c r="O54" s="4"/>
+      <c r="P54" s="4"/>
+      <c r="Q54" s="4"/>
+      <c r="R54" s="4"/>
+      <c r="S54" s="4"/>
+      <c r="T54" s="4"/>
+      <c r="U54" s="4"/>
+      <c r="V54" s="4"/>
+      <c r="W54" s="4"/>
+      <c r="X54" s="4"/>
+      <c r="Y54" s="4"/>
+      <c r="Z54" s="4"/>
+      <c r="AA54" s="4"/>
+      <c r="AB54" s="4"/>
+      <c r="AC54" s="4"/>
+      <c r="AD54" s="4"/>
+      <c r="AE54" s="4"/>
+      <c r="AF54" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:AF1"/>
     <mergeCell ref="A2:AF2"/>
-    <mergeCell ref="A52:AF52"/>
+    <mergeCell ref="A54:AF54"/>
     <mergeCell ref="A4:AF4"/>
-    <mergeCell ref="A28:AF28"/>
+    <mergeCell ref="A29:AF29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-31 11:29)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3182,4 +3182,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66CE3646-F9E9-4CC5-A950-F87C7931A56F}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E83CFD3-E86A-4BA7-9CE9-68BB919C9E97}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{000FA856-18B7-4B43-BE15-3F39206A1C1E}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-31 11:30)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{05B320A9-604F-4C76-A34B-75425A592C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B741E600-D1BE-4B34-9914-D18B0861021A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5928" yWindow="1668" windowWidth="14328" windowHeight="8880" xr2:uid="{72E01C85-E361-44C9-8AD2-133DCDFE32D3}"/>
+    <workbookView xWindow="5928" yWindow="1668" windowWidth="14328" windowHeight="8880" xr2:uid="{55B16079-8584-4218-B88F-88DC2BC55089}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -697,7 +697,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33AF483C-E886-4AE5-A452-03ABB9A8EEE3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE378DB2-06AE-4436-94EC-ACC152A141B3}">
   <dimension ref="A1:AF54"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3182,291 +3182,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66CE3646-F9E9-4CC5-A950-F87C7931A56F}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E83CFD3-E86A-4BA7-9CE9-68BB919C9E97}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{000FA856-18B7-4B43-BE15-3F39206A1C1E}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-31 12:45)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B741E600-D1BE-4B34-9914-D18B0861021A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{95FE187B-A00B-4B4E-86E1-3C87BBFD84E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5928" yWindow="1668" windowWidth="14328" windowHeight="8880" xr2:uid="{55B16079-8584-4218-B88F-88DC2BC55089}"/>
+    <workbookView xWindow="5928" yWindow="1668" windowWidth="14328" windowHeight="8880" xr2:uid="{AB752406-8B3B-4036-9024-01162D5DB5F6}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -697,7 +697,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE378DB2-06AE-4436-94EC-ACC152A141B3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C37B002E-48DB-4E51-865F-FC75F1568645}">
   <dimension ref="A1:AF54"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-08-31 15:16)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{95FE187B-A00B-4B4E-86E1-3C87BBFD84E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2A04DA36-7751-4EED-973E-4847AE91752F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5928" yWindow="1668" windowWidth="14328" windowHeight="8880" xr2:uid="{AB752406-8B3B-4036-9024-01162D5DB5F6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BA7519A2-7C5A-4CBC-AEC3-1316AFEA11D2}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -697,7 +697,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C37B002E-48DB-4E51-865F-FC75F1568645}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8D17305-615C-49B5-93FD-046059799B11}">
   <dimension ref="A1:AF54"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-01 10:40)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2A04DA36-7751-4EED-973E-4847AE91752F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1DEB5BF-F58E-4021-BB44-BFFAC07129F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BA7519A2-7C5A-4CBC-AEC3-1316AFEA11D2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FEA4C1C6-CFA0-44A7-B899-252118432047}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (21 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-08-31</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-01</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -697,7 +697,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8D17305-615C-49B5-93FD-046059799B11}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41489AD5-1A53-4044-8A42-4C4B2CCF02E3}">
   <dimension ref="A1:AF54"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1811,7 +1811,7 @@
         <v>55</v>
       </c>
       <c r="B26" s="10">
-        <v>150000</v>
+        <v>164242</v>
       </c>
       <c r="C26" s="8"/>
       <c r="D26" s="8"/>
@@ -1833,15 +1833,15 @@
       <c r="T26" s="8"/>
       <c r="U26" s="8"/>
       <c r="V26" s="8">
-        <v>45000</v>
-      </c>
-      <c r="W26" s="8"/>
+        <v>50341</v>
+      </c>
+      <c r="W26" s="8">
+        <v>83901</v>
+      </c>
       <c r="X26" s="8">
-        <v>75000</v>
-      </c>
-      <c r="Y26" s="8">
         <v>30000</v>
       </c>
+      <c r="Y26" s="8"/>
       <c r="Z26" s="8"/>
       <c r="AA26" s="8"/>
       <c r="AB26" s="8"/>
@@ -1849,7 +1849,7 @@
       <c r="AD26" s="8"/>
       <c r="AE26" s="8"/>
       <c r="AF26" s="10">
-        <v>150000</v>
+        <v>164242</v>
       </c>
     </row>
     <row r="27" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1857,7 +1857,7 @@
         <v>56</v>
       </c>
       <c r="B27" s="12">
-        <v>4470198</v>
+        <v>4484440</v>
       </c>
       <c r="C27" s="12">
         <v>139012</v>
@@ -1917,16 +1917,16 @@
         <v>327000</v>
       </c>
       <c r="V27" s="12">
-        <v>348217</v>
+        <v>353558</v>
       </c>
       <c r="W27" s="12">
-        <v>632991</v>
+        <v>716892</v>
       </c>
       <c r="X27" s="12">
-        <v>341922</v>
+        <v>296922</v>
       </c>
       <c r="Y27" s="12">
-        <v>185974</v>
+        <v>155974</v>
       </c>
       <c r="Z27" s="12">
         <v>187274</v>
@@ -1947,7 +1947,7 @@
         <v>0</v>
       </c>
       <c r="AF27" s="12">
-        <v>4470198</v>
+        <v>4484440</v>
       </c>
     </row>
     <row r="29" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3021,13 +3021,13 @@
       <c r="T51" s="8"/>
       <c r="U51" s="8"/>
       <c r="V51" s="8"/>
-      <c r="W51" s="8"/>
+      <c r="W51" s="8">
+        <v>60000</v>
+      </c>
       <c r="X51" s="8">
-        <v>60000</v>
-      </c>
-      <c r="Y51" s="8">
         <v>30000</v>
       </c>
+      <c r="Y51" s="8"/>
       <c r="Z51" s="8"/>
       <c r="AA51" s="8"/>
       <c r="AB51" s="8"/>
@@ -3106,13 +3106,13 @@
         <v>100926</v>
       </c>
       <c r="W52" s="12">
-        <v>1438838</v>
+        <v>1498838</v>
       </c>
       <c r="X52" s="12">
-        <v>379950</v>
+        <v>349950</v>
       </c>
       <c r="Y52" s="12">
-        <v>851658</v>
+        <v>821658</v>
       </c>
       <c r="Z52" s="12">
         <v>477638</v>

</xml_diff>

<commit_message>
Financial_Forecast.xlsx settled size after OneDrive rewrite
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3182,4 +3182,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A24790A1-8BFB-43DA-BBC8-6A9A9917DD83}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73BAC1AF-D6BF-495D-9345-BB7F3D86F8BF}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA5AF94D-E200-4282-8A2A-B032CC016602}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-01 10:47)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1DEB5BF-F58E-4021-BB44-BFFAC07129F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5FC5FA09-2CB8-4103-8B81-893055B4C621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FEA4C1C6-CFA0-44A7-B899-252118432047}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B74ECC4C-27F5-40E6-B6E7-200CA1E87C02}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -697,7 +697,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41489AD5-1A53-4044-8A42-4C4B2CCF02E3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{224F17D8-FA19-4BE7-BBC0-85B3957DB47C}">
   <dimension ref="A1:AF54"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3182,291 +3182,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A24790A1-8BFB-43DA-BBC8-6A9A9917DD83}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73BAC1AF-D6BF-495D-9345-BB7F3D86F8BF}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA5AF94D-E200-4282-8A2A-B032CC016602}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-01 10:49)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -3182,4 +3182,291 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
+    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
+                <xsd:element ref="ns2:Complete" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA57DECF-93B1-4E91-943E-E406798EDEC6}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DC9B2964-22BD-47A5-8992-5D39942B6FCA}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24430517-0A19-4F9D-A617-3C79420ECC55}"/>
 </file>
</xml_diff>

<commit_message>
Carry over files left uncommitted by an earlier run
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5FC5FA09-2CB8-4103-8B81-893055B4C621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{836CA9C3-59CF-479A-8EC2-44FC25CAB04C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B74ECC4C-27F5-40E6-B6E7-200CA1E87C02}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F069892B-DE09-42D8-A60A-B72A3F57B697}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -697,7 +697,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{224F17D8-FA19-4BE7-BBC0-85B3957DB47C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BB0EFA7-5F7A-4AE4-AA95-3F5FB2D189F1}">
   <dimension ref="A1:AF54"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3182,291 +3182,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
-    <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <xsd:import namespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:DateStart" minOccurs="0"/>
-                <xsd:element ref="ns2:Complete" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="afb6db77-3ef7-43e7-ae0d-97c1bb5e8330" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="14" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="DateStart" ma:index="23" nillable="true" ma:displayName="Date Start" ma:format="DateOnly" ma:internalName="DateStart">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Complete" ma:index="24" nillable="true" ma:displayName="Complete Date" ma:format="DateOnly" ma:internalName="Complete">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="25" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f20b5557-e70c-4568-8457-3e6232196297}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2d1b07a1-7849-4740-a4b1-3343cd5aadb6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA57DECF-93B1-4E91-943E-E406798EDEC6}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DC9B2964-22BD-47A5-8992-5D39942B6FCA}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24430517-0A19-4F9D-A617-3C79420ECC55}"/>
 </file>
</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-01 16:23)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CE589A1-2E58-42D4-8B5F-5041500CCDBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1F445DE-67E3-4100-A21C-C6679FC2DEC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{71F723CD-3AB5-449D-A13C-9345138A3D45}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{625CB53A-A7DC-462F-AA36-03DD2DF9FB10}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -697,7 +697,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A9E8F56-FACC-496A-8399-CD7E45710A9A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96ACD0A0-39EC-471F-8F01-0F39269FC5FA}">
   <dimension ref="A1:AF54"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (rebuild)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1F445DE-67E3-4100-A21C-C6679FC2DEC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A57CCCE-2145-4196-8E5A-6E00695CBE59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{625CB53A-A7DC-462F-AA36-03DD2DF9FB10}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C7CA7126-8496-4113-AC93-03F24C9DFF7C}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -697,7 +697,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96ACD0A0-39EC-471F-8F01-0F39269FC5FA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B37C61D-69AD-434A-9F49-46E308E51CCB}">
   <dimension ref="A1:AF54"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-02 10:29)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{63F6AD78-774C-4EE4-A797-8C54013D6B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{259485B8-53E8-4D5B-8C01-23E82891A8B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CC8E63CC-DD86-4C89-8D4C-F30B15FE944D}"/>
+    <workbookView xWindow="9036" yWindow="1128" windowWidth="13572" windowHeight="10368" xr2:uid="{10AE2A20-21DF-4799-85F9-DB7E9CFF9EF3}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (21 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-01</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-02</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -697,7 +697,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B502F0E7-F740-4A1F-A6A4-9BDF6040A0A5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B256601-23CB-4E43-A2AA-9419B914A760}">
   <dimension ref="A1:AF54"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-02 13:08)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{259485B8-53E8-4D5B-8C01-23E82891A8B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6EED35FE-62E8-4466-A456-39A8869B6D27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9036" yWindow="1128" windowWidth="13572" windowHeight="10368" xr2:uid="{10AE2A20-21DF-4799-85F9-DB7E9CFF9EF3}"/>
+    <workbookView xWindow="9036" yWindow="1128" windowWidth="13572" windowHeight="10368" xr2:uid="{CBF0A027-ADDD-4B35-AE0F-501ADE4F934F}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -697,7 +697,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B256601-23CB-4E43-A2AA-9419B914A760}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E101DDFA-2620-46CD-B758-B4B466B88FF9}">
   <dimension ref="A1:AF54"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-03 09:44)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6EED35FE-62E8-4466-A456-39A8869B6D27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C6267D6-D2CB-4CB3-9BBB-8258EE5E98DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9036" yWindow="1128" windowWidth="13572" windowHeight="10368" xr2:uid="{CBF0A027-ADDD-4B35-AE0F-501ADE4F934F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{17053454-EC3A-47CE-B50C-DF650D041A62}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (21 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-02</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-03</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -697,7 +697,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E101DDFA-2620-46CD-B758-B4B466B88FF9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3855F1D-1623-4716-99ED-5EDC912ED3C7}">
   <dimension ref="A1:AF54"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>